<commit_message>
Add Company Stats sheet: per-symbol trade count, win rate, P&L
New 5th sheet, same shape as Position Type Stats but grouped by Symbol
instead of LONG/SHORT. Since the distinct symbol set isn't fixed (unlike
LONG/SHORT) and UNIQUE()/FILTER() aren't allowed for LibreOffice/Google
Sheets compatibility, the symbol list is computed in Python from the same
`trades` already loaded for Trade Log and written as literal row labels --
same pattern as Position Type Stats' hardcoded LONG/SHORT rows, just
dynamically sized. Purely derived (no manual-entry rows below the real
data): a symbol only appears here once it's actually been traded.

Verified via LibreOffice recalc: repeat-symbol aggregation (3 trades on one
symbol, mixed open/closed/win/loss), win rate math, and the TOTAL row all
compute correctly with zero formula errors.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Wise PnL" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Position Type Stats" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Stats" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$M$503</definedName>
@@ -28959,4 +28960,350 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Company Stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Per-symbol performance across every logged trade, computed straight from Trade Log.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Trades</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Gross P&amp;L</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Net P&amp;L</t>
+        </is>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>Avg Net P&amp;L / Trade</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>Best Trade</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>Worst Trade</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>BAJAJHIND</t>
+        </is>
+      </c>
+      <c r="B4" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A4,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D4" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A4,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E4" s="29">
+        <f>IFERROR($C4/$B4,"")</f>
+        <v/>
+      </c>
+      <c r="F4" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A4,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G4" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A4,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H4" s="21">
+        <f>IFERROR($G4/$B4,"")</f>
+        <v/>
+      </c>
+      <c r="I4" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A4),"")</f>
+        <v/>
+      </c>
+      <c r="J4" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>GOPAL</t>
+        </is>
+      </c>
+      <c r="B5" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A5,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D5" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A5,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E5" s="29">
+        <f>IFERROR($C5/$B5,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A5,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A5,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H5" s="21">
+        <f>IFERROR($G5/$B5,"")</f>
+        <v/>
+      </c>
+      <c r="I5" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A5),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>NILKAMAL</t>
+        </is>
+      </c>
+      <c r="B6" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A6,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D6" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A6,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E6" s="29">
+        <f>IFERROR($C6/$B6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A6,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G6" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A6,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H6" s="21">
+        <f>IFERROR($G6/$B6,"")</f>
+        <v/>
+      </c>
+      <c r="I6" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A6),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>ORIENTHOT</t>
+        </is>
+      </c>
+      <c r="B7" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D7" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E7" s="29">
+        <f>IFERROR($C7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A7,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H7" s="21">
+        <f>IFERROR($G7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B8" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E8" s="29">
+        <f>IFERROR($C8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>IFERROR($G8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="30">
+        <f>SUM(B4:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="30">
+        <f>SUM(C4:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="30">
+        <f>SUM(D4:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="31">
+        <f>IFERROR(C9/B9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="32">
+        <f>SUM(F4:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
+        <f>SUM(G4:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="32">
+        <f>IFERROR(G9/B9,"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update today's pipeline state (2026-08-20 entries, exits, P&L sync)
Market cap fetch, 9:25 exit-check results, and the manually-placed
BAJAJHIND stop-loss (see prior commit's UC-fetch fix) for today's run.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1462,8 +1462,12 @@
       <c r="F4" s="26" t="n">
         <v>14742</v>
       </c>
-      <c r="G4" s="24" t="inlineStr"/>
-      <c r="H4" s="25" t="inlineStr"/>
+      <c r="G4" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H4" s="25" t="n">
+        <v>20.9689</v>
+      </c>
       <c r="I4" s="21">
         <f>IF(OR($B4="",$H4=""),"",IF($C4="LONG",($H4-$E4)*$F4,($E4-$H4)*$F4))</f>
         <v/>
@@ -1673,19 +1677,39 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n"/>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="25" t="n"/>
-      <c r="F9" s="26" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="25" t="n"/>
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082016509</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>BAJAJHIND</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>20.9605</v>
+      </c>
+      <c r="F9" s="26" t="n">
+        <v>14742</v>
+      </c>
+      <c r="G9" s="24" t="inlineStr"/>
+      <c r="H9" s="25" t="inlineStr"/>
       <c r="I9" s="21">
         <f>IF(OR($B9="",$H9=""),"",IF($C9="LONG",($H9-$E9)*$F9,($E9-$H9)*$F9))</f>
         <v/>
       </c>
-      <c r="J9" s="4" t="n"/>
+      <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($J9="",0,$J9))</f>
         <v/>

</xml_diff>

<commit_message>
Always compute position costs from the rate-model estimate, not the trade-book API
Verified live against a real BAJAJHIND fill: estimate_trade_charges()
matches the API's actual per-trade charges to within Rs 0.05 on a
Rs 378.78 leg (~0.01%). Meanwhile the trade-book API is unreliable for
this pipeline's purposes either way -- the historical range endpoint
doesn't index same-day trades, and the same-day single-order endpoint
doesn't carry charge fields at all (was silently producing a false
"api"-sourced Rs 0 for every same-day exit leg until this change).
Given the estimate is already accurate, position_charge_summary() now
uses it unconditionally instead of treating it as an outage fallback --
removes the network round-trips and the false-zero risk entirely.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>480.14</v>
+        <v>824.42</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0</v>
+        <v>112.41</v>
       </c>
       <c r="K9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($J9="",0,$J9))</f>

</xml_diff>

<commit_message>
Data update — 2026-08-20 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1513,14 +1513,18 @@
       <c r="F5" s="26" t="n">
         <v>1038</v>
       </c>
-      <c r="G5" s="24" t="inlineStr"/>
-      <c r="H5" s="25" t="inlineStr"/>
+      <c r="G5" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H5" s="25" t="n">
+        <v>281.1859</v>
+      </c>
       <c r="I5" s="21">
         <f>IF(OR($B5="",$H5=""),"",IF($C5="LONG",($H5-$E5)*$F5,($E5-$H5)*$F5))</f>
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>501.54</v>
+        <v>827.9299999999999</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1560,14 +1564,18 @@
       <c r="F6" s="26" t="n">
         <v>147</v>
       </c>
-      <c r="G6" s="24" t="inlineStr"/>
-      <c r="H6" s="25" t="inlineStr"/>
+      <c r="G6" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>2020.8687</v>
+      </c>
       <c r="I6" s="21">
         <f>IF(OR($B6="",$H6=""),"",IF($C6="LONG",($H6-$E6)*$F6,($E6-$H6)*$F6))</f>
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>479.48</v>
+        <v>811.26</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1607,14 +1615,18 @@
       <c r="F7" s="26" t="n">
         <v>2137</v>
       </c>
-      <c r="G7" s="24" t="inlineStr"/>
-      <c r="H7" s="25" t="inlineStr"/>
+      <c r="G7" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>134.2087</v>
+      </c>
       <c r="I7" s="21">
         <f>IF(OR($B7="",$H7=""),"",IF($C7="LONG",($H7-$E7)*$F7,($E7-$H7)*$F7))</f>
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>489.23</v>
+        <v>810.36</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1654,14 +1666,18 @@
       <c r="F8" s="26" t="n">
         <v>1609</v>
       </c>
-      <c r="G8" s="24" t="inlineStr"/>
-      <c r="H8" s="25" t="inlineStr"/>
+      <c r="G8" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>190.697</v>
+      </c>
       <c r="I8" s="21">
         <f>IF(OR($B8="",$H8=""),"",IF($C8="LONG",($H8-$E8)*$F8,($E8-$H8)*$F8))</f>
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>489.18</v>
+        <v>831.08</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1701,14 +1717,18 @@
       <c r="F9" s="26" t="n">
         <v>14742</v>
       </c>
-      <c r="G9" s="24" t="inlineStr"/>
-      <c r="H9" s="25" t="inlineStr"/>
+      <c r="G9" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>22.2519</v>
+      </c>
       <c r="I9" s="21">
         <f>IF(OR($B9="",$H9=""),"",IF($C9="LONG",($H9-$E9)*$F9,($E9-$H9)*$F9))</f>
         <v/>
       </c>
       <c r="J9" s="4" t="n">
-        <v>112.41</v>
+        <v>158.12</v>
       </c>
       <c r="K9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($J9="",0,$J9))</f>
@@ -1724,19 +1744,39 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n"/>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="25" t="n"/>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="25" t="n"/>
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082075909</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>BANARISUG</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>4243.582</v>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>39</v>
+      </c>
+      <c r="G10" s="24" t="inlineStr"/>
+      <c r="H10" s="25" t="inlineStr"/>
       <c r="I10" s="21">
         <f>IF(OR($B10="",$H10=""),"",IF($C10="LONG",($H10-$E10)*$F10,($E10-$H10)*$F10))</f>
         <v/>
       </c>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="4" t="n">
+        <v>270.27</v>
+      </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
         <v/>
@@ -1751,19 +1791,43 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n"/>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="25" t="n"/>
-      <c r="F11" s="26" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="25" t="n"/>
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126082044409</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>GOPAL</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>281.1067</v>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>1038</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>282.9361</v>
+      </c>
       <c r="I11" s="21">
         <f>IF(OR($B11="",$H11=""),"",IF($C11="LONG",($H11-$E11)*$F11,($E11-$H11)*$F11))</f>
         <v/>
       </c>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="4" t="n">
+        <v>150.86</v>
+      </c>
       <c r="K11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($J11="",0,$J11))</f>
         <v/>
@@ -1778,19 +1842,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n"/>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="25" t="n"/>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="H12" s="25" t="n"/>
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126082081809</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>HUBTOWN</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>201.5272</v>
+      </c>
+      <c r="F12" s="26" t="n">
+        <v>827</v>
+      </c>
+      <c r="G12" s="24" t="inlineStr"/>
+      <c r="H12" s="25" t="inlineStr"/>
       <c r="I12" s="21">
         <f>IF(OR($B12="",$H12=""),"",IF($C12="LONG",($H12-$E12)*$F12,($E12-$H12)*$F12))</f>
         <v/>
       </c>
-      <c r="J12" s="4" t="n"/>
+      <c r="J12" s="4" t="n">
+        <v>271.65</v>
+      </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
         <v/>
@@ -1805,19 +1889,39 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n"/>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="25" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="25" t="n"/>
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260820757209</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>KIRIINDUS</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>462.385</v>
+      </c>
+      <c r="F13" s="26" t="n">
+        <v>361</v>
+      </c>
+      <c r="G13" s="24" t="inlineStr"/>
+      <c r="H13" s="25" t="inlineStr"/>
       <c r="I13" s="21">
         <f>IF(OR($B13="",$H13=""),"",IF($C13="LONG",($H13-$E13)*$F13,($E13-$H13)*$F13))</f>
         <v/>
       </c>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="4" t="n">
+        <v>271.95</v>
+      </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
         <v/>
@@ -1832,19 +1936,39 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="n"/>
-      <c r="B14" s="23" t="n"/>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="25" t="n"/>
-      <c r="F14" s="26" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="25" t="n"/>
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260820757609</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>MANGLMCEM</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>988.9262</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <v>168</v>
+      </c>
+      <c r="G14" s="24" t="inlineStr"/>
+      <c r="H14" s="25" t="inlineStr"/>
       <c r="I14" s="21">
         <f>IF(OR($B14="",$H14=""),"",IF($C14="LONG",($H14-$E14)*$F14,($E14-$H14)*$F14))</f>
         <v/>
       </c>
-      <c r="J14" s="4" t="n"/>
+      <c r="J14" s="4" t="n">
+        <v>271.02</v>
+      </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
         <v/>
@@ -1859,19 +1983,39 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="n"/>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="25" t="n"/>
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260820757709</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>NETWORK18</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>30.4987</v>
+      </c>
+      <c r="F15" s="26" t="n">
+        <v>5468</v>
+      </c>
+      <c r="G15" s="24" t="inlineStr"/>
+      <c r="H15" s="25" t="inlineStr"/>
       <c r="I15" s="21">
         <f>IF(OR($B15="",$H15=""),"",IF($C15="LONG",($H15-$E15)*$F15,($E15-$H15)*$F15))</f>
         <v/>
       </c>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="4" t="n">
+        <v>271.77</v>
+      </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
         <v/>
@@ -1886,19 +2030,43 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="n"/>
-      <c r="B16" s="23" t="n"/>
-      <c r="C16" s="23" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="25" t="n"/>
-      <c r="F16" s="26" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="25" t="n"/>
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260820468709</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>NILKAMAL</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>2019.2572</v>
+      </c>
+      <c r="F16" s="26" t="n">
+        <v>147</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H16" s="25" t="n">
+        <v>2037.9993</v>
+      </c>
       <c r="I16" s="21">
         <f>IF(OR($B16="",$H16=""),"",IF($C16="LONG",($H16-$E16)*$F16,($E16-$H16)*$F16))</f>
         <v/>
       </c>
-      <c r="J16" s="4" t="n"/>
+      <c r="J16" s="4" t="n">
+        <v>152.7</v>
+      </c>
       <c r="K16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($J16="",0,$J16))</f>
         <v/>
@@ -1913,19 +2081,43 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="n"/>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="23" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="26" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="25" t="n"/>
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126082044709</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>ORIENTHOT</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>134.1808</v>
+      </c>
+      <c r="F17" s="26" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>134.9144</v>
+      </c>
       <c r="I17" s="21">
         <f>IF(OR($B17="",$H17=""),"",IF($C17="LONG",($H17-$E17)*$F17,($E17-$H17)*$F17))</f>
         <v/>
       </c>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="4" t="n">
+        <v>149.05</v>
+      </c>
       <c r="K17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($J17="",0,$J17))</f>
         <v/>
@@ -1940,19 +2132,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="n"/>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="23" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="25" t="n"/>
-      <c r="F18" s="26" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="25" t="n"/>
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260820757909</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>639.9</v>
+      </c>
+      <c r="F18" s="26" t="n">
+        <v>261</v>
+      </c>
+      <c r="G18" s="24" t="inlineStr"/>
+      <c r="H18" s="25" t="inlineStr"/>
       <c r="I18" s="21">
         <f>IF(OR($B18="",$H18=""),"",IF($C18="LONG",($H18-$E18)*$F18,($E18-$H18)*$F18))</f>
         <v/>
       </c>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="4" t="n">
+        <v>272.06</v>
+      </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
         <v/>
@@ -1967,19 +2179,43 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="25" t="n"/>
-      <c r="F19" s="26" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="25" t="n"/>
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126082044909</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>190.82</v>
+      </c>
+      <c r="F19" s="26" t="n">
+        <v>1609</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>197.6402</v>
+      </c>
       <c r="I19" s="21">
         <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
         <v/>
       </c>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="4" t="n">
+        <v>156.88</v>
+      </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
         <v/>
@@ -28992,7 +29228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29119,7 +29355,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -29162,7 +29398,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -29205,7 +29441,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -29248,78 +29484,336 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
+          <t>KIRIINDUS</t>
+        </is>
+      </c>
+      <c r="B8" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E8" s="29">
+        <f>IFERROR($C8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H8" s="21">
+        <f>IFERROR($G8/$B8,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>MANGLMCEM</t>
+        </is>
+      </c>
+      <c r="B9" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D9" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E9" s="29">
+        <f>IFERROR($C9/$B9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A9,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H9" s="21">
+        <f>IFERROR($G9/$B9,"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A9),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>NETWORK18</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D10" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E10" s="29">
+        <f>IFERROR($C10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A10,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H10" s="21">
+        <f>IFERROR($G10/$B10,"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>NILKAMAL</t>
+        </is>
+      </c>
+      <c r="B11" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D11" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E11" s="29">
+        <f>IFERROR($C11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A11,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H11" s="21">
+        <f>IFERROR($G11/$B11,"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A11),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>ORIENTHOT</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E12" s="29">
+        <f>IFERROR($C12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A12,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H12" s="21">
+        <f>IFERROR($G12/$B12,"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A12),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="B13" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D13" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E13" s="29">
+        <f>IFERROR($C13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A13,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H13" s="21">
+        <f>IFERROR($G13/$B13,"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A13),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B8" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A8)</f>
-        <v/>
-      </c>
-      <c r="C8" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D8" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E8" s="29">
-        <f>IFERROR($C8/$B8,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G8" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A8,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H8" s="21">
-        <f>IFERROR($G8/$B8,"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A8),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B14" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>IFERROR($C14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>IFERROR($G14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="30">
-        <f>SUM(B4:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="30">
-        <f>SUM(C4:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="30">
-        <f>SUM(D4:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="31">
-        <f>IFERROR(C9/B9,"")</f>
-        <v/>
-      </c>
-      <c r="F9" s="32">
-        <f>SUM(F4:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="32">
-        <f>SUM(G4:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="32">
-        <f>IFERROR(G9/B9,"")</f>
+      <c r="B15" s="30">
+        <f>SUM(B4:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="30">
+        <f>SUM(C4:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="30">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="31">
+        <f>IFERROR(C15/B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="32">
+        <f>SUM(F4:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="32">
+        <f>SUM(G4:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="32">
+        <f>IFERROR(G15/B15,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Route every Dhan pipeline stage to the split long/short position files
Follow-up to the previous commit's file split (positions_dhan_long.json /
positions_dhan_short.json) -- that commit only removed the old combined
file; this one carries the actual code. run_trades.py: every read/write
site in run_entry_321/place_targets_915/check_exit_925/force_exit_1159
routed to the long file, _open_short()/square_off_239 routed to the
short file. charges.py: product_map()/tracked_order_ids()/
print_mtf_interest_report() merge both files. build_pnl_simple.py's
Trade Log sync merges both files too (still shows long+short trades
together). Test suite (dhan/test_targets.py) updated to mock the
correct file per scenario -- all 21 scenarios passing.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -2181,68 +2181,88 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
+          <t>DHAN-23126082074409</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>257.6</v>
+      </c>
+      <c r="F19" s="26" t="n">
+        <v>650</v>
+      </c>
+      <c r="G19" s="24" t="inlineStr"/>
+      <c r="H19" s="25" t="inlineStr"/>
+      <c r="I19" s="21">
+        <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
+        <v/>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>272.57</v>
+      </c>
+      <c r="K19" s="21">
+        <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="22">
+        <f>IF(OR($B19="",$K19="",$E19=0,$F19=0),"",$K19/($E19*$F19))</f>
+        <v/>
+      </c>
+      <c r="M19" s="27">
+        <f>IF($B19="","",IF($H19="","Open","Closed"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
           <t>DHAN-22126082044909</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>SHORT</t>
         </is>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D20" s="24" t="n">
         <v>46254</v>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="E20" s="25" t="n">
         <v>190.82</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F20" s="26" t="n">
         <v>1609</v>
       </c>
-      <c r="G19" s="24" t="n">
+      <c r="G20" s="24" t="n">
         <v>46254</v>
       </c>
-      <c r="H19" s="25" t="n">
+      <c r="H20" s="25" t="n">
         <v>197.6402</v>
       </c>
-      <c r="I19" s="21">
-        <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
-        <v/>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>156.88</v>
-      </c>
-      <c r="K19" s="21">
-        <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
-        <v/>
-      </c>
-      <c r="L19" s="22">
-        <f>IF(OR($B19="",$K19="",$E19=0,$F19=0),"",$K19/($E19*$F19))</f>
-        <v/>
-      </c>
-      <c r="M19" s="27">
-        <f>IF($B19="","",IF($H19="","Open","Closed"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="25" t="n"/>
-      <c r="F20" s="26" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="25" t="n"/>
       <c r="I20" s="21">
         <f>IF(OR($B20="",$H20=""),"",IF($C20="LONG",($H20-$E20)*$F20,($E20-$H20)*$F20))</f>
         <v/>
       </c>
-      <c r="J20" s="4" t="n"/>
+      <c r="J20" s="4" t="n">
+        <v>156.88</v>
+      </c>
       <c r="K20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($J20="",0,$J20))</f>
         <v/>
@@ -29228,7 +29248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29742,78 +29762,121 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D14" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>IFERROR($C14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H14" s="21">
+        <f>IFERROR($G14/$B14,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B14" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A14)</f>
-        <v/>
-      </c>
-      <c r="C14" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D14" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>IFERROR($C14/$B14,"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G14" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A14,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H14" s="21">
-        <f>IFERROR($G14/$B14,"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A14),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B15" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>IFERROR($C15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H15" s="21">
+        <f>IFERROR($G15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="30">
-        <f>SUM(B4:B14)</f>
-        <v/>
-      </c>
-      <c r="C15" s="30">
-        <f>SUM(C4:C14)</f>
-        <v/>
-      </c>
-      <c r="D15" s="30">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="31">
-        <f>IFERROR(C15/B15,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="32">
-        <f>SUM(F4:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="32">
-        <f>SUM(G4:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="32">
-        <f>IFERROR(G15/B15,"")</f>
+      <c r="B16" s="30">
+        <f>SUM(B4:B15)</f>
+        <v/>
+      </c>
+      <c r="C16" s="30">
+        <f>SUM(C4:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="30">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="31">
+        <f>IFERROR(C16/B16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="32">
+        <f>SUM(F4:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="32">
+        <f>SUM(G4:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="32">
+        <f>IFERROR(G16/B16,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-08-21 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.08</v>
+        <v>830.98</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1768,14 +1768,18 @@
       <c r="F10" s="26" t="n">
         <v>39</v>
       </c>
-      <c r="G10" s="24" t="inlineStr"/>
-      <c r="H10" s="25" t="inlineStr"/>
+      <c r="G10" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H10" s="25" t="n">
+        <v>4030.5</v>
+      </c>
       <c r="I10" s="21">
         <f>IF(OR($B10="",$H10=""),"",IF($C10="LONG",($H10-$E10)*$F10,($E10-$H10)*$F10))</f>
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>270.27</v>
+        <v>485.23</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1866,14 +1870,18 @@
       <c r="F12" s="26" t="n">
         <v>827</v>
       </c>
-      <c r="G12" s="24" t="inlineStr"/>
-      <c r="H12" s="25" t="inlineStr"/>
+      <c r="G12" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>197.7805</v>
+      </c>
       <c r="I12" s="21">
         <f>IF(OR($B12="",$H12=""),"",IF($C12="LONG",($H12-$E12)*$F12,($E12-$H12)*$F12))</f>
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>271.65</v>
+        <v>499.13</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1913,14 +1921,18 @@
       <c r="F13" s="26" t="n">
         <v>361</v>
       </c>
-      <c r="G13" s="24" t="inlineStr"/>
-      <c r="H13" s="25" t="inlineStr"/>
+      <c r="G13" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>463.0857</v>
+      </c>
       <c r="I13" s="21">
         <f>IF(OR($B13="",$H13=""),"",IF($C13="LONG",($H13-$E13)*$F13,($E13-$H13)*$F13))</f>
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>271.95</v>
+        <v>505.32</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1960,14 +1972,18 @@
       <c r="F14" s="26" t="n">
         <v>168</v>
       </c>
-      <c r="G14" s="24" t="inlineStr"/>
-      <c r="H14" s="25" t="inlineStr"/>
+      <c r="G14" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H14" s="25" t="n">
+        <v>989.1455</v>
+      </c>
       <c r="I14" s="21">
         <f>IF(OR($B14="",$H14=""),"",IF($C14="LONG",($H14-$E14)*$F14,($E14-$H14)*$F14))</f>
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>271.02</v>
+        <v>501.11</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2007,14 +2023,18 @@
       <c r="F15" s="26" t="n">
         <v>5468</v>
       </c>
-      <c r="G15" s="24" t="inlineStr"/>
-      <c r="H15" s="25" t="inlineStr"/>
+      <c r="G15" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H15" s="25" t="n">
+        <v>30.5039</v>
+      </c>
       <c r="I15" s="21">
         <f>IF(OR($B15="",$H15=""),"",IF($C15="LONG",($H15-$E15)*$F15,($E15-$H15)*$F15))</f>
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>271.77</v>
+        <v>505.74</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2156,14 +2176,18 @@
       <c r="F18" s="26" t="n">
         <v>261</v>
       </c>
-      <c r="G18" s="24" t="inlineStr"/>
-      <c r="H18" s="25" t="inlineStr"/>
+      <c r="G18" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H18" s="25" t="n">
+        <v>615.2594</v>
+      </c>
       <c r="I18" s="21">
         <f>IF(OR($B18="",$H18=""),"",IF($C18="LONG",($H18-$E18)*$F18,($E18-$H18)*$F18))</f>
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>272.06</v>
+        <v>496.52</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2203,14 +2227,18 @@
       <c r="F19" s="26" t="n">
         <v>650</v>
       </c>
-      <c r="G19" s="24" t="inlineStr"/>
-      <c r="H19" s="25" t="inlineStr"/>
+      <c r="G19" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>259.5025</v>
+      </c>
       <c r="I19" s="21">
         <f>IF(OR($B19="",$H19=""),"",IF($C19="LONG",($H19-$E19)*$F19,($E19-$H19)*$F19))</f>
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>272.57</v>
+        <v>500.36</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2277,19 +2305,43 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="n"/>
-      <c r="B21" s="23" t="n"/>
-      <c r="C21" s="23" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="25" t="n"/>
-      <c r="F21" s="26" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="25" t="n"/>
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082147609</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>BANARISUG</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>4030.5103</v>
+      </c>
+      <c r="F21" s="26" t="n">
+        <v>39</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H21" s="25" t="n">
+        <v>4029.782</v>
+      </c>
       <c r="I21" s="21">
         <f>IF(OR($B21="",$H21=""),"",IF($C21="LONG",($H21-$E21)*$F21,($E21-$H21)*$F21))</f>
         <v/>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>102.97</v>
+      </c>
       <c r="K21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($J21="",0,$J21))</f>
         <v/>
@@ -2304,19 +2356,43 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
-      <c r="B22" s="23" t="n"/>
-      <c r="C22" s="23" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="25" t="n"/>
-      <c r="F22" s="26" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="25" t="n"/>
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082146909</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>HUBTOWN</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>197.3558</v>
+      </c>
+      <c r="F22" s="26" t="n">
+        <v>827</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H22" s="25" t="n">
+        <v>196.7219</v>
+      </c>
       <c r="I22" s="21">
         <f>IF(OR($B22="",$H22=""),"",IF($C22="LONG",($H22-$E22)*$F22,($E22-$H22)*$F22))</f>
         <v/>
       </c>
-      <c r="J22" s="4" t="n"/>
+      <c r="J22" s="4" t="n">
+        <v>105.07</v>
+      </c>
       <c r="K22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($J22="",0,$J22))</f>
         <v/>
@@ -2331,19 +2407,43 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-      <c r="B23" s="23" t="n"/>
-      <c r="C23" s="23" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="25" t="n"/>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="25" t="n"/>
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082116409</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>KIRIINDUS</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>462.9753</v>
+      </c>
+      <c r="F23" s="26" t="n">
+        <v>361</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H23" s="25" t="n">
+        <v>474</v>
+      </c>
       <c r="I23" s="21">
         <f>IF(OR($B23="",$H23=""),"",IF($C23="LONG",($H23-$E23)*$F23,($E23-$H23)*$F23))</f>
         <v/>
       </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="4" t="n">
+        <v>106.77</v>
+      </c>
       <c r="K23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($J23="",0,$J23))</f>
         <v/>
@@ -2358,19 +2458,43 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="n"/>
-      <c r="B24" s="23" t="n"/>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="25" t="n"/>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="25" t="n"/>
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260821106109</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>MANGLMCEM</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>988.4104</v>
+      </c>
+      <c r="F24" s="26" t="n">
+        <v>168</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H24" s="25" t="n">
+        <v>1013.811</v>
+      </c>
       <c r="I24" s="21">
         <f>IF(OR($B24="",$H24=""),"",IF($C24="LONG",($H24-$E24)*$F24,($E24-$H24)*$F24))</f>
         <v/>
       </c>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="4" t="n">
+        <v>106.4</v>
+      </c>
       <c r="K24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($J24="",0,$J24))</f>
         <v/>
@@ -2385,19 +2509,43 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="n"/>
-      <c r="B25" s="23" t="n"/>
-      <c r="C25" s="23" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="25" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="25" t="n"/>
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260821106709</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>NETWORK18</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>30.5074</v>
+      </c>
+      <c r="F25" s="26" t="n">
+        <v>5468</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H25" s="25" t="n">
+        <v>29.9088</v>
+      </c>
       <c r="I25" s="21">
         <f>IF(OR($B25="",$H25=""),"",IF($C25="LONG",($H25-$E25)*$F25,($E25-$H25)*$F25))</f>
         <v/>
       </c>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="4" t="n">
+        <v>106.17</v>
+      </c>
       <c r="K25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($J25="",0,$J25))</f>
         <v/>
@@ -2412,19 +2560,43 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="23" t="n"/>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="25" t="n"/>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="25" t="n"/>
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082147809</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>614.6021</v>
+      </c>
+      <c r="F26" s="26" t="n">
+        <v>261</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H26" s="25" t="n">
+        <v>614.4914</v>
+      </c>
       <c r="I26" s="21">
         <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
         <v/>
       </c>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="4" t="n">
+        <v>104.11</v>
+      </c>
       <c r="K26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($J26="",0,$J26))</f>
         <v/>
@@ -2439,19 +2611,39 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="23" t="n"/>
-      <c r="C27" s="23" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="25" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="25" t="n"/>
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260821720509</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>THOMASCOOK</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>113.4719</v>
+      </c>
+      <c r="F27" s="26" t="n">
+        <v>3301</v>
+      </c>
+      <c r="G27" s="24" t="inlineStr"/>
+      <c r="H27" s="25" t="inlineStr"/>
       <c r="I27" s="21">
         <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
         <v/>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="n">
+        <v>518.52</v>
+      </c>
       <c r="K27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($J27="",0,$J27))</f>
         <v/>
@@ -2466,19 +2658,43 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
-      <c r="B28" s="23" t="n"/>
-      <c r="C28" s="23" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="25" t="n"/>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="25" t="n"/>
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082115309</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <v>259.503</v>
+      </c>
+      <c r="F28" s="26" t="n">
+        <v>650</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H28" s="25" t="n">
+        <v>261.6704</v>
+      </c>
       <c r="I28" s="21">
         <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
         <v/>
       </c>
-      <c r="J28" s="4" t="n"/>
+      <c r="J28" s="4" t="n">
+        <v>107.14</v>
+      </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
         <v/>
@@ -29248,7 +29464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29762,7 +29978,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -29805,78 +30021,121 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D15" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>IFERROR($C15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G15" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H15" s="21">
+        <f>IFERROR($G15/$B15,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B15" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A15)</f>
-        <v/>
-      </c>
-      <c r="C15" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D15" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E15" s="29">
-        <f>IFERROR($C15/$B15,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G15" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A15,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H15" s="21">
-        <f>IFERROR($G15/$B15,"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A15),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="B16" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E16" s="29">
+        <f>IFERROR($C16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>IFERROR($G16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B16" s="30">
-        <f>SUM(B4:B15)</f>
-        <v/>
-      </c>
-      <c r="C16" s="30">
-        <f>SUM(C4:C15)</f>
-        <v/>
-      </c>
-      <c r="D16" s="30">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="31">
-        <f>IFERROR(C16/B16,"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="32">
-        <f>SUM(F4:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="32">
-        <f>SUM(G4:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="32">
-        <f>IFERROR(G16/B16,"")</f>
+      <c r="B17" s="30">
+        <f>SUM(B4:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="30">
+        <f>SUM(C4:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="30">
+        <f>SUM(D4:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="31">
+        <f>IFERROR(C17/B17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="32">
+        <f>SUM(F4:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="32">
+        <f>SUM(G4:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="32">
+        <f>IFERROR(G17/B17,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync strategy_pnl_simple.xlsx with KLBRENG-B/WELSPLSOL T+5 entries
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>827.9299999999999</v>
+        <v>827.96</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>830.98</v>
+        <v>831.04</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.32</v>
+        <v>505.3</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2460,40 +2460,36 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260821106109</t>
+          <t>DHAN-361260821483209</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D24" s="24" t="n">
         <v>46255</v>
       </c>
       <c r="E24" s="25" t="n">
-        <v>988.4104</v>
+        <v>406</v>
       </c>
       <c r="F24" s="26" t="n">
-        <v>168</v>
-      </c>
-      <c r="G24" s="24" t="n">
-        <v>46255</v>
-      </c>
-      <c r="H24" s="25" t="n">
-        <v>1013.811</v>
-      </c>
+        <v>950</v>
+      </c>
+      <c r="G24" s="24" t="inlineStr"/>
+      <c r="H24" s="25" t="inlineStr"/>
       <c r="I24" s="21">
         <f>IF(OR($B24="",$H24=""),"",IF($C24="LONG",($H24-$E24)*$F24,($E24-$H24)*$F24))</f>
         <v/>
       </c>
       <c r="J24" s="4" t="n">
-        <v>106.4</v>
+        <v>49.6</v>
       </c>
       <c r="K24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($J24="",0,$J24))</f>
@@ -2511,12 +2507,12 @@
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260821106709</t>
+          <t>DHAN-321260821106109</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="C25" s="23" t="inlineStr">
@@ -2528,23 +2524,23 @@
         <v>46255</v>
       </c>
       <c r="E25" s="25" t="n">
-        <v>30.5074</v>
+        <v>988.4104</v>
       </c>
       <c r="F25" s="26" t="n">
-        <v>5468</v>
+        <v>168</v>
       </c>
       <c r="G25" s="24" t="n">
         <v>46255</v>
       </c>
       <c r="H25" s="25" t="n">
-        <v>29.9088</v>
+        <v>1013.811</v>
       </c>
       <c r="I25" s="21">
         <f>IF(OR($B25="",$H25=""),"",IF($C25="LONG",($H25-$E25)*$F25,($E25-$H25)*$F25))</f>
         <v/>
       </c>
       <c r="J25" s="4" t="n">
-        <v>106.17</v>
+        <v>106.4</v>
       </c>
       <c r="K25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($J25="",0,$J25))</f>
@@ -2562,12 +2558,12 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126082147809</t>
+          <t>DHAN-321260821106709</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
@@ -2579,23 +2575,23 @@
         <v>46255</v>
       </c>
       <c r="E26" s="25" t="n">
-        <v>614.6021</v>
+        <v>30.5074</v>
       </c>
       <c r="F26" s="26" t="n">
-        <v>261</v>
+        <v>5468</v>
       </c>
       <c r="G26" s="24" t="n">
         <v>46255</v>
       </c>
       <c r="H26" s="25" t="n">
-        <v>614.4914</v>
+        <v>29.9088</v>
       </c>
       <c r="I26" s="21">
         <f>IF(OR($B26="",$H26=""),"",IF($C26="LONG",($H26-$E26)*$F26,($E26-$H26)*$F26))</f>
         <v/>
       </c>
       <c r="J26" s="4" t="n">
-        <v>104.11</v>
+        <v>106.17</v>
       </c>
       <c r="K26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($J26="",0,$J26))</f>
@@ -2613,115 +2609,139 @@
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
+          <t>DHAN-23126082147809</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>614.6021</v>
+      </c>
+      <c r="F27" s="26" t="n">
+        <v>261</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H27" s="25" t="n">
+        <v>614.4914</v>
+      </c>
+      <c r="I27" s="21">
+        <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>104.11</v>
+      </c>
+      <c r="K27" s="21">
+        <f>IF(OR($B27="",$I27=""),"",$I27-IF($J27="",0,$J27))</f>
+        <v/>
+      </c>
+      <c r="L27" s="22">
+        <f>IF(OR($B27="",$K27="",$E27=0,$F27=0),"",$K27/($E27*$F27))</f>
+        <v/>
+      </c>
+      <c r="M27" s="27">
+        <f>IF($B27="","",IF($H27="","Open","Closed"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
           <t>DHAN-321260821720509</t>
         </is>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>THOMASCOOK</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D28" s="24" t="n">
         <v>46255</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E28" s="25" t="n">
         <v>113.4719</v>
       </c>
-      <c r="F27" s="26" t="n">
+      <c r="F28" s="26" t="n">
         <v>3301</v>
       </c>
-      <c r="G27" s="24" t="inlineStr"/>
-      <c r="H27" s="25" t="inlineStr"/>
-      <c r="I27" s="21">
-        <f>IF(OR($B27="",$H27=""),"",IF($C27="LONG",($H27-$E27)*$F27,($E27-$H27)*$F27))</f>
-        <v/>
-      </c>
-      <c r="J27" s="4" t="n">
-        <v>518.52</v>
-      </c>
-      <c r="K27" s="21">
-        <f>IF(OR($B27="",$I27=""),"",$I27-IF($J27="",0,$J27))</f>
-        <v/>
-      </c>
-      <c r="L27" s="22">
-        <f>IF(OR($B27="",$K27="",$E27=0,$F27=0),"",$K27/($E27*$F27))</f>
-        <v/>
-      </c>
-      <c r="M27" s="27">
-        <f>IF($B27="","",IF($H27="","Open","Closed"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr"/>
+      <c r="H28" s="25" t="inlineStr"/>
+      <c r="I28" s="21">
+        <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>761.3200000000001</v>
+      </c>
+      <c r="K28" s="21">
+        <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
+        <v/>
+      </c>
+      <c r="L28" s="22">
+        <f>IF(OR($B28="",$K28="",$E28=0,$F28=0),"",$K28/($E28*$F28))</f>
+        <v/>
+      </c>
+      <c r="M28" s="27">
+        <f>IF($B28="","",IF($H28="","Open","Closed"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>DHAN-34126082115309</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>VERANDA</t>
         </is>
       </c>
-      <c r="C28" s="23" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>SHORT</t>
         </is>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D29" s="24" t="n">
         <v>46255</v>
       </c>
-      <c r="E28" s="25" t="n">
+      <c r="E29" s="25" t="n">
         <v>259.503</v>
       </c>
-      <c r="F28" s="26" t="n">
+      <c r="F29" s="26" t="n">
         <v>650</v>
       </c>
-      <c r="G28" s="24" t="n">
+      <c r="G29" s="24" t="n">
         <v>46255</v>
       </c>
-      <c r="H28" s="25" t="n">
+      <c r="H29" s="25" t="n">
         <v>261.6704</v>
       </c>
-      <c r="I28" s="21">
-        <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
-        <v/>
-      </c>
-      <c r="J28" s="4" t="n">
-        <v>107.14</v>
-      </c>
-      <c r="K28" s="21">
-        <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
-        <v/>
-      </c>
-      <c r="L28" s="22">
-        <f>IF(OR($B28="",$K28="",$E28=0,$F28=0),"",$K28/($E28*$F28))</f>
-        <v/>
-      </c>
-      <c r="M28" s="27">
-        <f>IF($B28="","",IF($H28="","Open","Closed"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="23" t="n"/>
-      <c r="B29" s="23" t="n"/>
-      <c r="C29" s="23" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="26" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="25" t="n"/>
       <c r="I29" s="21">
         <f>IF(OR($B29="",$H29=""),"",IF($C29="LONG",($H29-$E29)*$F29,($E29-$H29)*$F29))</f>
         <v/>
       </c>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="4" t="n">
+        <v>107.14</v>
+      </c>
       <c r="K29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($J29="",0,$J29))</f>
         <v/>
@@ -2736,19 +2756,39 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="n"/>
-      <c r="B30" s="23" t="n"/>
-      <c r="C30" s="23" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="25" t="n"/>
-      <c r="F30" s="26" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="25" t="n"/>
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-241260821716609</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E30" s="25" t="n">
+        <v>51.46937</v>
+      </c>
+      <c r="F30" s="26" t="n">
+        <v>7230</v>
+      </c>
+      <c r="G30" s="24" t="inlineStr"/>
+      <c r="H30" s="25" t="inlineStr"/>
       <c r="I30" s="21">
         <f>IF(OR($B30="",$H30=""),"",IF($C30="LONG",($H30-$E30)*$F30,($E30-$H30)*$F30))</f>
         <v/>
       </c>
-      <c r="J30" s="4" t="n"/>
+      <c r="J30" s="4" t="n">
+        <v>48.68</v>
+      </c>
       <c r="K30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($J30="",0,$J30))</f>
         <v/>
@@ -29464,7 +29504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29763,7 +29803,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -29806,7 +29846,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -29849,7 +29889,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -29892,7 +29932,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -29935,7 +29975,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -29978,7 +30018,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30021,7 +30061,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30064,78 +30104,164 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E16" s="29">
+        <f>IFERROR($C16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G16" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>IFERROR($G16/$B16,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A17)</f>
+        <v/>
+      </c>
+      <c r="C17" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E17" s="29">
+        <f>IFERROR($C17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A17,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H17" s="21">
+        <f>IFERROR($G17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A17),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B16" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A16)</f>
-        <v/>
-      </c>
-      <c r="C16" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D16" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E16" s="29">
-        <f>IFERROR($C16/$B16,"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G16" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A16,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H16" s="21">
-        <f>IFERROR($G16/$B16,"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A16),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="B18" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A18)</f>
+        <v/>
+      </c>
+      <c r="C18" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E18" s="29">
+        <f>IFERROR($C18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A18,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H18" s="21">
+        <f>IFERROR($G18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A18),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="30">
-        <f>SUM(B4:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="30">
-        <f>SUM(C4:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="30">
-        <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="31">
-        <f>IFERROR(C17/B17,"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="32">
-        <f>SUM(F4:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="32">
-        <f>SUM(G4:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="32">
-        <f>IFERROR(G17/B17,"")</f>
+      <c r="B19" s="30">
+        <f>SUM(B4:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="30">
+        <f>SUM(C4:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="30">
+        <f>SUM(D4:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="31">
+        <f>IFERROR(C19/B19,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="32">
+        <f>SUM(F4:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="32">
+        <f>SUM(G4:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="32">
+        <f>IFERROR(G19/B19,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-08-24 candle + results refresh
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -2682,14 +2682,18 @@
       <c r="F28" s="26" t="n">
         <v>3301</v>
       </c>
-      <c r="G28" s="24" t="inlineStr"/>
-      <c r="H28" s="25" t="inlineStr"/>
+      <c r="G28" s="24" t="n">
+        <v>46258</v>
+      </c>
+      <c r="H28" s="25" t="n">
+        <v>115.0974</v>
+      </c>
       <c r="I28" s="21">
         <f>IF(OR($B28="",$H28=""),"",IF($C28="LONG",($H28-$E28)*$F28,($E28-$H28)*$F28))</f>
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>761.3200000000001</v>
+        <v>1179.07</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2780,14 +2784,18 @@
       <c r="F30" s="26" t="n">
         <v>7230</v>
       </c>
-      <c r="G30" s="24" t="inlineStr"/>
-      <c r="H30" s="25" t="inlineStr"/>
+      <c r="G30" s="24" t="n">
+        <v>46258</v>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>52.017</v>
+      </c>
       <c r="I30" s="21">
         <f>IF(OR($B30="",$H30=""),"",IF($C30="LONG",($H30-$E30)*$F30,($E30-$H30)*$F30))</f>
         <v/>
       </c>
       <c r="J30" s="4" t="n">
-        <v>48.68</v>
+        <v>180.37</v>
       </c>
       <c r="K30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($J30="",0,$J30))</f>
@@ -2803,19 +2811,39 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
-      <c r="B31" s="23" t="n"/>
-      <c r="C31" s="23" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="25" t="n"/>
-      <c r="F31" s="26" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="25" t="n"/>
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082414109</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>THOMASCOOK</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E31" s="25" t="n">
+        <v>115.202</v>
+      </c>
+      <c r="F31" s="26" t="n">
+        <v>3301</v>
+      </c>
+      <c r="G31" s="24" t="inlineStr"/>
+      <c r="H31" s="25" t="inlineStr"/>
       <c r="I31" s="21">
         <f>IF(OR($B31="",$H31=""),"",IF($C31="LONG",($H31-$E31)*$F31,($E31-$H31)*$F31))</f>
         <v/>
       </c>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="n">
+        <v>132.89</v>
+      </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
         <v/>
@@ -2830,19 +2858,39 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n"/>
-      <c r="B32" s="23" t="n"/>
-      <c r="C32" s="23" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="25" t="n"/>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="25" t="n"/>
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082414209</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E32" s="25" t="n">
+        <v>51.8309</v>
+      </c>
+      <c r="F32" s="26" t="n">
+        <v>7230</v>
+      </c>
+      <c r="G32" s="24" t="inlineStr"/>
+      <c r="H32" s="25" t="inlineStr"/>
       <c r="I32" s="21">
         <f>IF(OR($B32="",$H32=""),"",IF($C32="LONG",($H32-$E32)*$F32,($E32-$H32)*$F32))</f>
         <v/>
       </c>
-      <c r="J32" s="4" t="n"/>
+      <c r="J32" s="4" t="n">
+        <v>131.3</v>
+      </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
         <v/>

</xml_diff>

<commit_message>
Charge non-MTF/non-INTRADAY products (MARGIN/T+5) at CNC rates
estimate_trade_charges() and position_charge_summary()'s DP-charge check
both had an implicit "else -> INTRADAY" default that silently
misclassified MARGIN (T+5) positions -- KLBRENG-B/WELSPLSOL were being
charged intraday rates (0.025% sell-side STT, no DP charge) instead of
delivery-style rates (0.1% STT both sides, DP charge applies). Per
explicit instruction: any product that isn't MTF or INTRADAY defaults
to CNC-style charges now, since MTF and INTRADAY are the only two
products with genuinely different (leveraged / same-day) charge
treatment -- everything else, including MARGIN, is delivery-style like
CNC.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -2489,7 +2489,7 @@
         <v/>
       </c>
       <c r="J24" s="4" t="n">
-        <v>49.6</v>
+        <v>472.73</v>
       </c>
       <c r="K24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($J24="",0,$J24))</f>
@@ -2795,7 +2795,7 @@
         <v/>
       </c>
       <c r="J30" s="4" t="n">
-        <v>180.37</v>
+        <v>846.76</v>
       </c>
       <c r="K30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($J30="",0,$J30))</f>

</xml_diff>

<commit_message>
Data update — 2026-08-25 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>824.42</v>
+        <v>810.1</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>827.96</v>
+        <v>828</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.04</v>
+        <v>831.01</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.3</v>
+        <v>505.24</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.74</v>
+        <v>505.76</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.07</v>
+        <v>1179.26</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2839,14 +2839,18 @@
       <c r="F31" s="26" t="n">
         <v>405</v>
       </c>
-      <c r="G31" s="24" t="inlineStr"/>
-      <c r="H31" s="25" t="inlineStr"/>
+      <c r="G31" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>412.7043</v>
+      </c>
       <c r="I31" s="21">
         <f>IF(OR($B31="",$H31=""),"",IF($C31="LONG",($H31-$E31)*$F31,($E31-$H31)*$F31))</f>
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>272.23</v>
+        <v>503.53</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2886,14 +2890,18 @@
       <c r="F32" s="26" t="n">
         <v>942</v>
       </c>
-      <c r="G32" s="24" t="inlineStr"/>
-      <c r="H32" s="25" t="inlineStr"/>
+      <c r="G32" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H32" s="25" t="n">
+        <v>173.0689</v>
+      </c>
       <c r="I32" s="21">
         <f>IF(OR($B32="",$H32=""),"",IF($C32="LONG",($H32-$E32)*$F32,($E32-$H32)*$F32))</f>
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>272.16</v>
+        <v>499.18</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -2984,14 +2992,18 @@
       <c r="F34" s="26" t="n">
         <v>284</v>
       </c>
-      <c r="G34" s="24" t="inlineStr"/>
-      <c r="H34" s="25" t="inlineStr"/>
+      <c r="G34" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H34" s="25" t="n">
+        <v>587.8211</v>
+      </c>
       <c r="I34" s="21">
         <f>IF(OR($B34="",$H34=""),"",IF($C34="LONG",($H34-$E34)*$F34,($E34-$H34)*$F34))</f>
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>271.36</v>
+        <v>502.95</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3031,14 +3043,18 @@
       <c r="F35" s="26" t="n">
         <v>375</v>
       </c>
-      <c r="G35" s="24" t="inlineStr"/>
-      <c r="H35" s="25" t="inlineStr"/>
+      <c r="G35" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H35" s="25" t="n">
+        <v>424.3155</v>
+      </c>
       <c r="I35" s="21">
         <f>IF(OR($B35="",$H35=""),"",IF($C35="LONG",($H35-$E35)*$F35,($E35-$H35)*$F35))</f>
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>271.43</v>
+        <v>492.96</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3156,19 +3172,43 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="n"/>
-      <c r="B38" s="23" t="n"/>
-      <c r="C38" s="23" t="n"/>
-      <c r="D38" s="24" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="25" t="n"/>
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082553409</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>GUJTHEM</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>412.5647</v>
+      </c>
+      <c r="F38" s="26" t="n">
+        <v>405</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H38" s="25" t="n">
+        <v>404.7939</v>
+      </c>
       <c r="I38" s="21">
         <f>IF(OR($B38="",$H38=""),"",IF($C38="LONG",($H38-$E38)*$F38,($E38-$H38)*$F38))</f>
         <v/>
       </c>
-      <c r="J38" s="4" t="n"/>
+      <c r="J38" s="4" t="n">
+        <v>106.27</v>
+      </c>
       <c r="K38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($J38="",0,$J38))</f>
         <v/>
@@ -3183,19 +3223,43 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="n"/>
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="25" t="n"/>
-      <c r="F39" s="26" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="25" t="n"/>
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260825378209</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>KCP</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>173.0006</v>
+      </c>
+      <c r="F39" s="26" t="n">
+        <v>942</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H39" s="25" t="n">
+        <v>177.3819</v>
+      </c>
       <c r="I39" s="21">
         <f>IF(OR($B39="",$H39=""),"",IF($C39="LONG",($H39-$E39)*$F39,($E39-$H39)*$F39))</f>
         <v/>
       </c>
-      <c r="J39" s="4" t="n"/>
+      <c r="J39" s="4" t="n">
+        <v>105.3</v>
+      </c>
       <c r="K39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($J39="",0,$J39))</f>
         <v/>
@@ -3210,19 +3274,43 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="n"/>
-      <c r="B40" s="23" t="n"/>
-      <c r="C40" s="23" t="n"/>
-      <c r="D40" s="24" t="n"/>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="26" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="25" t="n"/>
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260825110209</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>OPTIEMUS</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>587.5364</v>
+      </c>
+      <c r="F40" s="26" t="n">
+        <v>284</v>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H40" s="25" t="n">
+        <v>595.4639</v>
+      </c>
       <c r="I40" s="21">
         <f>IF(OR($B40="",$H40=""),"",IF($C40="LONG",($H40-$E40)*$F40,($E40-$H40)*$F40))</f>
         <v/>
       </c>
-      <c r="J40" s="4" t="n"/>
+      <c r="J40" s="4" t="n">
+        <v>106.56</v>
+      </c>
       <c r="K40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($J40="",0,$J40))</f>
         <v/>
@@ -3237,19 +3325,43 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="n"/>
-      <c r="B41" s="23" t="n"/>
-      <c r="C41" s="23" t="n"/>
-      <c r="D41" s="24" t="n"/>
-      <c r="E41" s="25" t="n"/>
-      <c r="F41" s="26" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="25" t="n"/>
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082553709</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>QUADFUTURE</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>424.2342</v>
+      </c>
+      <c r="F41" s="26" t="n">
+        <v>375</v>
+      </c>
+      <c r="G41" s="24" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H41" s="25" t="n">
+        <v>419.3061</v>
+      </c>
       <c r="I41" s="21">
         <f>IF(OR($B41="",$H41=""),"",IF($C41="LONG",($H41-$E41)*$F41,($E41-$H41)*$F41))</f>
         <v/>
       </c>
-      <c r="J41" s="4" t="n"/>
+      <c r="J41" s="4" t="n">
+        <v>103.52</v>
+      </c>
       <c r="K41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($J41="",0,$J41))</f>
         <v/>

</xml_diff>

<commit_message>
Trim candle history to 6 months, backfill new symbols at 6mo not 1yr, EOD fill + trading data for 2026-08-26
- data/candles/*.csv: dropped everything older than 6 months (only 36
  trading days needed for the volume signal) -- 3.45M rows -> 1.61M,
  207MB -> 97MB
- pipeline/main.py: new-symbol onboarding now backfills 6 months of
  history instead of 1 year, matching the trim above
- Ran today's EOD 15-min fill (was missed while the crontab was
  reduced to test-only entries) and today's Dhan dry-run entry results
- Misc daily data refresh: market cap snapshot, universe list, Upstox/
  Kite instrument masters, strategy P&L workbook

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828</v>
+        <v>828.02</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.01</v>
+        <v>831.0700000000001</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.24</v>
+        <v>505.27</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.76</v>
+        <v>505.78</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.26</v>
+        <v>1179.3</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>502.95</v>
+        <v>502.98</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>492.96</v>
+        <v>492.87</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>

</xml_diff>

<commit_message>
Data update — 2026-08-27 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.02</v>
+        <v>828.04</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.0700000000001</v>
+        <v>831.15</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.27</v>
+        <v>505.26</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.78</v>
+        <v>505.81</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.3</v>
+        <v>1179.49</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>502.98</v>
+        <v>502.99</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>492.87</v>
+        <v>480.6</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3376,19 +3376,39 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="n"/>
-      <c r="B42" s="23" t="n"/>
-      <c r="C42" s="23" t="n"/>
-      <c r="D42" s="24" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="26" t="n"/>
-      <c r="G42" s="24" t="n"/>
-      <c r="H42" s="25" t="n"/>
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126082781609</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>BOMDYEING</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E42" s="25" t="n">
+        <v>116.9946</v>
+      </c>
+      <c r="F42" s="26" t="n">
+        <v>2991</v>
+      </c>
+      <c r="G42" s="24" t="inlineStr"/>
+      <c r="H42" s="25" t="inlineStr"/>
       <c r="I42" s="21">
         <f>IF(OR($B42="",$H42=""),"",IF($C42="LONG",($H42-$E42)*$F42,($E42-$H42)*$F42))</f>
         <v/>
       </c>
-      <c r="J42" s="4" t="n"/>
+      <c r="J42" s="4" t="n">
+        <v>489.26</v>
+      </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
         <v/>
@@ -3403,19 +3423,39 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="23" t="n"/>
-      <c r="B43" s="23" t="n"/>
-      <c r="C43" s="23" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="26" t="n"/>
-      <c r="G43" s="24" t="n"/>
-      <c r="H43" s="25" t="n"/>
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260827577609</t>
+        </is>
+      </c>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>GKENERGY</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E43" s="25" t="n">
+        <v>139.6491</v>
+      </c>
+      <c r="F43" s="26" t="n">
+        <v>2508</v>
+      </c>
+      <c r="G43" s="24" t="inlineStr"/>
+      <c r="H43" s="25" t="inlineStr"/>
       <c r="I43" s="21">
         <f>IF(OR($B43="",$H43=""),"",IF($C43="LONG",($H43-$E43)*$F43,($E43-$H43)*$F43))</f>
         <v/>
       </c>
-      <c r="J43" s="4" t="n"/>
+      <c r="J43" s="4" t="n">
+        <v>489.63</v>
+      </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
         <v/>
@@ -3430,19 +3470,39 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="23" t="n"/>
-      <c r="B44" s="23" t="n"/>
-      <c r="C44" s="23" t="n"/>
-      <c r="D44" s="24" t="n"/>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="26" t="n"/>
-      <c r="G44" s="24" t="n"/>
-      <c r="H44" s="25" t="n"/>
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126082778209</t>
+        </is>
+      </c>
+      <c r="B44" s="23" t="inlineStr">
+        <is>
+          <t>RAMRAT</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E44" s="25" t="n">
+        <v>572.3033</v>
+      </c>
+      <c r="F44" s="26" t="n">
+        <v>614</v>
+      </c>
+      <c r="G44" s="24" t="inlineStr"/>
+      <c r="H44" s="25" t="inlineStr"/>
       <c r="I44" s="21">
         <f>IF(OR($B44="",$H44=""),"",IF($C44="LONG",($H44-$E44)*$F44,($E44-$H44)*$F44))</f>
         <v/>
       </c>
-      <c r="J44" s="4" t="n"/>
+      <c r="J44" s="4" t="n">
+        <v>491</v>
+      </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
         <v/>
@@ -29780,7 +29840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29950,7 +30010,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -29993,7 +30053,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30036,7 +30096,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30079,7 +30139,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30122,7 +30182,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30165,7 +30225,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30208,7 +30268,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30251,7 +30311,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30294,7 +30354,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30337,7 +30397,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30380,7 +30440,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -30423,7 +30483,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -30466,7 +30526,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -30509,7 +30569,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -30552,7 +30612,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -30595,7 +30655,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -30638,78 +30698,207 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
+          <t>THOMASCOOK</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A22)</f>
+        <v/>
+      </c>
+      <c r="C22" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E22" s="29">
+        <f>IFERROR($C22/$B22,"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G22" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H22" s="21">
+        <f>IFERROR($G22/$B22,"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B23" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D23" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E23" s="29">
+        <f>IFERROR($C23/$B23,"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G23" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A23,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H23" s="21">
+        <f>IFERROR($G23/$B23,"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A23),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B24" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D24" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E24" s="29">
+        <f>IFERROR($C24/$B24,"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G24" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A24,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H24" s="21">
+        <f>IFERROR($G24/$B24,"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A24),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B22" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A22)</f>
-        <v/>
-      </c>
-      <c r="C22" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D22" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E22" s="29">
-        <f>IFERROR($C22/$B22,"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G22" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A22,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H22" s="21">
-        <f>IFERROR($G22/$B22,"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A22),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="B25" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E25" s="29">
+        <f>IFERROR($C25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H25" s="21">
+        <f>IFERROR($G25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="30">
-        <f>SUM(B4:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="30">
-        <f>SUM(C4:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="30">
-        <f>SUM(D4:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="31">
-        <f>IFERROR(C23/B23,"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="32">
-        <f>SUM(F4:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="32">
-        <f>SUM(G4:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="32">
-        <f>IFERROR(G23/B23,"")</f>
+      <c r="B26" s="30">
+        <f>SUM(B4:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="30">
+        <f>SUM(C4:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="30">
+        <f>SUM(D4:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="31">
+        <f>IFERROR(C26/B26,"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="32">
+        <f>SUM(F4:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="32">
+        <f>SUM(G4:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="32">
+        <f>IFERROR(G26/B26,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-08-28 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.15</v>
+        <v>831.22</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.26</v>
+        <v>505.12</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.81</v>
+        <v>505.76</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.49</v>
+        <v>1179.69</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>502.99</v>
+        <v>503.02</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3407,7 +3407,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>489.26</v>
+        <v>561.0700000000001</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3454,7 +3454,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>489.63</v>
+        <v>549.52</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3501,7 +3501,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>491</v>
+        <v>563.1</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3517,19 +3517,39 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="23" t="n"/>
-      <c r="B45" s="23" t="n"/>
-      <c r="C45" s="23" t="n"/>
-      <c r="D45" s="24" t="n"/>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="26" t="n"/>
-      <c r="G45" s="24" t="n"/>
-      <c r="H45" s="25" t="n"/>
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2212608281405809</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>FMGOETZE</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E45" s="25" t="n">
+        <v>603.0422</v>
+      </c>
+      <c r="F45" s="26" t="n">
+        <v>464</v>
+      </c>
+      <c r="G45" s="24" t="inlineStr"/>
+      <c r="H45" s="25" t="inlineStr"/>
       <c r="I45" s="21">
         <f>IF(OR($B45="",$H45=""),"",IF($C45="LONG",($H45-$E45)*$F45,($E45-$H45)*$F45))</f>
         <v/>
       </c>
-      <c r="J45" s="4" t="n"/>
+      <c r="J45" s="4" t="n">
+        <v>406</v>
+      </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
         <v/>
@@ -3544,19 +3564,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="n"/>
-      <c r="B46" s="23" t="n"/>
-      <c r="C46" s="23" t="n"/>
-      <c r="D46" s="24" t="n"/>
-      <c r="E46" s="25" t="n"/>
-      <c r="F46" s="26" t="n"/>
-      <c r="G46" s="24" t="n"/>
-      <c r="H46" s="25" t="n"/>
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2312608281035809</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>JGCHEM</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D46" s="24" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E46" s="25" t="n">
+        <v>655.6077</v>
+      </c>
+      <c r="F46" s="26" t="n">
+        <v>428</v>
+      </c>
+      <c r="G46" s="24" t="inlineStr"/>
+      <c r="H46" s="25" t="inlineStr"/>
       <c r="I46" s="21">
         <f>IF(OR($B46="",$H46=""),"",IF($C46="LONG",($H46-$E46)*$F46,($E46-$H46)*$F46))</f>
         <v/>
       </c>
-      <c r="J46" s="4" t="n"/>
+      <c r="J46" s="4" t="n">
+        <v>406.94</v>
+      </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
         <v/>
@@ -3571,19 +3611,39 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="23" t="n"/>
-      <c r="B47" s="23" t="n"/>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="24" t="n"/>
-      <c r="E47" s="25" t="n"/>
-      <c r="F47" s="26" t="n"/>
-      <c r="G47" s="24" t="n"/>
-      <c r="H47" s="25" t="n"/>
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2312608281035709</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>MASTEK</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D47" s="24" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>1908.9741</v>
+      </c>
+      <c r="F47" s="26" t="n">
+        <v>147</v>
+      </c>
+      <c r="G47" s="24" t="inlineStr"/>
+      <c r="H47" s="25" t="inlineStr"/>
       <c r="I47" s="21">
         <f>IF(OR($B47="",$H47=""),"",IF($C47="LONG",($H47-$E47)*$F47,($E47-$H47)*$F47))</f>
         <v/>
       </c>
-      <c r="J47" s="4" t="n"/>
+      <c r="J47" s="4" t="n">
+        <v>406.96</v>
+      </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
         <v/>
@@ -3598,19 +3658,39 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="23" t="n"/>
-      <c r="B48" s="23" t="n"/>
-      <c r="C48" s="23" t="n"/>
-      <c r="D48" s="24" t="n"/>
-      <c r="E48" s="25" t="n"/>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="24" t="n"/>
-      <c r="H48" s="25" t="n"/>
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2212608281405909</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>OMAXE</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E48" s="25" t="n">
+        <v>130.8863</v>
+      </c>
+      <c r="F48" s="26" t="n">
+        <v>2161</v>
+      </c>
+      <c r="G48" s="24" t="inlineStr"/>
+      <c r="H48" s="25" t="inlineStr"/>
       <c r="I48" s="21">
         <f>IF(OR($B48="",$H48=""),"",IF($C48="LONG",($H48-$E48)*$F48,($E48-$H48)*$F48))</f>
         <v/>
       </c>
-      <c r="J48" s="4" t="n"/>
+      <c r="J48" s="4" t="n">
+        <v>409.6</v>
+      </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
         <v/>
@@ -3625,19 +3705,39 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="23" t="n"/>
-      <c r="B49" s="23" t="n"/>
-      <c r="C49" s="23" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="25" t="n"/>
-      <c r="F49" s="26" t="n"/>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="25" t="n"/>
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-2312608281035909</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D49" s="24" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E49" s="25" t="n">
+        <v>19.4799</v>
+      </c>
+      <c r="F49" s="26" t="n">
+        <v>14462</v>
+      </c>
+      <c r="G49" s="24" t="inlineStr"/>
+      <c r="H49" s="25" t="inlineStr"/>
       <c r="I49" s="21">
         <f>IF(OR($B49="",$H49=""),"",IF($C49="LONG",($H49-$E49)*$F49,($E49-$H49)*$F49))</f>
         <v/>
       </c>
-      <c r="J49" s="4" t="n"/>
+      <c r="J49" s="4" t="n">
+        <v>408.26</v>
+      </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
         <v/>
@@ -29840,7 +29940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30053,7 +30153,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30096,7 +30196,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30139,7 +30239,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30182,7 +30282,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30225,7 +30325,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30268,7 +30368,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30311,7 +30411,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30354,7 +30454,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30397,7 +30497,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30440,7 +30540,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -30483,7 +30583,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -30526,7 +30626,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -30569,7 +30669,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -30612,7 +30712,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -30655,7 +30755,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -30698,7 +30798,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -30741,7 +30841,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -30784,7 +30884,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -30827,78 +30927,293 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
+          <t>SOLARA</t>
+        </is>
+      </c>
+      <c r="B25" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E25" s="29">
+        <f>IFERROR($C25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G25" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H25" s="21">
+        <f>IFERROR($G25/$B25,"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="B26" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A26)</f>
+        <v/>
+      </c>
+      <c r="C26" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D26" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E26" s="29">
+        <f>IFERROR($C26/$B26,"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G26" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A26,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H26" s="21">
+        <f>IFERROR($G26/$B26,"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A26),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>THOMASCOOK</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A27)</f>
+        <v/>
+      </c>
+      <c r="C27" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D27" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E27" s="29">
+        <f>IFERROR($C27/$B27,"")</f>
+        <v/>
+      </c>
+      <c r="F27" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G27" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A27,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H27" s="21">
+        <f>IFERROR($G27/$B27,"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A27),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B28" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D28" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E28" s="29">
+        <f>IFERROR($C28/$B28,"")</f>
+        <v/>
+      </c>
+      <c r="F28" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A28,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H28" s="21">
+        <f>IFERROR($G28/$B28,"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A28),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B29" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D29" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E29" s="29">
+        <f>IFERROR($C29/$B29,"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G29" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A29,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H29" s="21">
+        <f>IFERROR($G29/$B29,"")</f>
+        <v/>
+      </c>
+      <c r="I29" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A29),"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B25" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A25)</f>
-        <v/>
-      </c>
-      <c r="C25" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D25" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E25" s="29">
-        <f>IFERROR($C25/$B25,"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G25" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A25,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H25" s="21">
-        <f>IFERROR($G25/$B25,"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A25),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="B30" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E30" s="29">
+        <f>IFERROR($C30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="F30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H30" s="21">
+        <f>IFERROR($G30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B26" s="30">
-        <f>SUM(B4:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="30">
-        <f>SUM(C4:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="30">
-        <f>SUM(D4:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="31">
-        <f>IFERROR(C26/B26,"")</f>
-        <v/>
-      </c>
-      <c r="F26" s="32">
-        <f>SUM(F4:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="32">
-        <f>SUM(G4:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="32">
-        <f>IFERROR(G26/B26,"")</f>
+      <c r="B31" s="30">
+        <f>SUM(B4:B30)</f>
+        <v/>
+      </c>
+      <c r="C31" s="30">
+        <f>SUM(C4:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="30">
+        <f>SUM(D4:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="31">
+        <f>IFERROR(C31/B31,"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="32">
+        <f>SUM(F4:F30)</f>
+        <v/>
+      </c>
+      <c r="G31" s="32">
+        <f>SUM(G4:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="32">
+        <f>IFERROR(G31/B31,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-08-31 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.04</v>
+        <v>828.0599999999999</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.22</v>
+        <v>831.29</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.76</v>
+        <v>505.78</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.69</v>
+        <v>1179.84</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.02</v>
+        <v>503.06</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3553,14 +3553,18 @@
       <c r="F45" s="26" t="n">
         <v>464</v>
       </c>
-      <c r="G45" s="24" t="inlineStr"/>
-      <c r="H45" s="25" t="inlineStr"/>
+      <c r="G45" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H45" s="25" t="n">
+        <v>625.1997</v>
+      </c>
       <c r="I45" s="21">
         <f>IF(OR($B45="",$H45=""),"",IF($C45="LONG",($H45-$E45)*$F45,($E45-$H45)*$F45))</f>
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>406</v>
+        <v>902.8</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3600,14 +3604,18 @@
       <c r="F46" s="26" t="n">
         <v>428</v>
       </c>
-      <c r="G46" s="24" t="inlineStr"/>
-      <c r="H46" s="25" t="inlineStr"/>
+      <c r="G46" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H46" s="25" t="n">
+        <v>650.2959</v>
+      </c>
       <c r="I46" s="21">
         <f>IF(OR($B46="",$H46=""),"",IF($C46="LONG",($H46-$E46)*$F46,($E46-$H46)*$F46))</f>
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>406.94</v>
+        <v>892.01</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3647,14 +3655,18 @@
       <c r="F47" s="26" t="n">
         <v>147</v>
       </c>
-      <c r="G47" s="24" t="inlineStr"/>
-      <c r="H47" s="25" t="inlineStr"/>
+      <c r="G47" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H47" s="25" t="n">
+        <v>1777.534</v>
+      </c>
       <c r="I47" s="21">
         <f>IF(OR($B47="",$H47=""),"",IF($C47="LONG",($H47-$E47)*$F47,($E47-$H47)*$F47))</f>
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>406.96</v>
+        <v>889.41</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3694,14 +3706,18 @@
       <c r="F48" s="26" t="n">
         <v>2161</v>
       </c>
-      <c r="G48" s="24" t="inlineStr"/>
-      <c r="H48" s="25" t="inlineStr"/>
+      <c r="G48" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H48" s="25" t="n">
+        <v>130.9149</v>
+      </c>
       <c r="I48" s="21">
         <f>IF(OR($B48="",$H48=""),"",IF($C48="LONG",($H48-$E48)*$F48,($E48-$H48)*$F48))</f>
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>409.6</v>
+        <v>899.3</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3741,14 +3757,18 @@
       <c r="F49" s="26" t="n">
         <v>14462</v>
       </c>
-      <c r="G49" s="24" t="inlineStr"/>
-      <c r="H49" s="25" t="inlineStr"/>
+      <c r="G49" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H49" s="25" t="n">
+        <v>19.6094</v>
+      </c>
       <c r="I49" s="21">
         <f>IF(OR($B49="",$H49=""),"",IF($C49="LONG",($H49-$E49)*$F49,($E49-$H49)*$F49))</f>
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>408.26</v>
+        <v>870.58</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3764,19 +3784,39 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="23" t="n"/>
-      <c r="B50" s="23" t="n"/>
-      <c r="C50" s="23" t="n"/>
-      <c r="D50" s="24" t="n"/>
-      <c r="E50" s="25" t="n"/>
-      <c r="F50" s="26" t="n"/>
-      <c r="G50" s="24" t="n"/>
-      <c r="H50" s="25" t="n"/>
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231260831122409</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>ASHOKA</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D50" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E50" s="25" t="n">
+        <v>120.2727</v>
+      </c>
+      <c r="F50" s="26" t="n">
+        <v>2933</v>
+      </c>
+      <c r="G50" s="24" t="inlineStr"/>
+      <c r="H50" s="25" t="inlineStr"/>
       <c r="I50" s="21">
         <f>IF(OR($B50="",$H50=""),"",IF($C50="LONG",($H50-$E50)*$F50,($E50-$H50)*$F50))</f>
         <v/>
       </c>
-      <c r="J50" s="4" t="n"/>
+      <c r="J50" s="4" t="n">
+        <v>492.62</v>
+      </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
         <v/>
@@ -3791,19 +3831,43 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="23" t="n"/>
-      <c r="B51" s="23" t="n"/>
-      <c r="C51" s="23" t="n"/>
-      <c r="D51" s="24" t="n"/>
-      <c r="E51" s="25" t="n"/>
-      <c r="F51" s="26" t="n"/>
-      <c r="G51" s="24" t="n"/>
-      <c r="H51" s="25" t="n"/>
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260831109609</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>FMGOETZE</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>625.4782</v>
+      </c>
+      <c r="F51" s="26" t="n">
+        <v>464</v>
+      </c>
+      <c r="G51" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H51" s="25" t="n">
+        <v>620</v>
+      </c>
       <c r="I51" s="21">
         <f>IF(OR($B51="",$H51=""),"",IF($C51="LONG",($H51-$E51)*$F51,($E51-$H51)*$F51))</f>
         <v/>
       </c>
-      <c r="J51" s="4" t="n"/>
+      <c r="J51" s="4" t="n">
+        <v>150</v>
+      </c>
       <c r="K51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($J51="",0,$J51))</f>
         <v/>
@@ -3818,19 +3882,43 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="23" t="n"/>
-      <c r="B52" s="23" t="n"/>
-      <c r="C52" s="23" t="n"/>
-      <c r="D52" s="24" t="n"/>
-      <c r="E52" s="25" t="n"/>
-      <c r="F52" s="26" t="n"/>
-      <c r="G52" s="24" t="n"/>
-      <c r="H52" s="25" t="n"/>
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260831423609</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>JGCHEM</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>648.4623</v>
+      </c>
+      <c r="F52" s="26" t="n">
+        <v>428</v>
+      </c>
+      <c r="G52" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H52" s="25" t="n">
+        <v>638.2939</v>
+      </c>
       <c r="I52" s="21">
         <f>IF(OR($B52="",$H52=""),"",IF($C52="LONG",($H52-$E52)*$F52,($E52-$H52)*$F52))</f>
         <v/>
       </c>
-      <c r="J52" s="4" t="n"/>
+      <c r="J52" s="4" t="n">
+        <v>145.38</v>
+      </c>
       <c r="K52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($J52="",0,$J52))</f>
         <v/>
@@ -3845,19 +3933,43 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="23" t="n"/>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="24" t="n"/>
-      <c r="E53" s="25" t="n"/>
-      <c r="F53" s="26" t="n"/>
-      <c r="G53" s="24" t="n"/>
-      <c r="H53" s="25" t="n"/>
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126083156509</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>MASTEK</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>1777.6041</v>
+      </c>
+      <c r="F53" s="26" t="n">
+        <v>147</v>
+      </c>
+      <c r="G53" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H53" s="25" t="n">
+        <v>1777.866</v>
+      </c>
       <c r="I53" s="21">
         <f>IF(OR($B53="",$H53=""),"",IF($C53="LONG",($H53-$E53)*$F53,($E53-$H53)*$F53))</f>
         <v/>
       </c>
-      <c r="J53" s="4" t="n"/>
+      <c r="J53" s="4" t="n">
+        <v>139.92</v>
+      </c>
       <c r="K53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($J53="",0,$J53))</f>
         <v/>
@@ -3872,19 +3984,39 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="n"/>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="23" t="n"/>
-      <c r="D54" s="24" t="n"/>
-      <c r="E54" s="25" t="n"/>
-      <c r="F54" s="26" t="n"/>
-      <c r="G54" s="24" t="n"/>
-      <c r="H54" s="25" t="n"/>
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231260831122309</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>NORTHARC</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D54" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E54" s="25" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="F54" s="26" t="n">
+        <v>1117</v>
+      </c>
+      <c r="G54" s="24" t="inlineStr"/>
+      <c r="H54" s="25" t="inlineStr"/>
       <c r="I54" s="21">
         <f>IF(OR($B54="",$H54=""),"",IF($C54="LONG",($H54-$E54)*$F54,($E54-$H54)*$F54))</f>
         <v/>
       </c>
-      <c r="J54" s="4" t="n"/>
+      <c r="J54" s="4" t="n">
+        <v>485.58</v>
+      </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
         <v/>
@@ -3899,19 +4031,43 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="23" t="n"/>
-      <c r="B55" s="23" t="n"/>
-      <c r="C55" s="23" t="n"/>
-      <c r="D55" s="24" t="n"/>
-      <c r="E55" s="25" t="n"/>
-      <c r="F55" s="26" t="n"/>
-      <c r="G55" s="24" t="n"/>
-      <c r="H55" s="25" t="n"/>
+      <c r="A55" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126083118409</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>OMAXE</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E55" s="25" t="n">
+        <v>130.7703</v>
+      </c>
+      <c r="F55" s="26" t="n">
+        <v>2161</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H55" s="25" t="n">
+        <v>126.3456</v>
+      </c>
       <c r="I55" s="21">
         <f>IF(OR($B55="",$H55=""),"",IF($C55="LONG",($H55-$E55)*$F55,($E55-$H55)*$F55))</f>
         <v/>
       </c>
-      <c r="J55" s="4" t="n"/>
+      <c r="J55" s="4" t="n">
+        <v>146.82</v>
+      </c>
       <c r="K55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($J55="",0,$J55))</f>
         <v/>
@@ -3926,19 +4082,43 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="n"/>
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="24" t="n"/>
-      <c r="E56" s="25" t="n"/>
-      <c r="F56" s="26" t="n"/>
-      <c r="G56" s="24" t="n"/>
-      <c r="H56" s="25" t="n"/>
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260831104409</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D56" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E56" s="25" t="n">
+        <v>19.6247</v>
+      </c>
+      <c r="F56" s="26" t="n">
+        <v>14462</v>
+      </c>
+      <c r="G56" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="H56" s="25" t="n">
+        <v>19.5263</v>
+      </c>
       <c r="I56" s="21">
         <f>IF(OR($B56="",$H56=""),"",IF($C56="LONG",($H56-$E56)*$F56,($E56-$H56)*$F56))</f>
         <v/>
       </c>
-      <c r="J56" s="4" t="n"/>
+      <c r="J56" s="4" t="n">
+        <v>147.8</v>
+      </c>
       <c r="K56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($J56="",0,$J56))</f>
         <v/>
@@ -3953,19 +4133,39 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="23" t="n"/>
-      <c r="B57" s="23" t="n"/>
-      <c r="C57" s="23" t="n"/>
-      <c r="D57" s="24" t="n"/>
-      <c r="E57" s="25" t="n"/>
-      <c r="F57" s="26" t="n"/>
-      <c r="G57" s="24" t="n"/>
-      <c r="H57" s="25" t="n"/>
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260831702509</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>VENKEYS</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D57" s="24" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E57" s="25" t="n">
+        <v>1702.7395</v>
+      </c>
+      <c r="F57" s="26" t="n">
+        <v>205</v>
+      </c>
+      <c r="G57" s="24" t="inlineStr"/>
+      <c r="H57" s="25" t="inlineStr"/>
       <c r="I57" s="21">
         <f>IF(OR($B57="",$H57=""),"",IF($C57="LONG",($H57-$E57)*$F57,($E57-$H57)*$F57))</f>
         <v/>
       </c>
-      <c r="J57" s="4" t="n"/>
+      <c r="J57" s="4" t="n">
+        <v>488.23</v>
+      </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
         <v/>
@@ -29952,7 +30152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30036,7 +30236,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B4" s="20">
@@ -30079,7 +30279,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -30122,7 +30322,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30165,7 +30365,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30208,7 +30408,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30251,7 +30451,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30294,7 +30494,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30337,7 +30537,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30380,7 +30580,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30423,7 +30623,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30466,7 +30666,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30509,7 +30709,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30552,7 +30752,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -30595,7 +30795,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -30638,7 +30838,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -30681,7 +30881,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -30724,7 +30924,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -30767,7 +30967,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -30810,7 +31010,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -30853,7 +31053,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -30896,7 +31096,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -30939,7 +31139,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -30982,7 +31182,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31025,7 +31225,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31068,7 +31268,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31111,7 +31311,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31154,78 +31354,207 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
+          <t>VENKEYS</t>
+        </is>
+      </c>
+      <c r="B30" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D30" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E30" s="29">
+        <f>IFERROR($C30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="F30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G30" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H30" s="21">
+        <f>IFERROR($G30/$B30,"")</f>
+        <v/>
+      </c>
+      <c r="I30" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B31" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D31" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E31" s="29">
+        <f>IFERROR($C31/$B31,"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G31" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A31,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H31" s="21">
+        <f>IFERROR($G31/$B31,"")</f>
+        <v/>
+      </c>
+      <c r="I31" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A31),"")</f>
+        <v/>
+      </c>
+      <c r="J31" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B32" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D32" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E32" s="29">
+        <f>IFERROR($C32/$B32,"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G32" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A32,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H32" s="21">
+        <f>IFERROR($G32/$B32,"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A32),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B30" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A30)</f>
-        <v/>
-      </c>
-      <c r="C30" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D30" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E30" s="29">
-        <f>IFERROR($C30/$B30,"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G30" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A30,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H30" s="21">
-        <f>IFERROR($G30/$B30,"")</f>
-        <v/>
-      </c>
-      <c r="I30" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A30),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="B33" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E33" s="29">
+        <f>IFERROR($C33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H33" s="21">
+        <f>IFERROR($G33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B31" s="30">
-        <f>SUM(B4:B30)</f>
-        <v/>
-      </c>
-      <c r="C31" s="30">
-        <f>SUM(C4:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="30">
-        <f>SUM(D4:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="31">
-        <f>IFERROR(C31/B31,"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="32">
-        <f>SUM(F4:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="32">
-        <f>SUM(G4:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="32">
-        <f>IFERROR(G31/B31,"")</f>
+      <c r="B34" s="30">
+        <f>SUM(B4:B33)</f>
+        <v/>
+      </c>
+      <c r="C34" s="30">
+        <f>SUM(C4:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="30">
+        <f>SUM(D4:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="31">
+        <f>IFERROR(C34/B34,"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="32">
+        <f>SUM(F4:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="32">
+        <f>SUM(G4:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="32">
+        <f>IFERROR(G34/B34,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-01 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>810.1</v>
+        <v>824.42</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.0599999999999</v>
+        <v>828.09</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.29</v>
+        <v>831.3099999999999</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>505.12</v>
+        <v>504.96</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.78</v>
+        <v>505.69</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1179.84</v>
+        <v>1180.03</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.06</v>
+        <v>503.08</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>889.41</v>
+        <v>888.46</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>899.3</v>
+        <v>899.13</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3808,14 +3808,18 @@
       <c r="F50" s="26" t="n">
         <v>2933</v>
       </c>
-      <c r="G50" s="24" t="inlineStr"/>
-      <c r="H50" s="25" t="inlineStr"/>
+      <c r="G50" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H50" s="25" t="n">
+        <v>121.8089</v>
+      </c>
       <c r="I50" s="21">
         <f>IF(OR($B50="",$H50=""),"",IF($C50="LONG",($H50-$E50)*$F50,($E50-$H50)*$F50))</f>
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>492.62</v>
+        <v>966.9299999999999</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4008,14 +4012,18 @@
       <c r="F54" s="26" t="n">
         <v>1117</v>
       </c>
-      <c r="G54" s="24" t="inlineStr"/>
-      <c r="H54" s="25" t="inlineStr"/>
+      <c r="G54" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H54" s="25" t="n">
+        <v>303.0902</v>
+      </c>
       <c r="I54" s="21">
         <f>IF(OR($B54="",$H54=""),"",IF($C54="LONG",($H54-$E54)*$F54,($E54-$H54)*$F54))</f>
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>485.58</v>
+        <v>939.3200000000001</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4157,14 +4165,18 @@
       <c r="F57" s="26" t="n">
         <v>205</v>
       </c>
-      <c r="G57" s="24" t="inlineStr"/>
-      <c r="H57" s="25" t="inlineStr"/>
+      <c r="G57" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H57" s="25" t="n">
+        <v>1666.1965</v>
+      </c>
       <c r="I57" s="21">
         <f>IF(OR($B57="",$H57=""),"",IF($C57="LONG",($H57-$E57)*$F57,($E57-$H57)*$F57))</f>
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>488.23</v>
+        <v>937.8</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4180,19 +4192,43 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="23" t="n"/>
-      <c r="B58" s="23" t="n"/>
-      <c r="C58" s="23" t="n"/>
-      <c r="D58" s="24" t="n"/>
-      <c r="E58" s="25" t="n"/>
-      <c r="F58" s="26" t="n"/>
-      <c r="G58" s="24" t="n"/>
-      <c r="H58" s="25" t="n"/>
+      <c r="A58" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126090197109</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>ASHOKA</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D58" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E58" s="25" t="n">
+        <v>121.775</v>
+      </c>
+      <c r="F58" s="26" t="n">
+        <v>2933</v>
+      </c>
+      <c r="G58" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H58" s="25" t="n">
+        <v>122.25</v>
+      </c>
       <c r="I58" s="21">
         <f>IF(OR($B58="",$H58=""),"",IF($C58="LONG",($H58-$E58)*$F58,($E58-$H58)*$F58))</f>
         <v/>
       </c>
-      <c r="J58" s="4" t="n"/>
+      <c r="J58" s="4" t="n">
+        <v>174.02</v>
+      </c>
       <c r="K58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($J58="",0,$J58))</f>
         <v/>
@@ -4207,19 +4243,43 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="23" t="n"/>
-      <c r="B59" s="23" t="n"/>
-      <c r="C59" s="23" t="n"/>
-      <c r="D59" s="24" t="n"/>
-      <c r="E59" s="25" t="n"/>
-      <c r="F59" s="26" t="n"/>
-      <c r="G59" s="24" t="n"/>
-      <c r="H59" s="25" t="n"/>
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260901437609</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>NORTHARC</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D59" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E59" s="25" t="n">
+        <v>303.0625</v>
+      </c>
+      <c r="F59" s="26" t="n">
+        <v>1117</v>
+      </c>
+      <c r="G59" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H59" s="25" t="n">
+        <v>299.1408</v>
+      </c>
       <c r="I59" s="21">
         <f>IF(OR($B59="",$H59=""),"",IF($C59="LONG",($H59-$E59)*$F59,($E59-$H59)*$F59))</f>
         <v/>
       </c>
-      <c r="J59" s="4" t="n"/>
+      <c r="J59" s="4" t="n">
+        <v>167.02</v>
+      </c>
       <c r="K59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($J59="",0,$J59))</f>
         <v/>
@@ -4234,19 +4294,39 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="23" t="n"/>
-      <c r="B60" s="23" t="n"/>
-      <c r="C60" s="23" t="n"/>
-      <c r="D60" s="24" t="n"/>
-      <c r="E60" s="25" t="n"/>
-      <c r="F60" s="26" t="n"/>
-      <c r="G60" s="24" t="n"/>
-      <c r="H60" s="25" t="n"/>
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260901669709</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>SAKAR</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D60" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E60" s="25" t="n">
+        <v>961.5373</v>
+      </c>
+      <c r="F60" s="26" t="n">
+        <v>181</v>
+      </c>
+      <c r="G60" s="24" t="inlineStr"/>
+      <c r="H60" s="25" t="inlineStr"/>
       <c r="I60" s="21">
         <f>IF(OR($B60="",$H60=""),"",IF($C60="LONG",($H60-$E60)*$F60,($E60-$H60)*$F60))</f>
         <v/>
       </c>
-      <c r="J60" s="4" t="n"/>
+      <c r="J60" s="4" t="n">
+        <v>221.4</v>
+      </c>
       <c r="K60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($J60="",0,$J60))</f>
         <v/>
@@ -4261,19 +4341,39 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="23" t="n"/>
-      <c r="B61" s="23" t="n"/>
-      <c r="C61" s="23" t="n"/>
-      <c r="D61" s="24" t="n"/>
-      <c r="E61" s="25" t="n"/>
-      <c r="F61" s="26" t="n"/>
-      <c r="G61" s="24" t="n"/>
-      <c r="H61" s="25" t="n"/>
+      <c r="A61" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260901678509</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>SOTL</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D61" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E61" s="25" t="n">
+        <v>773.7782999999999</v>
+      </c>
+      <c r="F61" s="26" t="n">
+        <v>454</v>
+      </c>
+      <c r="G61" s="24" t="inlineStr"/>
+      <c r="H61" s="25" t="inlineStr"/>
       <c r="I61" s="21">
         <f>IF(OR($B61="",$H61=""),"",IF($C61="LONG",($H61-$E61)*$F61,($E61-$H61)*$F61))</f>
         <v/>
       </c>
-      <c r="J61" s="4" t="n"/>
+      <c r="J61" s="4" t="n">
+        <v>490.88</v>
+      </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
         <v/>
@@ -4288,19 +4388,39 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="23" t="n"/>
-      <c r="B62" s="23" t="n"/>
-      <c r="C62" s="23" t="n"/>
-      <c r="D62" s="24" t="n"/>
-      <c r="E62" s="25" t="n"/>
-      <c r="F62" s="26" t="n"/>
-      <c r="G62" s="24" t="n"/>
-      <c r="H62" s="25" t="n"/>
+      <c r="A62" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090172909</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>SSWL</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D62" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E62" s="25" t="n">
+        <v>361.4802</v>
+      </c>
+      <c r="F62" s="26" t="n">
+        <v>981</v>
+      </c>
+      <c r="G62" s="24" t="inlineStr"/>
+      <c r="H62" s="25" t="inlineStr"/>
       <c r="I62" s="21">
         <f>IF(OR($B62="",$H62=""),"",IF($C62="LONG",($H62-$E62)*$F62,($E62-$H62)*$F62))</f>
         <v/>
       </c>
-      <c r="J62" s="4" t="n"/>
+      <c r="J62" s="4" t="n">
+        <v>494.82</v>
+      </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
         <v/>
@@ -4315,19 +4435,43 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="23" t="n"/>
-      <c r="B63" s="23" t="n"/>
-      <c r="C63" s="23" t="n"/>
-      <c r="D63" s="24" t="n"/>
-      <c r="E63" s="25" t="n"/>
-      <c r="F63" s="26" t="n"/>
-      <c r="G63" s="24" t="n"/>
-      <c r="H63" s="25" t="n"/>
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090154109</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>VENKEYS</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D63" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E63" s="25" t="n">
+        <v>1664.2166</v>
+      </c>
+      <c r="F63" s="26" t="n">
+        <v>205</v>
+      </c>
+      <c r="G63" s="24" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H63" s="25" t="n">
+        <v>1647.3204</v>
+      </c>
       <c r="I63" s="21">
         <f>IF(OR($B63="",$H63=""),"",IF($C63="LONG",($H63-$E63)*$F63,($E63-$H63)*$F63))</f>
         <v/>
       </c>
-      <c r="J63" s="4" t="n"/>
+      <c r="J63" s="4" t="n">
+        <v>168.01</v>
+      </c>
       <c r="K63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($J63="",0,$J63))</f>
         <v/>
@@ -30152,7 +30296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31225,7 +31369,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31268,7 +31412,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31311,7 +31455,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31354,7 +31498,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -31397,7 +31541,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -31440,7 +31584,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -31483,78 +31627,207 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
+          <t>VENKEYS</t>
+        </is>
+      </c>
+      <c r="B33" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D33" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E33" s="29">
+        <f>IFERROR($C33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G33" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H33" s="21">
+        <f>IFERROR($G33/$B33,"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B34" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A34)</f>
+        <v/>
+      </c>
+      <c r="C34" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E34" s="29">
+        <f>IFERROR($C34/$B34,"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G34" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A34,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H34" s="21">
+        <f>IFERROR($G34/$B34,"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A34),"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B35" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A35)</f>
+        <v/>
+      </c>
+      <c r="C35" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D35" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E35" s="29">
+        <f>IFERROR($C35/$B35,"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G35" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A35,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H35" s="21">
+        <f>IFERROR($G35/$B35,"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A35),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B33" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A33)</f>
-        <v/>
-      </c>
-      <c r="C33" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D33" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E33" s="29">
-        <f>IFERROR($C33/$B33,"")</f>
-        <v/>
-      </c>
-      <c r="F33" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G33" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A33,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H33" s="21">
-        <f>IFERROR($G33/$B33,"")</f>
-        <v/>
-      </c>
-      <c r="I33" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A33),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="B36" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E36" s="29">
+        <f>IFERROR($C36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H36" s="21">
+        <f>IFERROR($G36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="30">
-        <f>SUM(B4:B33)</f>
-        <v/>
-      </c>
-      <c r="C34" s="30">
-        <f>SUM(C4:C33)</f>
-        <v/>
-      </c>
-      <c r="D34" s="30">
-        <f>SUM(D4:D33)</f>
-        <v/>
-      </c>
-      <c r="E34" s="31">
-        <f>IFERROR(C34/B34,"")</f>
-        <v/>
-      </c>
-      <c r="F34" s="32">
-        <f>SUM(F4:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="32">
-        <f>SUM(G4:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="32">
-        <f>IFERROR(G34/B34,"")</f>
+      <c r="B37" s="30">
+        <f>SUM(B4:B36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="30">
+        <f>SUM(C4:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="30">
+        <f>SUM(D4:D36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="31">
+        <f>IFERROR(C37/B37,"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="32">
+        <f>SUM(F4:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="32">
+        <f>SUM(G4:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="32">
+        <f>IFERROR(G37/B37,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-02 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.09</v>
+        <v>828.11</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.3099999999999</v>
+        <v>831.38</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.69</v>
+        <v>505.68</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1180.03</v>
+        <v>1180.15</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.08</v>
+        <v>503.11</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>902.8</v>
+        <v>833.89</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>888.46</v>
+        <v>888.4299999999999</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>899.13</v>
+        <v>831.16</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>870.58</v>
+        <v>830.12</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>966.9299999999999</v>
+        <v>966.97</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>939.3200000000001</v>
+        <v>939.23</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4318,14 +4318,18 @@
       <c r="F60" s="26" t="n">
         <v>181</v>
       </c>
-      <c r="G60" s="24" t="inlineStr"/>
-      <c r="H60" s="25" t="inlineStr"/>
+      <c r="G60" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H60" s="25" t="n">
+        <v>987.1939</v>
+      </c>
       <c r="I60" s="21">
         <f>IF(OR($B60="",$H60=""),"",IF($C60="LONG",($H60-$E60)*$F60,($E60-$H60)*$F60))</f>
         <v/>
       </c>
       <c r="J60" s="4" t="n">
-        <v>221.4</v>
+        <v>406.77</v>
       </c>
       <c r="K60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($J60="",0,$J60))</f>
@@ -4365,14 +4369,18 @@
       <c r="F61" s="26" t="n">
         <v>454</v>
       </c>
-      <c r="G61" s="24" t="inlineStr"/>
-      <c r="H61" s="25" t="inlineStr"/>
+      <c r="G61" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H61" s="25" t="n">
+        <v>781.4043</v>
+      </c>
       <c r="I61" s="21">
         <f>IF(OR($B61="",$H61=""),"",IF($C61="LONG",($H61-$E61)*$F61,($E61-$H61)*$F61))</f>
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>490.88</v>
+        <v>954.59</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4412,14 +4420,18 @@
       <c r="F62" s="26" t="n">
         <v>981</v>
       </c>
-      <c r="G62" s="24" t="inlineStr"/>
-      <c r="H62" s="25" t="inlineStr"/>
+      <c r="G62" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H62" s="25" t="n">
+        <v>340.3868</v>
+      </c>
       <c r="I62" s="21">
         <f>IF(OR($B62="",$H62=""),"",IF($C62="LONG",($H62-$E62)*$F62,($E62-$H62)*$F62))</f>
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>494.82</v>
+        <v>944.74</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4486,19 +4498,39 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="23" t="n"/>
-      <c r="B64" s="23" t="n"/>
-      <c r="C64" s="23" t="n"/>
-      <c r="D64" s="24" t="n"/>
-      <c r="E64" s="25" t="n"/>
-      <c r="F64" s="26" t="n"/>
-      <c r="G64" s="24" t="n"/>
-      <c r="H64" s="25" t="n"/>
+      <c r="A64" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231260902149109</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>HERITGFOOD</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D64" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E64" s="25" t="n">
+        <v>378</v>
+      </c>
+      <c r="F64" s="26" t="n">
+        <v>529</v>
+      </c>
+      <c r="G64" s="24" t="inlineStr"/>
+      <c r="H64" s="25" t="inlineStr"/>
       <c r="I64" s="21">
         <f>IF(OR($B64="",$H64=""),"",IF($C64="LONG",($H64-$E64)*$F64,($E64-$H64)*$F64))</f>
         <v/>
       </c>
-      <c r="J64" s="4" t="n"/>
+      <c r="J64" s="4" t="n">
+        <v>311.19</v>
+      </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
         <v/>
@@ -4513,19 +4545,39 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="23" t="n"/>
-      <c r="B65" s="23" t="n"/>
-      <c r="C65" s="23" t="n"/>
-      <c r="D65" s="24" t="n"/>
-      <c r="E65" s="25" t="n"/>
-      <c r="F65" s="26" t="n"/>
-      <c r="G65" s="24" t="n"/>
-      <c r="H65" s="25" t="n"/>
+      <c r="A65" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260902743009</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E65" s="25" t="n">
+        <v>274.0386</v>
+      </c>
+      <c r="F65" s="26" t="n">
+        <v>731</v>
+      </c>
+      <c r="G65" s="24" t="inlineStr"/>
+      <c r="H65" s="25" t="inlineStr"/>
       <c r="I65" s="21">
         <f>IF(OR($B65="",$H65=""),"",IF($C65="LONG",($H65-$E65)*$F65,($E65-$H65)*$F65))</f>
         <v/>
       </c>
-      <c r="J65" s="4" t="n"/>
+      <c r="J65" s="4" t="n">
+        <v>311.61</v>
+      </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
         <v/>
@@ -4540,19 +4592,43 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="23" t="n"/>
-      <c r="B66" s="23" t="n"/>
-      <c r="C66" s="23" t="n"/>
-      <c r="D66" s="24" t="n"/>
-      <c r="E66" s="25" t="n"/>
-      <c r="F66" s="26" t="n"/>
-      <c r="G66" s="24" t="n"/>
-      <c r="H66" s="25" t="n"/>
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260902120009</t>
+        </is>
+      </c>
+      <c r="B66" s="23" t="inlineStr">
+        <is>
+          <t>SAKAR</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E66" s="25" t="n">
+        <v>987.1041</v>
+      </c>
+      <c r="F66" s="26" t="n">
+        <v>181</v>
+      </c>
+      <c r="G66" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H66" s="25" t="n">
+        <v>984.9721</v>
+      </c>
       <c r="I66" s="21">
         <f>IF(OR($B66="",$H66=""),"",IF($C66="LONG",($H66-$E66)*$F66,($E66-$H66)*$F66))</f>
         <v/>
       </c>
-      <c r="J66" s="4" t="n"/>
+      <c r="J66" s="4" t="n">
+        <v>110.57</v>
+      </c>
       <c r="K66" s="21">
         <f>IF(OR($B66="",$I66=""),"",$I66-IF($J66="",0,$J66))</f>
         <v/>
@@ -4567,19 +4643,43 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="23" t="n"/>
-      <c r="B67" s="23" t="n"/>
-      <c r="C67" s="23" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="E67" s="25" t="n"/>
-      <c r="F67" s="26" t="n"/>
-      <c r="G67" s="24" t="n"/>
-      <c r="H67" s="25" t="n"/>
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090223909</t>
+        </is>
+      </c>
+      <c r="B67" s="23" t="inlineStr">
+        <is>
+          <t>SOTL</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E67" s="25" t="n">
+        <v>781.15</v>
+      </c>
+      <c r="F67" s="26" t="n">
+        <v>454</v>
+      </c>
+      <c r="G67" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H67" s="25" t="n">
+        <v>759.8953</v>
+      </c>
       <c r="I67" s="21">
         <f>IF(OR($B67="",$H67=""),"",IF($C67="LONG",($H67-$E67)*$F67,($E67-$H67)*$F67))</f>
         <v/>
       </c>
-      <c r="J67" s="4" t="n"/>
+      <c r="J67" s="4" t="n">
+        <v>172.38</v>
+      </c>
       <c r="K67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($J67="",0,$J67))</f>
         <v/>
@@ -4594,19 +4694,43 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="23" t="n"/>
-      <c r="B68" s="23" t="n"/>
-      <c r="C68" s="23" t="n"/>
-      <c r="D68" s="24" t="n"/>
-      <c r="E68" s="25" t="n"/>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="24" t="n"/>
-      <c r="H68" s="25" t="n"/>
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-231260902110309</t>
+        </is>
+      </c>
+      <c r="B68" s="23" t="inlineStr">
+        <is>
+          <t>SSWL</t>
+        </is>
+      </c>
+      <c r="C68" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D68" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E68" s="25" t="n">
+        <v>340.3105</v>
+      </c>
+      <c r="F68" s="26" t="n">
+        <v>981</v>
+      </c>
+      <c r="G68" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H68" s="25" t="n">
+        <v>345.273</v>
+      </c>
       <c r="I68" s="21">
         <f>IF(OR($B68="",$H68=""),"",IF($C68="LONG",($H68-$E68)*$F68,($E68-$H68)*$F68))</f>
         <v/>
       </c>
-      <c r="J68" s="4" t="n"/>
+      <c r="J68" s="4" t="n">
+        <v>165.98</v>
+      </c>
       <c r="K68" s="21">
         <f>IF(OR($B68="",$I68=""),"",$I68-IF($J68="",0,$J68))</f>
         <v/>
@@ -4621,19 +4745,39 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="23" t="n"/>
-      <c r="B69" s="23" t="n"/>
-      <c r="C69" s="23" t="n"/>
-      <c r="D69" s="24" t="n"/>
-      <c r="E69" s="25" t="n"/>
-      <c r="F69" s="26" t="n"/>
-      <c r="G69" s="24" t="n"/>
-      <c r="H69" s="25" t="n"/>
+      <c r="A69" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260902743109</t>
+        </is>
+      </c>
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E69" s="25" t="n">
+        <v>1101.477</v>
+      </c>
+      <c r="F69" s="26" t="n">
+        <v>181</v>
+      </c>
+      <c r="G69" s="24" t="inlineStr"/>
+      <c r="H69" s="25" t="inlineStr"/>
       <c r="I69" s="21">
         <f>IF(OR($B69="",$H69=""),"",IF($C69="LONG",($H69-$E69)*$F69,($E69-$H69)*$F69))</f>
         <v/>
       </c>
-      <c r="J69" s="4" t="n"/>
+      <c r="J69" s="4" t="n">
+        <v>310.48</v>
+      </c>
       <c r="K69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($J69="",0,$J69))</f>
         <v/>
@@ -4648,19 +4792,39 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="23" t="n"/>
-      <c r="B70" s="23" t="n"/>
-      <c r="C70" s="23" t="n"/>
-      <c r="D70" s="24" t="n"/>
-      <c r="E70" s="25" t="n"/>
-      <c r="F70" s="26" t="n"/>
-      <c r="G70" s="24" t="n"/>
-      <c r="H70" s="25" t="n"/>
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260902743209</t>
+        </is>
+      </c>
+      <c r="B70" s="23" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="C70" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E70" s="25" t="n">
+        <v>1291.5</v>
+      </c>
+      <c r="F70" s="26" t="n">
+        <v>154</v>
+      </c>
+      <c r="G70" s="24" t="inlineStr"/>
+      <c r="H70" s="25" t="inlineStr"/>
       <c r="I70" s="21">
         <f>IF(OR($B70="",$H70=""),"",IF($C70="LONG",($H70-$E70)*$F70,($E70-$H70)*$F70))</f>
         <v/>
       </c>
-      <c r="J70" s="4" t="n"/>
+      <c r="J70" s="4" t="n">
+        <v>309.91</v>
+      </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
         <v/>
@@ -30296,7 +30460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30724,7 +30888,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30767,7 +30931,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30810,7 +30974,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -30853,7 +31017,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -30896,7 +31060,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -30939,7 +31103,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -30982,7 +31146,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31025,7 +31189,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31068,7 +31232,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31111,7 +31275,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31154,7 +31318,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31197,7 +31361,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31240,7 +31404,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31283,7 +31447,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31326,7 +31490,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31369,7 +31533,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31412,7 +31576,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31455,7 +31619,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31498,7 +31662,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -31541,7 +31705,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -31584,7 +31748,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -31627,7 +31791,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -31670,7 +31834,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -31713,7 +31877,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -31756,78 +31920,250 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B36" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E36" s="29">
+        <f>IFERROR($C36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G36" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H36" s="21">
+        <f>IFERROR($G36/$B36,"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B37" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A37)</f>
+        <v/>
+      </c>
+      <c r="C37" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D37" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E37" s="29">
+        <f>IFERROR($C37/$B37,"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G37" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A37,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H37" s="21">
+        <f>IFERROR($G37/$B37,"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A37),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B38" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A38)</f>
+        <v/>
+      </c>
+      <c r="C38" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D38" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E38" s="29">
+        <f>IFERROR($C38/$B38,"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G38" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A38,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H38" s="21">
+        <f>IFERROR($G38/$B38,"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A38),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A38),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B39" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A39)</f>
+        <v/>
+      </c>
+      <c r="C39" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D39" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E39" s="29">
+        <f>IFERROR($C39/$B39,"")</f>
+        <v/>
+      </c>
+      <c r="F39" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G39" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A39,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H39" s="21">
+        <f>IFERROR($G39/$B39,"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A39),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A39),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
           <t>ZAGGLE</t>
         </is>
       </c>
-      <c r="B36" s="20">
-        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A36)</f>
-        <v/>
-      </c>
-      <c r="C36" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D36" s="20">
-        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E36" s="29">
-        <f>IFERROR($C36/$B36,"")</f>
-        <v/>
-      </c>
-      <c r="F36" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$I$4:$I$503)</f>
-        <v/>
-      </c>
-      <c r="G36" s="21">
-        <f>SUMIF('Trade Log'!$B$4:$B$503,$A36,'Trade Log'!$K$4:$K$503)</f>
-        <v/>
-      </c>
-      <c r="H36" s="21">
-        <f>IFERROR($G36/$B36,"")</f>
-        <v/>
-      </c>
-      <c r="I36" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A36),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="B40" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A40)</f>
+        <v/>
+      </c>
+      <c r="C40" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D40" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E40" s="29">
+        <f>IFERROR($C40/$B40,"")</f>
+        <v/>
+      </c>
+      <c r="F40" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G40" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A40,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H40" s="21">
+        <f>IFERROR($G40/$B40,"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A40),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A40),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B37" s="30">
-        <f>SUM(B4:B36)</f>
-        <v/>
-      </c>
-      <c r="C37" s="30">
-        <f>SUM(C4:C36)</f>
-        <v/>
-      </c>
-      <c r="D37" s="30">
-        <f>SUM(D4:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="31">
-        <f>IFERROR(C37/B37,"")</f>
-        <v/>
-      </c>
-      <c r="F37" s="32">
-        <f>SUM(F4:F36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="32">
-        <f>SUM(G4:G36)</f>
-        <v/>
-      </c>
-      <c r="H37" s="32">
-        <f>IFERROR(G37/B37,"")</f>
+      <c r="B41" s="30">
+        <f>SUM(B4:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="30">
+        <f>SUM(C4:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="30">
+        <f>SUM(D4:D40)</f>
+        <v/>
+      </c>
+      <c r="E41" s="31">
+        <f>IFERROR(C41/B41,"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="32">
+        <f>SUM(F4:F40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="32">
+        <f>SUM(G4:G40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="32">
+        <f>IFERROR(G41/B41,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-03 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.38</v>
+        <v>831.45</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>504.96</v>
+        <v>504.98</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1180.15</v>
+        <v>1180.34</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.11</v>
+        <v>503.13</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>480.6</v>
+        <v>493.01</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>888.4299999999999</v>
+        <v>888.46</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>966.97</v>
+        <v>966.91</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>939.23</v>
+        <v>939.29</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>944.74</v>
+        <v>944.76</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4522,14 +4522,18 @@
       <c r="F64" s="26" t="n">
         <v>529</v>
       </c>
-      <c r="G64" s="24" t="inlineStr"/>
-      <c r="H64" s="25" t="inlineStr"/>
+      <c r="G64" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H64" s="25" t="n">
+        <v>372.563</v>
+      </c>
       <c r="I64" s="21">
         <f>IF(OR($B64="",$H64=""),"",IF($C64="LONG",($H64-$E64)*$F64,($E64-$H64)*$F64))</f>
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>311.19</v>
+        <v>585.75</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4569,14 +4573,18 @@
       <c r="F65" s="26" t="n">
         <v>731</v>
       </c>
-      <c r="G65" s="24" t="inlineStr"/>
-      <c r="H65" s="25" t="inlineStr"/>
+      <c r="G65" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H65" s="25" t="n">
+        <v>274.9479</v>
+      </c>
       <c r="I65" s="21">
         <f>IF(OR($B65="",$H65=""),"",IF($C65="LONG",($H65-$E65)*$F65,($E65-$H65)*$F65))</f>
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>311.61</v>
+        <v>584.8200000000001</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4747,12 +4755,12 @@
     <row r="69">
       <c r="A69" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260902743109</t>
+          <t>DHAN-221260902724009</t>
         </is>
       </c>
       <c r="B69" s="23" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="C69" s="23" t="inlineStr">
@@ -4764,19 +4772,23 @@
         <v>46267</v>
       </c>
       <c r="E69" s="25" t="n">
-        <v>1101.477</v>
+        <v>416.35</v>
       </c>
       <c r="F69" s="26" t="n">
-        <v>181</v>
-      </c>
-      <c r="G69" s="24" t="inlineStr"/>
-      <c r="H69" s="25" t="inlineStr"/>
+        <v>242</v>
+      </c>
+      <c r="G69" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H69" s="25" t="n">
+        <v>422.9651</v>
+      </c>
       <c r="I69" s="21">
         <f>IF(OR($B69="",$H69=""),"",IF($C69="LONG",($H69-$E69)*$F69,($E69-$H69)*$F69))</f>
         <v/>
       </c>
       <c r="J69" s="4" t="n">
-        <v>310.48</v>
+        <v>240.58</v>
       </c>
       <c r="K69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($J69="",0,$J69))</f>
@@ -4794,12 +4806,12 @@
     <row r="70">
       <c r="A70" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260902743209</t>
+          <t>DHAN-321260902743109</t>
         </is>
       </c>
       <c r="B70" s="23" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>WINDLAS</t>
         </is>
       </c>
       <c r="C70" s="23" t="inlineStr">
@@ -4811,19 +4823,23 @@
         <v>46267</v>
       </c>
       <c r="E70" s="25" t="n">
-        <v>1291.5</v>
+        <v>1101.477</v>
       </c>
       <c r="F70" s="26" t="n">
-        <v>154</v>
-      </c>
-      <c r="G70" s="24" t="inlineStr"/>
-      <c r="H70" s="25" t="inlineStr"/>
+        <v>181</v>
+      </c>
+      <c r="G70" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H70" s="25" t="n">
+        <v>1138.2559</v>
+      </c>
       <c r="I70" s="21">
         <f>IF(OR($B70="",$H70=""),"",IF($C70="LONG",($H70-$E70)*$F70,($E70-$H70)*$F70))</f>
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>309.91</v>
+        <v>588.72</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4839,19 +4855,43 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="n"/>
-      <c r="B71" s="23" t="n"/>
-      <c r="C71" s="23" t="n"/>
-      <c r="D71" s="24" t="n"/>
-      <c r="E71" s="25" t="n"/>
-      <c r="F71" s="26" t="n"/>
-      <c r="G71" s="24" t="n"/>
-      <c r="H71" s="25" t="n"/>
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260902743209</t>
+        </is>
+      </c>
+      <c r="B71" s="23" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="C71" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E71" s="25" t="n">
+        <v>1291.5</v>
+      </c>
+      <c r="F71" s="26" t="n">
+        <v>154</v>
+      </c>
+      <c r="G71" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H71" s="25" t="n">
+        <v>1300.3182</v>
+      </c>
       <c r="I71" s="21">
         <f>IF(OR($B71="",$H71=""),"",IF($C71="LONG",($H71-$E71)*$F71,($E71-$H71)*$F71))</f>
         <v/>
       </c>
-      <c r="J71" s="4" t="n"/>
+      <c r="J71" s="4" t="n">
+        <v>582.0700000000001</v>
+      </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
         <v/>
@@ -4866,19 +4906,39 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="n"/>
-      <c r="B72" s="23" t="n"/>
-      <c r="C72" s="23" t="n"/>
-      <c r="D72" s="24" t="n"/>
-      <c r="E72" s="25" t="n"/>
-      <c r="F72" s="26" t="n"/>
-      <c r="G72" s="24" t="n"/>
-      <c r="H72" s="25" t="n"/>
+      <c r="A72" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090364809</t>
+        </is>
+      </c>
+      <c r="B72" s="23" t="inlineStr">
+        <is>
+          <t>ALEMBICLTD</t>
+        </is>
+      </c>
+      <c r="C72" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E72" s="25" t="n">
+        <v>109.8863</v>
+      </c>
+      <c r="F72" s="26" t="n">
+        <v>1597</v>
+      </c>
+      <c r="G72" s="24" t="inlineStr"/>
+      <c r="H72" s="25" t="inlineStr"/>
       <c r="I72" s="21">
         <f>IF(OR($B72="",$H72=""),"",IF($C72="LONG",($H72-$E72)*$F72,($E72-$H72)*$F72))</f>
         <v/>
       </c>
-      <c r="J72" s="4" t="n"/>
+      <c r="J72" s="4" t="n">
+        <v>282.13</v>
+      </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
         <v/>
@@ -4893,19 +4953,39 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="23" t="n"/>
-      <c r="B73" s="23" t="n"/>
-      <c r="C73" s="23" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="25" t="n"/>
-      <c r="F73" s="26" t="n"/>
-      <c r="G73" s="24" t="n"/>
-      <c r="H73" s="25" t="n"/>
+      <c r="A73" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260903596709</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>ANTELOPUS</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E73" s="25" t="n">
+        <v>1012.0773</v>
+      </c>
+      <c r="F73" s="26" t="n">
+        <v>86</v>
+      </c>
+      <c r="G73" s="24" t="inlineStr"/>
+      <c r="H73" s="25" t="inlineStr"/>
       <c r="I73" s="21">
         <f>IF(OR($B73="",$H73=""),"",IF($C73="LONG",($H73-$E73)*$F73,($E73-$H73)*$F73))</f>
         <v/>
       </c>
-      <c r="J73" s="4" t="n"/>
+      <c r="J73" s="4" t="n">
+        <v>118.1</v>
+      </c>
       <c r="K73" s="21">
         <f>IF(OR($B73="",$I73=""),"",$I73-IF($J73="",0,$J73))</f>
         <v/>
@@ -4920,19 +5000,39 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="23" t="n"/>
-      <c r="B74" s="23" t="n"/>
-      <c r="C74" s="23" t="n"/>
-      <c r="D74" s="24" t="n"/>
-      <c r="E74" s="25" t="n"/>
-      <c r="F74" s="26" t="n"/>
-      <c r="G74" s="24" t="n"/>
-      <c r="H74" s="25" t="n"/>
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090364909</t>
+        </is>
+      </c>
+      <c r="B74" s="23" t="inlineStr">
+        <is>
+          <t>BFUTILITIE</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E74" s="25" t="n">
+        <v>544.1489</v>
+      </c>
+      <c r="F74" s="26" t="n">
+        <v>321</v>
+      </c>
+      <c r="G74" s="24" t="inlineStr"/>
+      <c r="H74" s="25" t="inlineStr"/>
       <c r="I74" s="21">
         <f>IF(OR($B74="",$H74=""),"",IF($C74="LONG",($H74-$E74)*$F74,($E74-$H74)*$F74))</f>
         <v/>
       </c>
-      <c r="J74" s="4" t="n"/>
+      <c r="J74" s="4" t="n">
+        <v>281.16</v>
+      </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
         <v/>
@@ -4947,19 +5047,39 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="23" t="n"/>
-      <c r="B75" s="23" t="n"/>
-      <c r="C75" s="23" t="n"/>
-      <c r="D75" s="24" t="n"/>
-      <c r="E75" s="25" t="n"/>
-      <c r="F75" s="26" t="n"/>
-      <c r="G75" s="24" t="n"/>
-      <c r="H75" s="25" t="n"/>
+      <c r="A75" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260903780209</t>
+        </is>
+      </c>
+      <c r="B75" s="23" t="inlineStr">
+        <is>
+          <t>GOCLCORP</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E75" s="25" t="n">
+        <v>421.586</v>
+      </c>
+      <c r="F75" s="26" t="n">
+        <v>414</v>
+      </c>
+      <c r="G75" s="24" t="inlineStr"/>
+      <c r="H75" s="25" t="inlineStr"/>
       <c r="I75" s="21">
         <f>IF(OR($B75="",$H75=""),"",IF($C75="LONG",($H75-$E75)*$F75,($E75-$H75)*$F75))</f>
         <v/>
       </c>
-      <c r="J75" s="4" t="n"/>
+      <c r="J75" s="4" t="n">
+        <v>281</v>
+      </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
         <v/>
@@ -4974,19 +5094,43 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="23" t="n"/>
-      <c r="B76" s="23" t="n"/>
-      <c r="C76" s="23" t="n"/>
-      <c r="D76" s="24" t="n"/>
-      <c r="E76" s="25" t="n"/>
-      <c r="F76" s="26" t="n"/>
-      <c r="G76" s="24" t="n"/>
-      <c r="H76" s="25" t="n"/>
+      <c r="A76" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090343709</t>
+        </is>
+      </c>
+      <c r="B76" s="23" t="inlineStr">
+        <is>
+          <t>HERITGFOOD</t>
+        </is>
+      </c>
+      <c r="C76" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E76" s="25" t="n">
+        <v>372.1501</v>
+      </c>
+      <c r="F76" s="26" t="n">
+        <v>529</v>
+      </c>
+      <c r="G76" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H76" s="25" t="n">
+        <v>372.0471</v>
+      </c>
       <c r="I76" s="21">
         <f>IF(OR($B76="",$H76=""),"",IF($C76="LONG",($H76-$E76)*$F76,($E76-$H76)*$F76))</f>
         <v/>
       </c>
-      <c r="J76" s="4" t="n"/>
+      <c r="J76" s="4" t="n">
+        <v>117.05</v>
+      </c>
       <c r="K76" s="21">
         <f>IF(OR($B76="",$I76=""),"",$I76-IF($J76="",0,$J76))</f>
         <v/>
@@ -5001,19 +5145,39 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="23" t="n"/>
-      <c r="B77" s="23" t="n"/>
-      <c r="C77" s="23" t="n"/>
-      <c r="D77" s="24" t="n"/>
-      <c r="E77" s="25" t="n"/>
-      <c r="F77" s="26" t="n"/>
-      <c r="G77" s="24" t="n"/>
-      <c r="H77" s="25" t="n"/>
+      <c r="A77" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090365609</t>
+        </is>
+      </c>
+      <c r="B77" s="23" t="inlineStr">
+        <is>
+          <t>HINDOILEXP</t>
+        </is>
+      </c>
+      <c r="C77" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E77" s="25" t="n">
+        <v>183.9966</v>
+      </c>
+      <c r="F77" s="26" t="n">
+        <v>951</v>
+      </c>
+      <c r="G77" s="24" t="inlineStr"/>
+      <c r="H77" s="25" t="inlineStr"/>
       <c r="I77" s="21">
         <f>IF(OR($B77="",$H77=""),"",IF($C77="LONG",($H77-$E77)*$F77,($E77-$H77)*$F77))</f>
         <v/>
       </c>
-      <c r="J77" s="4" t="n"/>
+      <c r="J77" s="4" t="n">
+        <v>281.52</v>
+      </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
         <v/>
@@ -5028,19 +5192,43 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="23" t="n"/>
-      <c r="B78" s="23" t="n"/>
-      <c r="C78" s="23" t="n"/>
-      <c r="D78" s="24" t="n"/>
-      <c r="E78" s="25" t="n"/>
-      <c r="F78" s="26" t="n"/>
-      <c r="G78" s="24" t="n"/>
-      <c r="H78" s="25" t="n"/>
+      <c r="A78" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126090392509</t>
+        </is>
+      </c>
+      <c r="B78" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C78" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E78" s="25" t="n">
+        <v>274.0624</v>
+      </c>
+      <c r="F78" s="26" t="n">
+        <v>731</v>
+      </c>
+      <c r="G78" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H78" s="25" t="n">
+        <v>278.0089</v>
+      </c>
       <c r="I78" s="21">
         <f>IF(OR($B78="",$H78=""),"",IF($C78="LONG",($H78-$E78)*$F78,($E78-$H78)*$F78))</f>
         <v/>
       </c>
-      <c r="J78" s="4" t="n"/>
+      <c r="J78" s="4" t="n">
+        <v>118.48</v>
+      </c>
       <c r="K78" s="21">
         <f>IF(OR($B78="",$I78=""),"",$I78-IF($J78="",0,$J78))</f>
         <v/>
@@ -5055,19 +5243,39 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="23" t="n"/>
-      <c r="B79" s="23" t="n"/>
-      <c r="C79" s="23" t="n"/>
-      <c r="D79" s="24" t="n"/>
-      <c r="E79" s="25" t="n"/>
-      <c r="F79" s="26" t="n"/>
-      <c r="G79" s="24" t="n"/>
-      <c r="H79" s="25" t="n"/>
+      <c r="A79" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090365509</t>
+        </is>
+      </c>
+      <c r="B79" s="23" t="inlineStr">
+        <is>
+          <t>KIRIINDUS</t>
+        </is>
+      </c>
+      <c r="C79" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D79" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E79" s="25" t="n">
+        <v>579.35</v>
+      </c>
+      <c r="F79" s="26" t="n">
+        <v>302</v>
+      </c>
+      <c r="G79" s="24" t="inlineStr"/>
+      <c r="H79" s="25" t="inlineStr"/>
       <c r="I79" s="21">
         <f>IF(OR($B79="",$H79=""),"",IF($C79="LONG",($H79-$E79)*$F79,($E79-$H79)*$F79))</f>
         <v/>
       </c>
-      <c r="J79" s="4" t="n"/>
+      <c r="J79" s="4" t="n">
+        <v>281.5</v>
+      </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
         <v/>
@@ -5082,19 +5290,39 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="23" t="n"/>
-      <c r="B80" s="23" t="n"/>
-      <c r="C80" s="23" t="n"/>
-      <c r="D80" s="24" t="n"/>
-      <c r="E80" s="25" t="n"/>
-      <c r="F80" s="26" t="n"/>
-      <c r="G80" s="24" t="n"/>
-      <c r="H80" s="25" t="n"/>
+      <c r="A80" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090365009</t>
+        </is>
+      </c>
+      <c r="B80" s="23" t="inlineStr">
+        <is>
+          <t>RAYMOND</t>
+        </is>
+      </c>
+      <c r="C80" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E80" s="25" t="n">
+        <v>763</v>
+      </c>
+      <c r="F80" s="26" t="n">
+        <v>231</v>
+      </c>
+      <c r="G80" s="24" t="inlineStr"/>
+      <c r="H80" s="25" t="inlineStr"/>
       <c r="I80" s="21">
         <f>IF(OR($B80="",$H80=""),"",IF($C80="LONG",($H80-$E80)*$F80,($E80-$H80)*$F80))</f>
         <v/>
       </c>
-      <c r="J80" s="4" t="n"/>
+      <c r="J80" s="4" t="n">
+        <v>283.03</v>
+      </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
         <v/>
@@ -5109,19 +5337,43 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="23" t="n"/>
-      <c r="B81" s="23" t="n"/>
-      <c r="C81" s="23" t="n"/>
-      <c r="D81" s="24" t="n"/>
-      <c r="E81" s="25" t="n"/>
-      <c r="F81" s="26" t="n"/>
-      <c r="G81" s="24" t="n"/>
-      <c r="H81" s="25" t="n"/>
+      <c r="A81" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126090398709</t>
+        </is>
+      </c>
+      <c r="B81" s="23" t="inlineStr">
+        <is>
+          <t>TBZ</t>
+        </is>
+      </c>
+      <c r="C81" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E81" s="25" t="n">
+        <v>423.45</v>
+      </c>
+      <c r="F81" s="26" t="n">
+        <v>242</v>
+      </c>
+      <c r="G81" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H81" s="25" t="n">
+        <v>423.6072</v>
+      </c>
       <c r="I81" s="21">
         <f>IF(OR($B81="",$H81=""),"",IF($C81="LONG",($H81-$E81)*$F81,($E81-$H81)*$F81))</f>
         <v/>
       </c>
-      <c r="J81" s="4" t="n"/>
+      <c r="J81" s="4" t="n">
+        <v>83.56</v>
+      </c>
       <c r="K81" s="21">
         <f>IF(OR($B81="",$I81=""),"",$I81-IF($J81="",0,$J81))</f>
         <v/>
@@ -5136,19 +5388,43 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="23" t="n"/>
-      <c r="B82" s="23" t="n"/>
-      <c r="C82" s="23" t="n"/>
-      <c r="D82" s="24" t="n"/>
-      <c r="E82" s="25" t="n"/>
-      <c r="F82" s="26" t="n"/>
-      <c r="G82" s="24" t="n"/>
-      <c r="H82" s="25" t="n"/>
+      <c r="A82" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260903384009</t>
+        </is>
+      </c>
+      <c r="B82" s="23" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="C82" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E82" s="25" t="n">
+        <v>1139.3014</v>
+      </c>
+      <c r="F82" s="26" t="n">
+        <v>181</v>
+      </c>
+      <c r="G82" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H82" s="25" t="n">
+        <v>1127.3989</v>
+      </c>
       <c r="I82" s="21">
         <f>IF(OR($B82="",$H82=""),"",IF($C82="LONG",($H82-$E82)*$F82,($E82-$H82)*$F82))</f>
         <v/>
       </c>
-      <c r="J82" s="4" t="n"/>
+      <c r="J82" s="4" t="n">
+        <v>120.22</v>
+      </c>
       <c r="K82" s="21">
         <f>IF(OR($B82="",$I82=""),"",$I82-IF($J82="",0,$J82))</f>
         <v/>
@@ -5163,19 +5439,43 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="23" t="n"/>
-      <c r="B83" s="23" t="n"/>
-      <c r="C83" s="23" t="n"/>
-      <c r="D83" s="24" t="n"/>
-      <c r="E83" s="25" t="n"/>
-      <c r="F83" s="26" t="n"/>
-      <c r="G83" s="24" t="n"/>
-      <c r="H83" s="25" t="n"/>
+      <c r="A83" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090316409</t>
+        </is>
+      </c>
+      <c r="B83" s="23" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="C83" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E83" s="25" t="n">
+        <v>1302.759</v>
+      </c>
+      <c r="F83" s="26" t="n">
+        <v>154</v>
+      </c>
+      <c r="G83" s="24" t="n">
+        <v>46268</v>
+      </c>
+      <c r="H83" s="25" t="n">
+        <v>1290.8416</v>
+      </c>
       <c r="I83" s="21">
         <f>IF(OR($B83="",$H83=""),"",IF($C83="LONG",($H83-$E83)*$F83,($E83-$H83)*$F83))</f>
         <v/>
       </c>
-      <c r="J83" s="4" t="n"/>
+      <c r="J83" s="4" t="n">
+        <v>118.26</v>
+      </c>
       <c r="K83" s="21">
         <f>IF(OR($B83="",$I83=""),"",$I83-IF($J83="",0,$J83))</f>
         <v/>
@@ -30460,7 +30760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30544,7 +30844,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>ASHOKA</t>
+          <t>ALEMBICLTD</t>
         </is>
       </c>
       <c r="B4" s="20">
@@ -30587,7 +30887,7 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>ANTELOPUS</t>
         </is>
       </c>
       <c r="B5" s="20">
@@ -30630,7 +30930,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -30673,7 +30973,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -30716,7 +31016,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -30759,7 +31059,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -30802,7 +31102,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -30845,7 +31145,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -30888,7 +31188,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -30931,7 +31231,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -30974,7 +31274,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31017,7 +31317,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31060,7 +31360,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31103,7 +31403,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31146,7 +31446,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31189,7 +31489,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31232,7 +31532,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31275,7 +31575,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31318,7 +31618,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31361,7 +31661,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -31404,7 +31704,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31447,7 +31747,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31490,7 +31790,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31533,7 +31833,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31576,7 +31876,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31619,7 +31919,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31662,7 +31962,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -31705,7 +32005,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -31748,7 +32048,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -31791,7 +32091,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -31834,7 +32134,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -31877,7 +32177,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -31920,7 +32220,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -31963,7 +32263,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32006,7 +32306,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32049,7 +32349,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32092,7 +32392,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32133,37 +32433,338 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>THOMASCOOK</t>
+        </is>
+      </c>
+      <c r="B41" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A41)</f>
+        <v/>
+      </c>
+      <c r="C41" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D41" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E41" s="29">
+        <f>IFERROR($C41/$B41,"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G41" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A41,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H41" s="21">
+        <f>IFERROR($G41/$B41,"")</f>
+        <v/>
+      </c>
+      <c r="I41" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A41),"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A41),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>VENKEYS</t>
+        </is>
+      </c>
+      <c r="B42" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A42)</f>
+        <v/>
+      </c>
+      <c r="C42" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D42" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E42" s="29">
+        <f>IFERROR($C42/$B42,"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G42" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A42,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H42" s="21">
+        <f>IFERROR($G42/$B42,"")</f>
+        <v/>
+      </c>
+      <c r="I42" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A42),"")</f>
+        <v/>
+      </c>
+      <c r="J42" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A42),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B43" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A43)</f>
+        <v/>
+      </c>
+      <c r="C43" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D43" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E43" s="29">
+        <f>IFERROR($C43/$B43,"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G43" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A43,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H43" s="21">
+        <f>IFERROR($G43/$B43,"")</f>
+        <v/>
+      </c>
+      <c r="I43" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A43),"")</f>
+        <v/>
+      </c>
+      <c r="J43" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A43),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B44" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A44)</f>
+        <v/>
+      </c>
+      <c r="C44" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D44" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E44" s="29">
+        <f>IFERROR($C44/$B44,"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G44" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A44,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H44" s="21">
+        <f>IFERROR($G44/$B44,"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A44),"")</f>
+        <v/>
+      </c>
+      <c r="J44" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A44),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B45" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A45)</f>
+        <v/>
+      </c>
+      <c r="C45" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D45" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E45" s="29">
+        <f>IFERROR($C45/$B45,"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G45" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A45,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>IFERROR($G45/$B45,"")</f>
+        <v/>
+      </c>
+      <c r="I45" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A45),"")</f>
+        <v/>
+      </c>
+      <c r="J45" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A45),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B46" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A46)</f>
+        <v/>
+      </c>
+      <c r="C46" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D46" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E46" s="29">
+        <f>IFERROR($C46/$B46,"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G46" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A46,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H46" s="21">
+        <f>IFERROR($G46/$B46,"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A46),"")</f>
+        <v/>
+      </c>
+      <c r="J46" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A46),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B47" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A47)</f>
+        <v/>
+      </c>
+      <c r="C47" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D47" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E47" s="29">
+        <f>IFERROR($C47/$B47,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G47" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A47,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H47" s="21">
+        <f>IFERROR($G47/$B47,"")</f>
+        <v/>
+      </c>
+      <c r="I47" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A47),"")</f>
+        <v/>
+      </c>
+      <c r="J47" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A47),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B41" s="30">
-        <f>SUM(B4:B40)</f>
-        <v/>
-      </c>
-      <c r="C41" s="30">
-        <f>SUM(C4:C40)</f>
-        <v/>
-      </c>
-      <c r="D41" s="30">
-        <f>SUM(D4:D40)</f>
-        <v/>
-      </c>
-      <c r="E41" s="31">
-        <f>IFERROR(C41/B41,"")</f>
-        <v/>
-      </c>
-      <c r="F41" s="32">
-        <f>SUM(F4:F40)</f>
-        <v/>
-      </c>
-      <c r="G41" s="32">
-        <f>SUM(G4:G40)</f>
-        <v/>
-      </c>
-      <c r="H41" s="32">
-        <f>IFERROR(G41/B41,"")</f>
+      <c r="B48" s="30">
+        <f>SUM(B4:B47)</f>
+        <v/>
+      </c>
+      <c r="C48" s="30">
+        <f>SUM(C4:C47)</f>
+        <v/>
+      </c>
+      <c r="D48" s="30">
+        <f>SUM(D4:D47)</f>
+        <v/>
+      </c>
+      <c r="E48" s="31">
+        <f>IFERROR(C48/B48,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="32">
+        <f>SUM(F4:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="32">
+        <f>SUM(G4:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="32">
+        <f>IFERROR(G48/B48,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-04 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.11</v>
+        <v>828.14</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.45</v>
+        <v>831.53</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>504.98</v>
+        <v>504.67</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.68</v>
+        <v>505.7</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1180.34</v>
+        <v>1180.53</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.13</v>
+        <v>503.16</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>493.01</v>
+        <v>493.04</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>888.46</v>
+        <v>888.54</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>966.91</v>
+        <v>966.97</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>939.29</v>
+        <v>939.3200000000001</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>944.76</v>
+        <v>944.73</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4930,14 +4930,18 @@
       <c r="F72" s="26" t="n">
         <v>1597</v>
       </c>
-      <c r="G72" s="24" t="inlineStr"/>
-      <c r="H72" s="25" t="inlineStr"/>
+      <c r="G72" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H72" s="25" t="n">
+        <v>114.1086</v>
+      </c>
       <c r="I72" s="21">
         <f>IF(OR($B72="",$H72=""),"",IF($C72="LONG",($H72-$E72)*$F72,($E72-$H72)*$F72))</f>
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>282.13</v>
+        <v>530.78</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -4977,14 +4981,18 @@
       <c r="F73" s="26" t="n">
         <v>86</v>
       </c>
-      <c r="G73" s="24" t="inlineStr"/>
-      <c r="H73" s="25" t="inlineStr"/>
+      <c r="G73" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H73" s="25" t="n">
+        <v>1004.061</v>
+      </c>
       <c r="I73" s="21">
         <f>IF(OR($B73="",$H73=""),"",IF($C73="LONG",($H73-$E73)*$F73,($E73-$H73)*$F73))</f>
         <v/>
       </c>
       <c r="J73" s="4" t="n">
-        <v>118.1</v>
+        <v>207.68</v>
       </c>
       <c r="K73" s="21">
         <f>IF(OR($B73="",$I73=""),"",$I73-IF($J73="",0,$J73))</f>
@@ -5024,14 +5032,18 @@
       <c r="F74" s="26" t="n">
         <v>321</v>
       </c>
-      <c r="G74" s="24" t="inlineStr"/>
-      <c r="H74" s="25" t="inlineStr"/>
+      <c r="G74" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H74" s="25" t="n">
+        <v>559.1366</v>
+      </c>
       <c r="I74" s="21">
         <f>IF(OR($B74="",$H74=""),"",IF($C74="LONG",($H74-$E74)*$F74,($E74-$H74)*$F74))</f>
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>281.16</v>
+        <v>520.8200000000001</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5071,14 +5083,18 @@
       <c r="F75" s="26" t="n">
         <v>414</v>
       </c>
-      <c r="G75" s="24" t="inlineStr"/>
-      <c r="H75" s="25" t="inlineStr"/>
+      <c r="G75" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H75" s="25" t="n">
+        <v>424.026</v>
+      </c>
       <c r="I75" s="21">
         <f>IF(OR($B75="",$H75=""),"",IF($C75="LONG",($H75-$E75)*$F75,($E75-$H75)*$F75))</f>
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>281</v>
+        <v>522.52</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5169,14 +5185,18 @@
       <c r="F77" s="26" t="n">
         <v>951</v>
       </c>
-      <c r="G77" s="24" t="inlineStr"/>
-      <c r="H77" s="25" t="inlineStr"/>
+      <c r="G77" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H77" s="25" t="n">
+        <v>181.9446</v>
+      </c>
       <c r="I77" s="21">
         <f>IF(OR($B77="",$H77=""),"",IF($C77="LONG",($H77-$E77)*$F77,($E77-$H77)*$F77))</f>
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>281.52</v>
+        <v>522.75</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5267,14 +5287,18 @@
       <c r="F79" s="26" t="n">
         <v>302</v>
       </c>
-      <c r="G79" s="24" t="inlineStr"/>
-      <c r="H79" s="25" t="inlineStr"/>
+      <c r="G79" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H79" s="25" t="n">
+        <v>591.2967</v>
+      </c>
       <c r="I79" s="21">
         <f>IF(OR($B79="",$H79=""),"",IF($C79="LONG",($H79-$E79)*$F79,($E79-$H79)*$F79))</f>
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>281.5</v>
+        <v>527.76</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5314,14 +5338,18 @@
       <c r="F80" s="26" t="n">
         <v>231</v>
       </c>
-      <c r="G80" s="24" t="inlineStr"/>
-      <c r="H80" s="25" t="inlineStr"/>
+      <c r="G80" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H80" s="25" t="n">
+        <v>751.7106</v>
+      </c>
       <c r="I80" s="21">
         <f>IF(OR($B80="",$H80=""),"",IF($C80="LONG",($H80-$E80)*$F80,($E80-$H80)*$F80))</f>
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>283.03</v>
+        <v>524.63</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5490,19 +5518,43 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="23" t="n"/>
-      <c r="B84" s="23" t="n"/>
-      <c r="C84" s="23" t="n"/>
-      <c r="D84" s="24" t="n"/>
-      <c r="E84" s="25" t="n"/>
-      <c r="F84" s="26" t="n"/>
-      <c r="G84" s="24" t="n"/>
-      <c r="H84" s="25" t="n"/>
+      <c r="A84" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126090489209</t>
+        </is>
+      </c>
+      <c r="B84" s="23" t="inlineStr">
+        <is>
+          <t>ALEMBICLTD</t>
+        </is>
+      </c>
+      <c r="C84" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E84" s="25" t="n">
+        <v>114.098</v>
+      </c>
+      <c r="F84" s="26" t="n">
+        <v>1597</v>
+      </c>
+      <c r="G84" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H84" s="25" t="n">
+        <v>111.8446</v>
+      </c>
       <c r="I84" s="21">
         <f>IF(OR($B84="",$H84=""),"",IF($C84="LONG",($H84-$E84)*$F84,($E84-$H84)*$F84))</f>
         <v/>
       </c>
-      <c r="J84" s="4" t="n"/>
+      <c r="J84" s="4" t="n">
+        <v>111.61</v>
+      </c>
       <c r="K84" s="21">
         <f>IF(OR($B84="",$I84=""),"",$I84-IF($J84="",0,$J84))</f>
         <v/>
@@ -5517,19 +5569,43 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="23" t="n"/>
-      <c r="B85" s="23" t="n"/>
-      <c r="C85" s="23" t="n"/>
-      <c r="D85" s="24" t="n"/>
-      <c r="E85" s="25" t="n"/>
-      <c r="F85" s="26" t="n"/>
-      <c r="G85" s="24" t="n"/>
-      <c r="H85" s="25" t="n"/>
+      <c r="A85" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090463509</t>
+        </is>
+      </c>
+      <c r="B85" s="23" t="inlineStr">
+        <is>
+          <t>ANTELOPUS</t>
+        </is>
+      </c>
+      <c r="C85" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E85" s="25" t="n">
+        <v>1003.9</v>
+      </c>
+      <c r="F85" s="26" t="n">
+        <v>86</v>
+      </c>
+      <c r="G85" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H85" s="25" t="n">
+        <v>987.1866</v>
+      </c>
       <c r="I85" s="21">
         <f>IF(OR($B85="",$H85=""),"",IF($C85="LONG",($H85-$E85)*$F85,($E85-$H85)*$F85))</f>
         <v/>
       </c>
-      <c r="J85" s="4" t="n"/>
+      <c r="J85" s="4" t="n">
+        <v>77.73999999999999</v>
+      </c>
       <c r="K85" s="21">
         <f>IF(OR($B85="",$I85=""),"",$I85-IF($J85="",0,$J85))</f>
         <v/>
@@ -5544,19 +5620,43 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="23" t="n"/>
-      <c r="B86" s="23" t="n"/>
-      <c r="C86" s="23" t="n"/>
-      <c r="D86" s="24" t="n"/>
-      <c r="E86" s="25" t="n"/>
-      <c r="F86" s="26" t="n"/>
-      <c r="G86" s="24" t="n"/>
-      <c r="H86" s="25" t="n"/>
+      <c r="A86" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090416009</t>
+        </is>
+      </c>
+      <c r="B86" s="23" t="inlineStr">
+        <is>
+          <t>BFUTILITIE</t>
+        </is>
+      </c>
+      <c r="C86" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D86" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E86" s="25" t="n">
+        <v>557.8248</v>
+      </c>
+      <c r="F86" s="26" t="n">
+        <v>321</v>
+      </c>
+      <c r="G86" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H86" s="25" t="n">
+        <v>545.7992</v>
+      </c>
       <c r="I86" s="21">
         <f>IF(OR($B86="",$H86=""),"",IF($C86="LONG",($H86-$E86)*$F86,($E86-$H86)*$F86))</f>
         <v/>
       </c>
-      <c r="J86" s="4" t="n"/>
+      <c r="J86" s="4" t="n">
+        <v>110.47</v>
+      </c>
       <c r="K86" s="21">
         <f>IF(OR($B86="",$I86=""),"",$I86-IF($J86="",0,$J86))</f>
         <v/>
@@ -5571,19 +5671,43 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="23" t="n"/>
-      <c r="B87" s="23" t="n"/>
-      <c r="C87" s="23" t="n"/>
-      <c r="D87" s="24" t="n"/>
-      <c r="E87" s="25" t="n"/>
-      <c r="F87" s="26" t="n"/>
-      <c r="G87" s="24" t="n"/>
-      <c r="H87" s="25" t="n"/>
+      <c r="A87" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126090492309</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>GOCLCORP</t>
+        </is>
+      </c>
+      <c r="C87" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D87" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E87" s="25" t="n">
+        <v>423.9067</v>
+      </c>
+      <c r="F87" s="26" t="n">
+        <v>414</v>
+      </c>
+      <c r="G87" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H87" s="25" t="n">
+        <v>429.4497</v>
+      </c>
       <c r="I87" s="21">
         <f>IF(OR($B87="",$H87=""),"",IF($C87="LONG",($H87-$E87)*$F87,($E87-$H87)*$F87))</f>
         <v/>
       </c>
-      <c r="J87" s="4" t="n"/>
+      <c r="J87" s="4" t="n">
+        <v>109.62</v>
+      </c>
       <c r="K87" s="21">
         <f>IF(OR($B87="",$I87=""),"",$I87-IF($J87="",0,$J87))</f>
         <v/>
@@ -5598,19 +5722,43 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="23" t="n"/>
-      <c r="B88" s="23" t="n"/>
-      <c r="C88" s="23" t="n"/>
-      <c r="D88" s="24" t="n"/>
-      <c r="E88" s="25" t="n"/>
-      <c r="F88" s="26" t="n"/>
-      <c r="G88" s="24" t="n"/>
-      <c r="H88" s="25" t="n"/>
+      <c r="A88" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090463609</t>
+        </is>
+      </c>
+      <c r="B88" s="23" t="inlineStr">
+        <is>
+          <t>HINDOILEXP</t>
+        </is>
+      </c>
+      <c r="C88" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D88" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E88" s="25" t="n">
+        <v>181.8259</v>
+      </c>
+      <c r="F88" s="26" t="n">
+        <v>951</v>
+      </c>
+      <c r="G88" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H88" s="25" t="n">
+        <v>182</v>
+      </c>
       <c r="I88" s="21">
         <f>IF(OR($B88="",$H88=""),"",IF($C88="LONG",($H88-$E88)*$F88,($E88-$H88)*$F88))</f>
         <v/>
       </c>
-      <c r="J88" s="4" t="n"/>
+      <c r="J88" s="4" t="n">
+        <v>108.56</v>
+      </c>
       <c r="K88" s="21">
         <f>IF(OR($B88="",$I88=""),"",$I88-IF($J88="",0,$J88))</f>
         <v/>
@@ -5625,19 +5773,43 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="23" t="n"/>
-      <c r="B89" s="23" t="n"/>
-      <c r="C89" s="23" t="n"/>
-      <c r="D89" s="24" t="n"/>
-      <c r="E89" s="25" t="n"/>
-      <c r="F89" s="26" t="n"/>
-      <c r="G89" s="24" t="n"/>
-      <c r="H89" s="25" t="n"/>
+      <c r="A89" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090415409</t>
+        </is>
+      </c>
+      <c r="B89" s="23" t="inlineStr">
+        <is>
+          <t>KIRIINDUS</t>
+        </is>
+      </c>
+      <c r="C89" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E89" s="25" t="n">
+        <v>591.654</v>
+      </c>
+      <c r="F89" s="26" t="n">
+        <v>302</v>
+      </c>
+      <c r="G89" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H89" s="25" t="n">
+        <v>562.05</v>
+      </c>
       <c r="I89" s="21">
         <f>IF(OR($B89="",$H89=""),"",IF($C89="LONG",($H89-$E89)*$F89,($E89-$H89)*$F89))</f>
         <v/>
       </c>
-      <c r="J89" s="4" t="n"/>
+      <c r="J89" s="4" t="n">
+        <v>109.99</v>
+      </c>
       <c r="K89" s="21">
         <f>IF(OR($B89="",$I89=""),"",$I89-IF($J89="",0,$J89))</f>
         <v/>
@@ -5652,19 +5824,39 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="23" t="n"/>
-      <c r="B90" s="23" t="n"/>
-      <c r="C90" s="23" t="n"/>
-      <c r="D90" s="24" t="n"/>
-      <c r="E90" s="25" t="n"/>
-      <c r="F90" s="26" t="n"/>
-      <c r="G90" s="24" t="n"/>
-      <c r="H90" s="25" t="n"/>
+      <c r="A90" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090488609</t>
+        </is>
+      </c>
+      <c r="B90" s="23" t="inlineStr">
+        <is>
+          <t>MAITHANALL</t>
+        </is>
+      </c>
+      <c r="C90" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D90" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E90" s="25" t="n">
+        <v>1086.426</v>
+      </c>
+      <c r="F90" s="26" t="n">
+        <v>321</v>
+      </c>
+      <c r="G90" s="24" t="inlineStr"/>
+      <c r="H90" s="25" t="inlineStr"/>
       <c r="I90" s="21">
         <f>IF(OR($B90="",$H90=""),"",IF($C90="LONG",($H90-$E90)*$F90,($E90-$H90)*$F90))</f>
         <v/>
       </c>
-      <c r="J90" s="4" t="n"/>
+      <c r="J90" s="4" t="n">
+        <v>487.85</v>
+      </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
         <v/>
@@ -5679,19 +5871,43 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="23" t="n"/>
-      <c r="B91" s="23" t="n"/>
-      <c r="C91" s="23" t="n"/>
-      <c r="D91" s="24" t="n"/>
-      <c r="E91" s="25" t="n"/>
-      <c r="F91" s="26" t="n"/>
-      <c r="G91" s="24" t="n"/>
-      <c r="H91" s="25" t="n"/>
+      <c r="A91" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260904383309</t>
+        </is>
+      </c>
+      <c r="B91" s="23" t="inlineStr">
+        <is>
+          <t>RAYMOND</t>
+        </is>
+      </c>
+      <c r="C91" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D91" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E91" s="25" t="n">
+        <v>752.5812</v>
+      </c>
+      <c r="F91" s="26" t="n">
+        <v>231</v>
+      </c>
+      <c r="G91" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H91" s="25" t="n">
+        <v>740.4414</v>
+      </c>
       <c r="I91" s="21">
         <f>IF(OR($B91="",$H91=""),"",IF($C91="LONG",($H91-$E91)*$F91,($E91-$H91)*$F91))</f>
         <v/>
       </c>
-      <c r="J91" s="4" t="n"/>
+      <c r="J91" s="4" t="n">
+        <v>108.69</v>
+      </c>
       <c r="K91" s="21">
         <f>IF(OR($B91="",$I91=""),"",$I91-IF($J91="",0,$J91))</f>
         <v/>
@@ -5706,19 +5922,39 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="23" t="n"/>
-      <c r="B92" s="23" t="n"/>
-      <c r="C92" s="23" t="n"/>
-      <c r="D92" s="24" t="n"/>
-      <c r="E92" s="25" t="n"/>
-      <c r="F92" s="26" t="n"/>
-      <c r="G92" s="24" t="n"/>
-      <c r="H92" s="25" t="n"/>
+      <c r="A92" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260904639609</t>
+        </is>
+      </c>
+      <c r="B92" s="23" t="inlineStr">
+        <is>
+          <t>RML</t>
+        </is>
+      </c>
+      <c r="C92" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D92" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E92" s="25" t="n">
+        <v>1291.9929</v>
+      </c>
+      <c r="F92" s="26" t="n">
+        <v>270</v>
+      </c>
+      <c r="G92" s="24" t="inlineStr"/>
+      <c r="H92" s="25" t="inlineStr"/>
       <c r="I92" s="21">
         <f>IF(OR($B92="",$H92=""),"",IF($C92="LONG",($H92-$E92)*$F92,($E92-$H92)*$F92))</f>
         <v/>
       </c>
-      <c r="J92" s="4" t="n"/>
+      <c r="J92" s="4" t="n">
+        <v>487.96</v>
+      </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
         <v/>
@@ -5733,19 +5969,39 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="23" t="n"/>
-      <c r="B93" s="23" t="n"/>
-      <c r="C93" s="23" t="n"/>
-      <c r="D93" s="24" t="n"/>
-      <c r="E93" s="25" t="n"/>
-      <c r="F93" s="26" t="n"/>
-      <c r="G93" s="24" t="n"/>
-      <c r="H93" s="25" t="n"/>
+      <c r="A93" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090486609</t>
+        </is>
+      </c>
+      <c r="B93" s="23" t="inlineStr">
+        <is>
+          <t>SINDHUTRAD</t>
+        </is>
+      </c>
+      <c r="C93" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D93" s="24" t="n">
+        <v>46269</v>
+      </c>
+      <c r="E93" s="25" t="n">
+        <v>25.2263</v>
+      </c>
+      <c r="F93" s="26" t="n">
+        <v>13916</v>
+      </c>
+      <c r="G93" s="24" t="inlineStr"/>
+      <c r="H93" s="25" t="inlineStr"/>
       <c r="I93" s="21">
         <f>IF(OR($B93="",$H93=""),"",IF($C93="LONG",($H93-$E93)*$F93,($E93-$H93)*$F93))</f>
         <v/>
       </c>
-      <c r="J93" s="4" t="n"/>
+      <c r="J93" s="4" t="n">
+        <v>490.59</v>
+      </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
         <v/>
@@ -30760,7 +31016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31704,7 +31960,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -31747,7 +32003,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -31790,7 +32046,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -31833,7 +32089,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -31876,7 +32132,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -31919,7 +32175,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -31962,7 +32218,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32005,7 +32261,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32048,7 +32304,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32091,7 +32347,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32134,7 +32390,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32177,7 +32433,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32220,7 +32476,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32263,7 +32519,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32306,7 +32562,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32349,7 +32605,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32392,7 +32648,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32435,7 +32691,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32478,7 +32734,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -32521,7 +32777,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -32564,7 +32820,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -32607,7 +32863,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -32650,7 +32906,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -32693,7 +32949,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -32734,37 +32990,166 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B48" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A48)</f>
+        <v/>
+      </c>
+      <c r="C48" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D48" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E48" s="29">
+        <f>IFERROR($C48/$B48,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G48" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A48,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H48" s="21">
+        <f>IFERROR($G48/$B48,"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A48),"")</f>
+        <v/>
+      </c>
+      <c r="J48" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A48),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B49" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A49)</f>
+        <v/>
+      </c>
+      <c r="C49" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D49" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E49" s="29">
+        <f>IFERROR($C49/$B49,"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G49" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A49,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H49" s="21">
+        <f>IFERROR($G49/$B49,"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A49),"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A49),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B50" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A50)</f>
+        <v/>
+      </c>
+      <c r="C50" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D50" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E50" s="29">
+        <f>IFERROR($C50/$B50,"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G50" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A50,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H50" s="21">
+        <f>IFERROR($G50/$B50,"")</f>
+        <v/>
+      </c>
+      <c r="I50" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A50),"")</f>
+        <v/>
+      </c>
+      <c r="J50" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A50),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B48" s="30">
-        <f>SUM(B4:B47)</f>
-        <v/>
-      </c>
-      <c r="C48" s="30">
-        <f>SUM(C4:C47)</f>
-        <v/>
-      </c>
-      <c r="D48" s="30">
-        <f>SUM(D4:D47)</f>
-        <v/>
-      </c>
-      <c r="E48" s="31">
-        <f>IFERROR(C48/B48,"")</f>
-        <v/>
-      </c>
-      <c r="F48" s="32">
-        <f>SUM(F4:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="32">
-        <f>SUM(G4:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="32">
-        <f>IFERROR(G48/B48,"")</f>
+      <c r="B51" s="30">
+        <f>SUM(B4:B50)</f>
+        <v/>
+      </c>
+      <c r="C51" s="30">
+        <f>SUM(C4:C50)</f>
+        <v/>
+      </c>
+      <c r="D51" s="30">
+        <f>SUM(D4:D50)</f>
+        <v/>
+      </c>
+      <c r="E51" s="31">
+        <f>IFERROR(C51/B51,"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="32">
+        <f>SUM(F4:F50)</f>
+        <v/>
+      </c>
+      <c r="G51" s="32">
+        <f>SUM(G4:G50)</f>
+        <v/>
+      </c>
+      <c r="H51" s="32">
+        <f>IFERROR(G51/B51,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Dhan UC-fetch 429s: persist 9:15am circuit cache, widen quote rate limiter, retry on 429
check_exit_925/force_exit_1159's mirrored-short stop-loss placement kept
losing the UC fetch to a 429, leaving shorts unprotected (MAITHANALL today,
FMGOETZE/SYNCOMF/SOTL/ANTELOPUS on prior days) -- confirmed live that even a
strict 1.0s gap between quote calls isn't enough margin for Dhan's real
server-side window. Since UC is a fixed daily value, place_targets_915's
existing 9:15am batch fetch is now persisted to results/dhan_uc_cache.json
and read back by the later exit stages instead of re-fetched on demand right
when a short opens. Also widened the quote rate limiter to 1.5s and added
retry-with-backoff on any 429 that still slips through.

Manually reconciled MAITHANALL's missing stop-loss placed live today, plus
carrying forward the TBZ position fix and BOMDYEING/GKENERGY/RAMRAT exit
reconciliation from prior sessions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>828.14</v>
+        <v>828.1799999999999</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>831.53</v>
+        <v>831.59</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>504.67</v>
+        <v>504.66</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>505.7</v>
+        <v>505.69</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>1180.53</v>
+        <v>1180.15</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>503.16</v>
+        <v>503.19</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>493.04</v>
+        <v>493.06</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>888.54</v>
+        <v>888.66</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>966.97</v>
+        <v>966.99</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>939.3200000000001</v>
+        <v>939.37</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>944.73</v>
+        <v>944.79</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>585.75</v>
+        <v>585.74</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>522.75</v>
+        <v>522.78</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>527.76</v>
+        <v>527.75</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>524.63</v>
+        <v>524.65</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5848,14 +5848,18 @@
       <c r="F90" s="26" t="n">
         <v>321</v>
       </c>
-      <c r="G90" s="24" t="inlineStr"/>
-      <c r="H90" s="25" t="inlineStr"/>
+      <c r="G90" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H90" s="25" t="n">
+        <v>1185</v>
+      </c>
       <c r="I90" s="21">
         <f>IF(OR($B90="",$H90=""),"",IF($C90="LONG",($H90-$E90)*$F90,($E90-$H90)*$F90))</f>
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>487.85</v>
+        <v>1120.75</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5946,14 +5950,18 @@
       <c r="F92" s="26" t="n">
         <v>270</v>
       </c>
-      <c r="G92" s="24" t="inlineStr"/>
-      <c r="H92" s="25" t="inlineStr"/>
+      <c r="G92" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H92" s="25" t="n">
+        <v>1337.4363</v>
+      </c>
       <c r="I92" s="21">
         <f>IF(OR($B92="",$H92=""),"",IF($C92="LONG",($H92-$E92)*$F92,($E92-$H92)*$F92))</f>
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>487.96</v>
+        <v>1100.92</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6000,7 +6008,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>490.59</v>
+        <v>706.6900000000001</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6016,19 +6024,39 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="23" t="n"/>
-      <c r="B94" s="23" t="n"/>
-      <c r="C94" s="23" t="n"/>
-      <c r="D94" s="24" t="n"/>
-      <c r="E94" s="25" t="n"/>
-      <c r="F94" s="26" t="n"/>
-      <c r="G94" s="24" t="n"/>
-      <c r="H94" s="25" t="n"/>
+      <c r="A94" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090714709</t>
+        </is>
+      </c>
+      <c r="B94" s="23" t="inlineStr">
+        <is>
+          <t>MAITHANALL</t>
+        </is>
+      </c>
+      <c r="C94" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D94" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E94" s="25" t="n">
+        <v>1183.4504</v>
+      </c>
+      <c r="F94" s="26" t="n">
+        <v>321</v>
+      </c>
+      <c r="G94" s="24" t="inlineStr"/>
+      <c r="H94" s="25" t="inlineStr"/>
       <c r="I94" s="21">
         <f>IF(OR($B94="",$H94=""),"",IF($C94="LONG",($H94-$E94)*$F94,($E94-$H94)*$F94))</f>
         <v/>
       </c>
-      <c r="J94" s="4" t="n"/>
+      <c r="J94" s="4" t="n">
+        <v>132.78</v>
+      </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
         <v/>
@@ -6043,19 +6071,39 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="23" t="n"/>
-      <c r="B95" s="23" t="n"/>
-      <c r="C95" s="23" t="n"/>
-      <c r="D95" s="24" t="n"/>
-      <c r="E95" s="25" t="n"/>
-      <c r="F95" s="26" t="n"/>
-      <c r="G95" s="24" t="n"/>
-      <c r="H95" s="25" t="n"/>
+      <c r="A95" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260907112709</t>
+        </is>
+      </c>
+      <c r="B95" s="23" t="inlineStr">
+        <is>
+          <t>RML</t>
+        </is>
+      </c>
+      <c r="C95" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D95" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E95" s="25" t="n">
+        <v>1345.7526</v>
+      </c>
+      <c r="F95" s="26" t="n">
+        <v>270</v>
+      </c>
+      <c r="G95" s="24" t="inlineStr"/>
+      <c r="H95" s="25" t="inlineStr"/>
       <c r="I95" s="21">
         <f>IF(OR($B95="",$H95=""),"",IF($C95="LONG",($H95-$E95)*$F95,($E95-$H95)*$F95))</f>
         <v/>
       </c>
-      <c r="J95" s="4" t="n"/>
+      <c r="J95" s="4" t="n">
+        <v>128.03</v>
+      </c>
       <c r="K95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($J95="",0,$J95))</f>
         <v/>

</xml_diff>

<commit_message>
Data update — 2026-09-07 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -6001,14 +6001,18 @@
       <c r="F93" s="26" t="n">
         <v>13916</v>
       </c>
-      <c r="G93" s="24" t="inlineStr"/>
-      <c r="H93" s="25" t="inlineStr"/>
+      <c r="G93" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H93" s="25" t="n">
+        <v>25.2263</v>
+      </c>
       <c r="I93" s="21">
         <f>IF(OR($B93="",$H93=""),"",IF($C93="LONG",($H93-$E93)*$F93,($E93-$H93)*$F93))</f>
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>706.6900000000001</v>
+        <v>1094.47</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6026,27 +6030,27 @@
     <row r="94">
       <c r="A94" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126090714709</t>
+          <t>DHAN-221260907740209</t>
         </is>
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="C94" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D94" s="24" t="n">
         <v>46272</v>
       </c>
       <c r="E94" s="25" t="n">
-        <v>1183.4504</v>
+        <v>184.7831</v>
       </c>
       <c r="F94" s="26" t="n">
-        <v>321</v>
+        <v>1261</v>
       </c>
       <c r="G94" s="24" t="inlineStr"/>
       <c r="H94" s="25" t="inlineStr"/>
@@ -6055,7 +6059,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>132.78</v>
+        <v>350.43</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6073,27 +6077,27 @@
     <row r="95">
       <c r="A95" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260907112709</t>
+          <t>DHAN-23126090769809</t>
         </is>
       </c>
       <c r="B95" s="23" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="C95" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D95" s="24" t="n">
         <v>46272</v>
       </c>
       <c r="E95" s="25" t="n">
-        <v>1345.7526</v>
+        <v>114.89</v>
       </c>
       <c r="F95" s="26" t="n">
-        <v>270</v>
+        <v>1019</v>
       </c>
       <c r="G95" s="24" t="inlineStr"/>
       <c r="H95" s="25" t="inlineStr"/>
@@ -6102,7 +6106,7 @@
         <v/>
       </c>
       <c r="J95" s="4" t="n">
-        <v>128.03</v>
+        <v>153.76</v>
       </c>
       <c r="K95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($J95="",0,$J95))</f>
@@ -6118,19 +6122,39 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="23" t="n"/>
-      <c r="B96" s="23" t="n"/>
-      <c r="C96" s="23" t="n"/>
-      <c r="D96" s="24" t="n"/>
-      <c r="E96" s="25" t="n"/>
-      <c r="F96" s="26" t="n"/>
-      <c r="G96" s="24" t="n"/>
-      <c r="H96" s="25" t="n"/>
+      <c r="A96" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090769609</t>
+        </is>
+      </c>
+      <c r="B96" s="23" t="inlineStr">
+        <is>
+          <t>HIKAL</t>
+        </is>
+      </c>
+      <c r="C96" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D96" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E96" s="25" t="n">
+        <v>242.9411</v>
+      </c>
+      <c r="F96" s="26" t="n">
+        <v>959</v>
+      </c>
+      <c r="G96" s="24" t="inlineStr"/>
+      <c r="H96" s="25" t="inlineStr"/>
       <c r="I96" s="21">
         <f>IF(OR($B96="",$H96=""),"",IF($C96="LONG",($H96-$E96)*$F96,($E96-$H96)*$F96))</f>
         <v/>
       </c>
-      <c r="J96" s="4" t="n"/>
+      <c r="J96" s="4" t="n">
+        <v>350.39</v>
+      </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
         <v/>
@@ -6145,19 +6169,43 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="23" t="n"/>
-      <c r="B97" s="23" t="n"/>
-      <c r="C97" s="23" t="n"/>
-      <c r="D97" s="24" t="n"/>
-      <c r="E97" s="25" t="n"/>
-      <c r="F97" s="26" t="n"/>
-      <c r="G97" s="24" t="n"/>
-      <c r="H97" s="25" t="n"/>
+      <c r="A97" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090714709</t>
+        </is>
+      </c>
+      <c r="B97" s="23" t="inlineStr">
+        <is>
+          <t>MAITHANALL</t>
+        </is>
+      </c>
+      <c r="C97" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D97" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E97" s="25" t="n">
+        <v>1183.4504</v>
+      </c>
+      <c r="F97" s="26" t="n">
+        <v>321</v>
+      </c>
+      <c r="G97" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H97" s="25" t="n">
+        <v>1129.9305</v>
+      </c>
       <c r="I97" s="21">
         <f>IF(OR($B97="",$H97=""),"",IF($C97="LONG",($H97-$E97)*$F97,($E97-$H97)*$F97))</f>
         <v/>
       </c>
-      <c r="J97" s="4" t="n"/>
+      <c r="J97" s="4" t="n">
+        <v>180.83</v>
+      </c>
       <c r="K97" s="21">
         <f>IF(OR($B97="",$I97=""),"",$I97-IF($J97="",0,$J97))</f>
         <v/>
@@ -6172,19 +6220,39 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="23" t="n"/>
-      <c r="B98" s="23" t="n"/>
-      <c r="C98" s="23" t="n"/>
-      <c r="D98" s="24" t="n"/>
-      <c r="E98" s="25" t="n"/>
-      <c r="F98" s="26" t="n"/>
-      <c r="G98" s="24" t="n"/>
-      <c r="H98" s="25" t="n"/>
+      <c r="A98" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090769709</t>
+        </is>
+      </c>
+      <c r="B98" s="23" t="inlineStr">
+        <is>
+          <t>PITTIENG</t>
+        </is>
+      </c>
+      <c r="C98" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D98" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E98" s="25" t="n">
+        <v>1174.901</v>
+      </c>
+      <c r="F98" s="26" t="n">
+        <v>198</v>
+      </c>
+      <c r="G98" s="24" t="inlineStr"/>
+      <c r="H98" s="25" t="inlineStr"/>
       <c r="I98" s="21">
         <f>IF(OR($B98="",$H98=""),"",IF($C98="LONG",($H98-$E98)*$F98,($E98-$H98)*$F98))</f>
         <v/>
       </c>
-      <c r="J98" s="4" t="n"/>
+      <c r="J98" s="4" t="n">
+        <v>349.98</v>
+      </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
         <v/>
@@ -6199,19 +6267,43 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="23" t="n"/>
-      <c r="B99" s="23" t="n"/>
-      <c r="C99" s="23" t="n"/>
-      <c r="D99" s="24" t="n"/>
-      <c r="E99" s="25" t="n"/>
-      <c r="F99" s="26" t="n"/>
-      <c r="G99" s="24" t="n"/>
-      <c r="H99" s="25" t="n"/>
+      <c r="A99" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260907112709</t>
+        </is>
+      </c>
+      <c r="B99" s="23" t="inlineStr">
+        <is>
+          <t>RML</t>
+        </is>
+      </c>
+      <c r="C99" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D99" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E99" s="25" t="n">
+        <v>1345.7526</v>
+      </c>
+      <c r="F99" s="26" t="n">
+        <v>270</v>
+      </c>
+      <c r="G99" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H99" s="25" t="n">
+        <v>1363.1344</v>
+      </c>
       <c r="I99" s="21">
         <f>IF(OR($B99="",$H99=""),"",IF($C99="LONG",($H99-$E99)*$F99,($E99-$H99)*$F99))</f>
         <v/>
       </c>
-      <c r="J99" s="4" t="n"/>
+      <c r="J99" s="4" t="n">
+        <v>176.44</v>
+      </c>
       <c r="K99" s="21">
         <f>IF(OR($B99="",$I99=""),"",$I99-IF($J99="",0,$J99))</f>
         <v/>
@@ -6226,19 +6318,43 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="23" t="n"/>
-      <c r="B100" s="23" t="n"/>
-      <c r="C100" s="23" t="n"/>
-      <c r="D100" s="24" t="n"/>
-      <c r="E100" s="25" t="n"/>
-      <c r="F100" s="26" t="n"/>
-      <c r="G100" s="24" t="n"/>
-      <c r="H100" s="25" t="n"/>
+      <c r="A100" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090734409</t>
+        </is>
+      </c>
+      <c r="B100" s="23" t="inlineStr">
+        <is>
+          <t>SINDHUTRAD</t>
+        </is>
+      </c>
+      <c r="C100" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D100" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E100" s="25" t="n">
+        <v>24.77</v>
+      </c>
+      <c r="F100" s="26" t="n">
+        <v>13916</v>
+      </c>
+      <c r="G100" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H100" s="25" t="n">
+        <v>25.2993</v>
+      </c>
       <c r="I100" s="21">
         <f>IF(OR($B100="",$H100=""),"",IF($C100="LONG",($H100-$E100)*$F100,($E100-$H100)*$F100))</f>
         <v/>
       </c>
-      <c r="J100" s="4" t="n"/>
+      <c r="J100" s="4" t="n">
+        <v>170</v>
+      </c>
       <c r="K100" s="21">
         <f>IF(OR($B100="",$I100=""),"",$I100-IF($J100="",0,$J100))</f>
         <v/>
@@ -6253,19 +6369,39 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="23" t="n"/>
-      <c r="B101" s="23" t="n"/>
-      <c r="C101" s="23" t="n"/>
-      <c r="D101" s="24" t="n"/>
-      <c r="E101" s="25" t="n"/>
-      <c r="F101" s="26" t="n"/>
-      <c r="G101" s="24" t="n"/>
-      <c r="H101" s="25" t="n"/>
+      <c r="A101" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260907804109</t>
+        </is>
+      </c>
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>TALBROAUTO</t>
+        </is>
+      </c>
+      <c r="C101" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D101" s="24" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E101" s="25" t="n">
+        <v>433.5513</v>
+      </c>
+      <c r="F101" s="26" t="n">
+        <v>538</v>
+      </c>
+      <c r="G101" s="24" t="inlineStr"/>
+      <c r="H101" s="25" t="inlineStr"/>
       <c r="I101" s="21">
         <f>IF(OR($B101="",$H101=""),"",IF($C101="LONG",($H101-$E101)*$F101,($E101-$H101)*$F101))</f>
         <v/>
       </c>
-      <c r="J101" s="4" t="n"/>
+      <c r="J101" s="4" t="n">
+        <v>350.71</v>
+      </c>
       <c r="K101" s="21">
         <f>IF(OR($B101="",$I101=""),"",$I101-IF($J101="",0,$J101))</f>
         <v/>
@@ -31064,7 +31200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31449,7 +31585,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -31492,7 +31628,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -31535,7 +31671,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31578,7 +31714,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -31621,7 +31757,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -31664,7 +31800,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -31707,7 +31843,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -31750,7 +31886,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -31793,7 +31929,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -31836,7 +31972,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -31879,7 +32015,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -31922,7 +32058,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -31965,7 +32101,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32008,7 +32144,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32051,7 +32187,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32094,7 +32230,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32137,7 +32273,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32180,7 +32316,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32223,7 +32359,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32266,7 +32402,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32309,7 +32445,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32352,7 +32488,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32395,7 +32531,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32438,7 +32574,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32481,7 +32617,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32524,7 +32660,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32567,7 +32703,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -32610,7 +32746,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -32653,7 +32789,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -32696,7 +32832,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -32739,7 +32875,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -32782,7 +32918,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -32825,7 +32961,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -32868,7 +33004,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -32911,7 +33047,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -32954,7 +33090,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -32997,7 +33133,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33040,7 +33176,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33083,7 +33219,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33126,7 +33262,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33167,37 +33303,252 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B51" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A51)</f>
+        <v/>
+      </c>
+      <c r="C51" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D51" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E51" s="29">
+        <f>IFERROR($C51/$B51,"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G51" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A51,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H51" s="21">
+        <f>IFERROR($G51/$B51,"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A51),"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A51),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B52" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A52)</f>
+        <v/>
+      </c>
+      <c r="C52" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D52" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E52" s="29">
+        <f>IFERROR($C52/$B52,"")</f>
+        <v/>
+      </c>
+      <c r="F52" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G52" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A52,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H52" s="21">
+        <f>IFERROR($G52/$B52,"")</f>
+        <v/>
+      </c>
+      <c r="I52" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A52),"")</f>
+        <v/>
+      </c>
+      <c r="J52" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A52),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B53" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A53)</f>
+        <v/>
+      </c>
+      <c r="C53" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D53" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E53" s="29">
+        <f>IFERROR($C53/$B53,"")</f>
+        <v/>
+      </c>
+      <c r="F53" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G53" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A53,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H53" s="21">
+        <f>IFERROR($G53/$B53,"")</f>
+        <v/>
+      </c>
+      <c r="I53" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A53),"")</f>
+        <v/>
+      </c>
+      <c r="J53" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A53),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B54" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A54)</f>
+        <v/>
+      </c>
+      <c r="C54" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D54" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E54" s="29">
+        <f>IFERROR($C54/$B54,"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G54" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A54,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H54" s="21">
+        <f>IFERROR($G54/$B54,"")</f>
+        <v/>
+      </c>
+      <c r="I54" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A54),"")</f>
+        <v/>
+      </c>
+      <c r="J54" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A54),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B55" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A55)</f>
+        <v/>
+      </c>
+      <c r="C55" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D55" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E55" s="29">
+        <f>IFERROR($C55/$B55,"")</f>
+        <v/>
+      </c>
+      <c r="F55" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G55" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A55,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H55" s="21">
+        <f>IFERROR($G55/$B55,"")</f>
+        <v/>
+      </c>
+      <c r="I55" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A55),"")</f>
+        <v/>
+      </c>
+      <c r="J55" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A55),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B51" s="30">
-        <f>SUM(B4:B50)</f>
-        <v/>
-      </c>
-      <c r="C51" s="30">
-        <f>SUM(C4:C50)</f>
-        <v/>
-      </c>
-      <c r="D51" s="30">
-        <f>SUM(D4:D50)</f>
-        <v/>
-      </c>
-      <c r="E51" s="31">
-        <f>IFERROR(C51/B51,"")</f>
-        <v/>
-      </c>
-      <c r="F51" s="32">
-        <f>SUM(F4:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="32">
-        <f>SUM(G4:G50)</f>
-        <v/>
-      </c>
-      <c r="H51" s="32">
-        <f>IFERROR(G51/B51,"")</f>
+      <c r="B56" s="30">
+        <f>SUM(B4:B55)</f>
+        <v/>
+      </c>
+      <c r="C56" s="30">
+        <f>SUM(C4:C55)</f>
+        <v/>
+      </c>
+      <c r="D56" s="30">
+        <f>SUM(D4:D55)</f>
+        <v/>
+      </c>
+      <c r="E56" s="31">
+        <f>IFERROR(C56/B56,"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="32">
+        <f>SUM(F4:F55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="32">
+        <f>SUM(G4:G55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="32">
+        <f>IFERROR(G56/B56,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-08 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -6052,14 +6052,18 @@
       <c r="F94" s="26" t="n">
         <v>1261</v>
       </c>
-      <c r="G94" s="24" t="inlineStr"/>
-      <c r="H94" s="25" t="inlineStr"/>
+      <c r="G94" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="H94" s="25" t="n">
+        <v>185.135</v>
+      </c>
       <c r="I94" s="21">
         <f>IF(OR($B94="",$H94=""),"",IF($C94="LONG",($H94-$E94)*$F94,($E94-$H94)*$F94))</f>
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>401.26</v>
+        <v>667.05</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6146,14 +6150,18 @@
       <c r="F96" s="26" t="n">
         <v>959</v>
       </c>
-      <c r="G96" s="24" t="inlineStr"/>
-      <c r="H96" s="25" t="inlineStr"/>
+      <c r="G96" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="H96" s="25" t="n">
+        <v>249.6418</v>
+      </c>
       <c r="I96" s="21">
         <f>IF(OR($B96="",$H96=""),"",IF($C96="LONG",($H96-$E96)*$F96,($E96-$H96)*$F96))</f>
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>398.2</v>
+        <v>670.16</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6463,19 +6471,39 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="23" t="n"/>
-      <c r="B103" s="23" t="n"/>
-      <c r="C103" s="23" t="n"/>
-      <c r="D103" s="24" t="n"/>
-      <c r="E103" s="25" t="n"/>
-      <c r="F103" s="26" t="n"/>
-      <c r="G103" s="24" t="n"/>
-      <c r="H103" s="25" t="n"/>
+      <c r="A103" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090817409</t>
+        </is>
+      </c>
+      <c r="B103" s="23" t="inlineStr">
+        <is>
+          <t>CHEMPLASTS</t>
+        </is>
+      </c>
+      <c r="C103" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D103" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E103" s="25" t="n">
+        <v>184.8514</v>
+      </c>
+      <c r="F103" s="26" t="n">
+        <v>1261</v>
+      </c>
+      <c r="G103" s="24" t="inlineStr"/>
+      <c r="H103" s="25" t="inlineStr"/>
       <c r="I103" s="21">
         <f>IF(OR($B103="",$H103=""),"",IF($C103="LONG",($H103-$E103)*$F103,($E103-$H103)*$F103))</f>
         <v/>
       </c>
-      <c r="J103" s="4" t="n"/>
+      <c r="J103" s="4" t="n">
+        <v>90.59</v>
+      </c>
       <c r="K103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($J103="",0,$J103))</f>
         <v/>
@@ -6490,19 +6518,39 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="23" t="n"/>
-      <c r="B104" s="23" t="n"/>
-      <c r="C104" s="23" t="n"/>
-      <c r="D104" s="24" t="n"/>
-      <c r="E104" s="25" t="n"/>
-      <c r="F104" s="26" t="n"/>
-      <c r="G104" s="24" t="n"/>
-      <c r="H104" s="25" t="n"/>
+      <c r="A104" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090817509</t>
+        </is>
+      </c>
+      <c r="B104" s="23" t="inlineStr">
+        <is>
+          <t>HIKAL</t>
+        </is>
+      </c>
+      <c r="C104" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D104" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E104" s="25" t="n">
+        <v>250.9033</v>
+      </c>
+      <c r="F104" s="26" t="n">
+        <v>959</v>
+      </c>
+      <c r="G104" s="24" t="inlineStr"/>
+      <c r="H104" s="25" t="inlineStr"/>
       <c r="I104" s="21">
         <f>IF(OR($B104="",$H104=""),"",IF($C104="LONG",($H104-$E104)*$F104,($E104-$H104)*$F104))</f>
         <v/>
       </c>
-      <c r="J104" s="4" t="n"/>
+      <c r="J104" s="4" t="n">
+        <v>92.75</v>
+      </c>
       <c r="K104" s="21">
         <f>IF(OR($B104="",$I104=""),"",$I104-IF($J104="",0,$J104))</f>
         <v/>

</xml_diff>

<commit_message>
Data update — 2026-09-09 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>570.0599999999999</v>
+        <v>570.03</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>686.25</v>
+        <v>686.28</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>568.91</v>
+        <v>568.88</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>660.97</v>
+        <v>660.9400000000001</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>588.4</v>
+        <v>588.48</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>397.66</v>
+        <v>397.65</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>413</v>
+        <v>412.99</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>375.65</v>
+        <v>375.69</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>413.34</v>
+        <v>413.32</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>378.85</v>
+        <v>378.87</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>412.76</v>
+        <v>412.75</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>405.47</v>
+        <v>405.45</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.97</v>
+        <v>865.58</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>395.75</v>
+        <v>391.18</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>354.37</v>
+        <v>349.79</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>354.52</v>
+        <v>349.89</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>390.79</v>
+        <v>386.3</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>987.89</v>
+        <v>978.3099999999999</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>965.7</v>
+        <v>957.7</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>1001.93</v>
+        <v>992.3</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>545.22</v>
+        <v>599.74</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>616.22</v>
+        <v>600.85</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>695.01</v>
+        <v>678.41</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>619.58</v>
+        <v>672.55</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>547.97</v>
+        <v>538.71</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>631.8</v>
+        <v>626.49</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>623.02</v>
+        <v>617.78</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>615.9</v>
+        <v>611.13</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>689.77</v>
+        <v>689.78</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>613.25</v>
+        <v>613.3099999999999</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>439.24</v>
+        <v>439.26</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>385.26</v>
+        <v>385.27</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>383.87</v>
+        <v>383.88</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>329.58</v>
+        <v>329.59</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>331.14</v>
+        <v>331.16</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>332.59</v>
+        <v>332.41</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>667.05</v>
+        <v>433.6</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6114,7 +6114,7 @@
         <v/>
       </c>
       <c r="J95" s="4" t="n">
-        <v>267.46</v>
+        <v>181.46</v>
       </c>
       <c r="K95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($J95="",0,$J95))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>670.16</v>
+        <v>430.76</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>658.89</v>
+        <v>487.6</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6318,7 +6318,7 @@
         <v/>
       </c>
       <c r="J99" s="4" t="n">
-        <v>287.94</v>
+        <v>311.54</v>
       </c>
       <c r="K99" s="21">
         <f>IF(OR($B99="",$I99=""),"",$I99-IF($J99="",0,$J99))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>658.87</v>
+        <v>487.69</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6511,14 +6511,18 @@
       <c r="F103" s="26" t="n">
         <v>91</v>
       </c>
-      <c r="G103" s="24" t="inlineStr"/>
-      <c r="H103" s="25" t="inlineStr"/>
+      <c r="G103" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H103" s="25" t="n">
+        <v>1138.4203</v>
+      </c>
       <c r="I103" s="21">
         <f>IF(OR($B103="",$H103=""),"",IF($C103="LONG",($H103-$E103)*$F103,($E103-$H103)*$F103))</f>
         <v/>
       </c>
       <c r="J103" s="4" t="n">
-        <v>133.89</v>
+        <v>241.35</v>
       </c>
       <c r="K103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($J103="",0,$J103))</f>
@@ -6558,14 +6562,18 @@
       <c r="F104" s="26" t="n">
         <v>9469</v>
       </c>
-      <c r="G104" s="24" t="inlineStr"/>
-      <c r="H104" s="25" t="inlineStr"/>
+      <c r="G104" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H104" s="25" t="n">
+        <v>10.7</v>
+      </c>
       <c r="I104" s="21">
         <f>IF(OR($B104="",$H104=""),"",IF($C104="LONG",($H104-$E104)*$F104,($E104-$H104)*$F104))</f>
         <v/>
       </c>
       <c r="J104" s="4" t="n">
-        <v>133.35</v>
+        <v>238.47</v>
       </c>
       <c r="K104" s="21">
         <f>IF(OR($B104="",$I104=""),"",$I104-IF($J104="",0,$J104))</f>
@@ -6616,7 +6624,7 @@
         <v/>
       </c>
       <c r="J105" s="4" t="n">
-        <v>129.57</v>
+        <v>337.14</v>
       </c>
       <c r="K105" s="21">
         <f>IF(OR($B105="",$I105=""),"",$I105-IF($J105="",0,$J105))</f>
@@ -6667,7 +6675,7 @@
         <v/>
       </c>
       <c r="J106" s="4" t="n">
-        <v>86.03</v>
+        <v>172.01</v>
       </c>
       <c r="K106" s="21">
         <f>IF(OR($B106="",$I106=""),"",$I106-IF($J106="",0,$J106))</f>
@@ -6718,7 +6726,7 @@
         <v/>
       </c>
       <c r="J107" s="4" t="n">
-        <v>131.76</v>
+        <v>343.41</v>
       </c>
       <c r="K107" s="21">
         <f>IF(OR($B107="",$I107=""),"",$I107-IF($J107="",0,$J107))</f>
@@ -6758,14 +6766,18 @@
       <c r="F108" s="26" t="n">
         <v>54</v>
       </c>
-      <c r="G108" s="24" t="inlineStr"/>
-      <c r="H108" s="25" t="inlineStr"/>
+      <c r="G108" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H108" s="25" t="n">
+        <v>1990.874</v>
+      </c>
       <c r="I108" s="21">
         <f>IF(OR($B108="",$H108=""),"",IF($C108="LONG",($H108-$E108)*$F108,($E108-$H108)*$F108))</f>
         <v/>
       </c>
       <c r="J108" s="4" t="n">
-        <v>132.11</v>
+        <v>243.65</v>
       </c>
       <c r="K108" s="21">
         <f>IF(OR($B108="",$I108=""),"",$I108-IF($J108="",0,$J108))</f>
@@ -6816,7 +6828,7 @@
         <v/>
       </c>
       <c r="J109" s="4" t="n">
-        <v>128.69</v>
+        <v>278.06</v>
       </c>
       <c r="K109" s="21">
         <f>IF(OR($B109="",$I109=""),"",$I109-IF($J109="",0,$J109))</f>
@@ -6856,14 +6868,18 @@
       <c r="F110" s="26" t="n">
         <v>324</v>
       </c>
-      <c r="G110" s="24" t="inlineStr"/>
-      <c r="H110" s="25" t="inlineStr"/>
+      <c r="G110" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H110" s="25" t="n">
+        <v>614.6335</v>
+      </c>
       <c r="I110" s="21">
         <f>IF(OR($B110="",$H110=""),"",IF($C110="LONG",($H110-$E110)*$F110,($E110-$H110)*$F110))</f>
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>309.97</v>
+        <v>586.91</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6914,7 +6930,7 @@
         <v/>
       </c>
       <c r="J111" s="4" t="n">
-        <v>128</v>
+        <v>275.39</v>
       </c>
       <c r="K111" s="21">
         <f>IF(OR($B111="",$I111=""),"",$I111-IF($J111="",0,$J111))</f>
@@ -6954,14 +6970,18 @@
       <c r="F112" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="G112" s="24" t="inlineStr"/>
-      <c r="H112" s="25" t="inlineStr"/>
+      <c r="G112" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H112" s="25" t="n">
+        <v>1990.0922</v>
+      </c>
       <c r="I112" s="21">
         <f>IF(OR($B112="",$H112=""),"",IF($C112="LONG",($H112-$E112)*$F112,($E112-$H112)*$F112))</f>
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>310.52</v>
+        <v>585.62</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -6977,19 +6997,39 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="23" t="n"/>
-      <c r="B113" s="23" t="n"/>
-      <c r="C113" s="23" t="n"/>
-      <c r="D113" s="24" t="n"/>
-      <c r="E113" s="25" t="n"/>
-      <c r="F113" s="26" t="n"/>
-      <c r="G113" s="24" t="n"/>
-      <c r="H113" s="25" t="n"/>
+      <c r="A113" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260909716709</t>
+        </is>
+      </c>
+      <c r="B113" s="23" t="inlineStr">
+        <is>
+          <t>ANTELOPUS</t>
+        </is>
+      </c>
+      <c r="C113" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D113" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E113" s="25" t="n">
+        <v>1162.9767</v>
+      </c>
+      <c r="F113" s="26" t="n">
+        <v>75</v>
+      </c>
+      <c r="G113" s="24" t="inlineStr"/>
+      <c r="H113" s="25" t="inlineStr"/>
       <c r="I113" s="21">
         <f>IF(OR($B113="",$H113=""),"",IF($C113="LONG",($H113-$E113)*$F113,($E113-$H113)*$F113))</f>
         <v/>
       </c>
-      <c r="J113" s="4" t="n"/>
+      <c r="J113" s="4" t="n">
+        <v>118.32</v>
+      </c>
       <c r="K113" s="21">
         <f>IF(OR($B113="",$I113=""),"",$I113-IF($J113="",0,$J113))</f>
         <v/>
@@ -7004,19 +7044,43 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="23" t="n"/>
-      <c r="B114" s="23" t="n"/>
-      <c r="C114" s="23" t="n"/>
-      <c r="D114" s="24" t="n"/>
-      <c r="E114" s="25" t="n"/>
-      <c r="F114" s="26" t="n"/>
-      <c r="G114" s="24" t="n"/>
-      <c r="H114" s="25" t="n"/>
+      <c r="A114" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260909102909</t>
+        </is>
+      </c>
+      <c r="B114" s="23" t="inlineStr">
+        <is>
+          <t>ANTELOPUS</t>
+        </is>
+      </c>
+      <c r="C114" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D114" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E114" s="25" t="n">
+        <v>1140.9686</v>
+      </c>
+      <c r="F114" s="26" t="n">
+        <v>91</v>
+      </c>
+      <c r="G114" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H114" s="25" t="n">
+        <v>1162.65</v>
+      </c>
       <c r="I114" s="21">
         <f>IF(OR($B114="",$H114=""),"",IF($C114="LONG",($H114-$E114)*$F114,($E114-$H114)*$F114))</f>
         <v/>
       </c>
-      <c r="J114" s="4" t="n"/>
+      <c r="J114" s="4" t="n">
+        <v>84.17</v>
+      </c>
       <c r="K114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($J114="",0,$J114))</f>
         <v/>
@@ -7031,19 +7095,43 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="23" t="n"/>
-      <c r="B115" s="23" t="n"/>
-      <c r="C115" s="23" t="n"/>
-      <c r="D115" s="24" t="n"/>
-      <c r="E115" s="25" t="n"/>
-      <c r="F115" s="26" t="n"/>
-      <c r="G115" s="24" t="n"/>
-      <c r="H115" s="25" t="n"/>
+      <c r="A115" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260909102809</t>
+        </is>
+      </c>
+      <c r="B115" s="23" t="inlineStr">
+        <is>
+          <t>BCG</t>
+        </is>
+      </c>
+      <c r="C115" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D115" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E115" s="25" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F115" s="26" t="n">
+        <v>9469</v>
+      </c>
+      <c r="G115" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H115" s="25" t="n">
+        <v>10.16</v>
+      </c>
       <c r="I115" s="21">
         <f>IF(OR($B115="",$H115=""),"",IF($C115="LONG",($H115-$E115)*$F115,($E115-$H115)*$F115))</f>
         <v/>
       </c>
-      <c r="J115" s="4" t="n"/>
+      <c r="J115" s="4" t="n">
+        <v>82.8</v>
+      </c>
       <c r="K115" s="21">
         <f>IF(OR($B115="",$I115=""),"",$I115-IF($J115="",0,$J115))</f>
         <v/>
@@ -7058,19 +7146,39 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="23" t="n"/>
-      <c r="B116" s="23" t="n"/>
-      <c r="C116" s="23" t="n"/>
-      <c r="D116" s="24" t="n"/>
-      <c r="E116" s="25" t="n"/>
-      <c r="F116" s="26" t="n"/>
-      <c r="G116" s="24" t="n"/>
-      <c r="H116" s="25" t="n"/>
+      <c r="A116" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090981309</t>
+        </is>
+      </c>
+      <c r="B116" s="23" t="inlineStr">
+        <is>
+          <t>EIEL</t>
+        </is>
+      </c>
+      <c r="C116" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D116" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E116" s="25" t="n">
+        <v>206.0991</v>
+      </c>
+      <c r="F116" s="26" t="n">
+        <v>847</v>
+      </c>
+      <c r="G116" s="24" t="inlineStr"/>
+      <c r="H116" s="25" t="inlineStr"/>
       <c r="I116" s="21">
         <f>IF(OR($B116="",$H116=""),"",IF($C116="LONG",($H116-$E116)*$F116,($E116-$H116)*$F116))</f>
         <v/>
       </c>
-      <c r="J116" s="4" t="n"/>
+      <c r="J116" s="4" t="n">
+        <v>281.03</v>
+      </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
         <v/>
@@ -7085,19 +7193,39 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="23" t="n"/>
-      <c r="B117" s="23" t="n"/>
-      <c r="C117" s="23" t="n"/>
-      <c r="D117" s="24" t="n"/>
-      <c r="E117" s="25" t="n"/>
-      <c r="F117" s="26" t="n"/>
-      <c r="G117" s="24" t="n"/>
-      <c r="H117" s="25" t="n"/>
+      <c r="A117" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090980209</t>
+        </is>
+      </c>
+      <c r="B117" s="23" t="inlineStr">
+        <is>
+          <t>INDNIPPON</t>
+        </is>
+      </c>
+      <c r="C117" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D117" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E117" s="25" t="n">
+        <v>1340</v>
+      </c>
+      <c r="F117" s="26" t="n">
+        <v>207</v>
+      </c>
+      <c r="G117" s="24" t="inlineStr"/>
+      <c r="H117" s="25" t="inlineStr"/>
       <c r="I117" s="21">
         <f>IF(OR($B117="",$H117=""),"",IF($C117="LONG",($H117-$E117)*$F117,($E117-$H117)*$F117))</f>
         <v/>
       </c>
-      <c r="J117" s="4" t="n"/>
+      <c r="J117" s="4" t="n">
+        <v>403.11</v>
+      </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
         <v/>
@@ -7112,19 +7240,39 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="23" t="n"/>
-      <c r="B118" s="23" t="n"/>
-      <c r="C118" s="23" t="n"/>
-      <c r="D118" s="24" t="n"/>
-      <c r="E118" s="25" t="n"/>
-      <c r="F118" s="26" t="n"/>
-      <c r="G118" s="24" t="n"/>
-      <c r="H118" s="25" t="n"/>
+      <c r="A118" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090981209</t>
+        </is>
+      </c>
+      <c r="B118" s="23" t="inlineStr">
+        <is>
+          <t>INDORAMA</t>
+        </is>
+      </c>
+      <c r="C118" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D118" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E118" s="25" t="n">
+        <v>85.4701</v>
+      </c>
+      <c r="F118" s="26" t="n">
+        <v>1022</v>
+      </c>
+      <c r="G118" s="24" t="inlineStr"/>
+      <c r="H118" s="25" t="inlineStr"/>
       <c r="I118" s="21">
         <f>IF(OR($B118="",$H118=""),"",IF($C118="LONG",($H118-$E118)*$F118,($E118-$H118)*$F118))</f>
         <v/>
       </c>
-      <c r="J118" s="4" t="n"/>
+      <c r="J118" s="4" t="n">
+        <v>118.47</v>
+      </c>
       <c r="K118" s="21">
         <f>IF(OR($B118="",$I118=""),"",$I118-IF($J118="",0,$J118))</f>
         <v/>
@@ -7139,19 +7287,39 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="23" t="n"/>
-      <c r="B119" s="23" t="n"/>
-      <c r="C119" s="23" t="n"/>
-      <c r="D119" s="24" t="n"/>
-      <c r="E119" s="25" t="n"/>
-      <c r="F119" s="26" t="n"/>
-      <c r="G119" s="24" t="n"/>
-      <c r="H119" s="25" t="n"/>
+      <c r="A119" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260909100409</t>
+        </is>
+      </c>
+      <c r="B119" s="23" t="inlineStr">
+        <is>
+          <t>NOVARTIND</t>
+        </is>
+      </c>
+      <c r="C119" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D119" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E119" s="25" t="n">
+        <v>1982.2908</v>
+      </c>
+      <c r="F119" s="26" t="n">
+        <v>54</v>
+      </c>
+      <c r="G119" s="24" t="inlineStr"/>
+      <c r="H119" s="25" t="inlineStr"/>
       <c r="I119" s="21">
         <f>IF(OR($B119="",$H119=""),"",IF($C119="LONG",($H119-$E119)*$F119,($E119-$H119)*$F119))</f>
         <v/>
       </c>
-      <c r="J119" s="4" t="n"/>
+      <c r="J119" s="4" t="n">
+        <v>54.36</v>
+      </c>
       <c r="K119" s="21">
         <f>IF(OR($B119="",$I119=""),"",$I119-IF($J119="",0,$J119))</f>
         <v/>
@@ -7166,19 +7334,39 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="23" t="n"/>
-      <c r="B120" s="23" t="n"/>
-      <c r="C120" s="23" t="n"/>
-      <c r="D120" s="24" t="n"/>
-      <c r="E120" s="25" t="n"/>
-      <c r="F120" s="26" t="n"/>
-      <c r="G120" s="24" t="n"/>
-      <c r="H120" s="25" t="n"/>
+      <c r="A120" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260909672309</t>
+        </is>
+      </c>
+      <c r="B120" s="23" t="inlineStr">
+        <is>
+          <t>RESPONIND</t>
+        </is>
+      </c>
+      <c r="C120" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D120" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E120" s="25" t="n">
+        <v>169.585</v>
+      </c>
+      <c r="F120" s="26" t="n">
+        <v>1026</v>
+      </c>
+      <c r="G120" s="24" t="inlineStr"/>
+      <c r="H120" s="25" t="inlineStr"/>
       <c r="I120" s="21">
         <f>IF(OR($B120="",$H120=""),"",IF($C120="LONG",($H120-$E120)*$F120,($E120-$H120)*$F120))</f>
         <v/>
       </c>
-      <c r="J120" s="4" t="n"/>
+      <c r="J120" s="4" t="n">
+        <v>280.35</v>
+      </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
         <v/>
@@ -7193,19 +7381,39 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="23" t="n"/>
-      <c r="B121" s="23" t="n"/>
-      <c r="C121" s="23" t="n"/>
-      <c r="D121" s="24" t="n"/>
-      <c r="E121" s="25" t="n"/>
-      <c r="F121" s="26" t="n"/>
-      <c r="G121" s="24" t="n"/>
-      <c r="H121" s="25" t="n"/>
+      <c r="A121" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126090989309</t>
+        </is>
+      </c>
+      <c r="B121" s="23" t="inlineStr">
+        <is>
+          <t>SHAREINDIA</t>
+        </is>
+      </c>
+      <c r="C121" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D121" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E121" s="25" t="n">
+        <v>190.2983</v>
+      </c>
+      <c r="F121" s="26" t="n">
+        <v>923</v>
+      </c>
+      <c r="G121" s="24" t="inlineStr"/>
+      <c r="H121" s="25" t="inlineStr"/>
       <c r="I121" s="21">
         <f>IF(OR($B121="",$H121=""),"",IF($C121="LONG",($H121-$E121)*$F121,($E121-$H121)*$F121))</f>
         <v/>
       </c>
-      <c r="J121" s="4" t="n"/>
+      <c r="J121" s="4" t="n">
+        <v>282.31</v>
+      </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
         <v/>
@@ -7220,19 +7428,43 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="23" t="n"/>
-      <c r="B122" s="23" t="n"/>
-      <c r="C122" s="23" t="n"/>
-      <c r="D122" s="24" t="n"/>
-      <c r="E122" s="25" t="n"/>
-      <c r="F122" s="26" t="n"/>
-      <c r="G122" s="24" t="n"/>
-      <c r="H122" s="25" t="n"/>
+      <c r="A122" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126090953709</t>
+        </is>
+      </c>
+      <c r="B122" s="23" t="inlineStr">
+        <is>
+          <t>SYMPHONY</t>
+        </is>
+      </c>
+      <c r="C122" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D122" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E122" s="25" t="n">
+        <v>613.9752</v>
+      </c>
+      <c r="F122" s="26" t="n">
+        <v>324</v>
+      </c>
+      <c r="G122" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H122" s="25" t="n">
+        <v>616.5076</v>
+      </c>
       <c r="I122" s="21">
         <f>IF(OR($B122="",$H122=""),"",IF($C122="LONG",($H122-$E122)*$F122,($E122-$H122)*$F122))</f>
         <v/>
       </c>
-      <c r="J122" s="4" t="n"/>
+      <c r="J122" s="4" t="n">
+        <v>117.84</v>
+      </c>
       <c r="K122" s="21">
         <f>IF(OR($B122="",$I122=""),"",$I122-IF($J122="",0,$J122))</f>
         <v/>
@@ -7247,19 +7479,43 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="23" t="n"/>
-      <c r="B123" s="23" t="n"/>
-      <c r="C123" s="23" t="n"/>
-      <c r="D123" s="24" t="n"/>
-      <c r="E123" s="25" t="n"/>
-      <c r="F123" s="26" t="n"/>
-      <c r="G123" s="24" t="n"/>
-      <c r="H123" s="25" t="n"/>
+      <c r="A123" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260909100309</t>
+        </is>
+      </c>
+      <c r="B123" s="23" t="inlineStr">
+        <is>
+          <t>VENUSPIPES</t>
+        </is>
+      </c>
+      <c r="C123" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D123" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E123" s="25" t="n">
+        <v>1987.3264</v>
+      </c>
+      <c r="F123" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="G123" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H123" s="25" t="n">
+        <v>1943.597</v>
+      </c>
       <c r="I123" s="21">
         <f>IF(OR($B123="",$H123=""),"",IF($C123="LONG",($H123-$E123)*$F123,($E123-$H123)*$F123))</f>
         <v/>
       </c>
-      <c r="J123" s="4" t="n"/>
+      <c r="J123" s="4" t="n">
+        <v>118.82</v>
+      </c>
       <c r="K123" s="21">
         <f>IF(OR($B123="",$I123=""),"",$I123-IF($J123="",0,$J123))</f>
         <v/>
@@ -31464,7 +31720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31935,7 +32191,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -31978,7 +32234,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -32021,7 +32277,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -32064,7 +32320,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -32107,7 +32363,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -32150,7 +32406,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -32193,7 +32449,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -32236,7 +32492,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32279,7 +32535,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32322,7 +32578,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32365,7 +32621,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32408,7 +32664,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32451,7 +32707,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -32494,7 +32750,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -32537,7 +32793,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -32580,7 +32836,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -32623,7 +32879,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -32666,7 +32922,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -32709,7 +32965,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -32752,7 +33008,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -32795,7 +33051,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -32838,7 +33094,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -32881,7 +33137,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -32924,7 +33180,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -32967,7 +33223,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -33010,7 +33266,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -33053,7 +33309,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33096,7 +33352,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33139,7 +33395,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33182,7 +33438,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33225,7 +33481,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33268,7 +33524,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33311,7 +33567,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33354,7 +33610,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33397,7 +33653,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33440,7 +33696,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33483,7 +33739,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33526,7 +33782,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33569,7 +33825,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -33612,7 +33868,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -33655,7 +33911,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -33698,7 +33954,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -33741,7 +33997,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -33784,7 +34040,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -33827,7 +34083,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -33870,7 +34126,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -33913,7 +34169,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -33954,37 +34210,252 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B60" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A60)</f>
+        <v/>
+      </c>
+      <c r="C60" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D60" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E60" s="29">
+        <f>IFERROR($C60/$B60,"")</f>
+        <v/>
+      </c>
+      <c r="F60" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G60" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A60,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H60" s="21">
+        <f>IFERROR($G60/$B60,"")</f>
+        <v/>
+      </c>
+      <c r="I60" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A60),"")</f>
+        <v/>
+      </c>
+      <c r="J60" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A60),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B61" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A61)</f>
+        <v/>
+      </c>
+      <c r="C61" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D61" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E61" s="29">
+        <f>IFERROR($C61/$B61,"")</f>
+        <v/>
+      </c>
+      <c r="F61" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G61" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A61,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H61" s="21">
+        <f>IFERROR($G61/$B61,"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A61),"")</f>
+        <v/>
+      </c>
+      <c r="J61" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A61),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B62" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A62)</f>
+        <v/>
+      </c>
+      <c r="C62" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A62,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D62" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A62,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E62" s="29">
+        <f>IFERROR($C62/$B62,"")</f>
+        <v/>
+      </c>
+      <c r="F62" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A62,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G62" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A62,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H62" s="21">
+        <f>IFERROR($G62/$B62,"")</f>
+        <v/>
+      </c>
+      <c r="I62" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A62),"")</f>
+        <v/>
+      </c>
+      <c r="J62" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A62),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B63" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A63)</f>
+        <v/>
+      </c>
+      <c r="C63" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A63,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D63" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A63,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E63" s="29">
+        <f>IFERROR($C63/$B63,"")</f>
+        <v/>
+      </c>
+      <c r="F63" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A63,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G63" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A63,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H63" s="21">
+        <f>IFERROR($G63/$B63,"")</f>
+        <v/>
+      </c>
+      <c r="I63" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A63),"")</f>
+        <v/>
+      </c>
+      <c r="J63" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A63),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B64" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A64)</f>
+        <v/>
+      </c>
+      <c r="C64" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A64,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D64" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A64,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E64" s="29">
+        <f>IFERROR($C64/$B64,"")</f>
+        <v/>
+      </c>
+      <c r="F64" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A64,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G64" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A64,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H64" s="21">
+        <f>IFERROR($G64/$B64,"")</f>
+        <v/>
+      </c>
+      <c r="I64" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A64),"")</f>
+        <v/>
+      </c>
+      <c r="J64" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A64),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B60" s="30">
-        <f>SUM(B4:B59)</f>
-        <v/>
-      </c>
-      <c r="C60" s="30">
-        <f>SUM(C4:C59)</f>
-        <v/>
-      </c>
-      <c r="D60" s="30">
-        <f>SUM(D4:D59)</f>
-        <v/>
-      </c>
-      <c r="E60" s="31">
-        <f>IFERROR(C60/B60,"")</f>
-        <v/>
-      </c>
-      <c r="F60" s="32">
-        <f>SUM(F4:F59)</f>
-        <v/>
-      </c>
-      <c r="G60" s="32">
-        <f>SUM(G4:G59)</f>
-        <v/>
-      </c>
-      <c r="H60" s="32">
-        <f>IFERROR(G60/B60,"")</f>
+      <c r="B65" s="30">
+        <f>SUM(B4:B64)</f>
+        <v/>
+      </c>
+      <c r="C65" s="30">
+        <f>SUM(C4:C64)</f>
+        <v/>
+      </c>
+      <c r="D65" s="30">
+        <f>SUM(D4:D64)</f>
+        <v/>
+      </c>
+      <c r="E65" s="31">
+        <f>IFERROR(C65/B65,"")</f>
+        <v/>
+      </c>
+      <c r="F65" s="32">
+        <f>SUM(F4:F64)</f>
+        <v/>
+      </c>
+      <c r="G65" s="32">
+        <f>SUM(G4:G64)</f>
+        <v/>
+      </c>
+      <c r="H65" s="32">
+        <f>IFERROR(G65/B65,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconcile NOVARTIND's short: stopped out at 10:35am, not left open
square_off_239's mismatch-safety-check correctly skipped it rather than
guess -- the resting stop-loss order triggered mid-day but surfaced under
a new broker order id (321260909315209) instead of updating the original,
so both cancel attempts at 2:39pm found "already cancelled" and the real
broker short qty read 0 against a local record of 54. Reconciled by hand
from dhan_trades.log + dhan_live_monitor.log order-update timestamps:
covered at avg ₹2,159.2258, realized_pnl -₹9,554.49.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -7311,14 +7311,18 @@
       <c r="F119" s="26" t="n">
         <v>54</v>
       </c>
-      <c r="G119" s="24" t="inlineStr"/>
-      <c r="H119" s="25" t="inlineStr"/>
+      <c r="G119" s="24" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H119" s="25" t="n">
+        <v>2159.2258</v>
+      </c>
       <c r="I119" s="21">
         <f>IF(OR($B119="",$H119=""),"",IF($C119="LONG",($H119-$E119)*$F119,($E119-$H119)*$F119))</f>
         <v/>
       </c>
       <c r="J119" s="4" t="n">
-        <v>54.36</v>
+        <v>85.81999999999999</v>
       </c>
       <c r="K119" s="21">
         <f>IF(OR($B119="",$I119=""),"",$I119-IF($J119="",0,$J119))</f>

</xml_diff>

<commit_message>
Data update — 2026-09-10 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>570.03</v>
+        <v>571.84</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>686.28</v>
+        <v>688.87</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>568.88</v>
+        <v>570.6900000000001</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>660.9400000000001</v>
+        <v>663.11</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>588.48</v>
+        <v>590.6900000000001</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>397.65</v>
+        <v>398.65</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>412.99</v>
+        <v>414.2</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>375.69</v>
+        <v>345.09</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>413.32</v>
+        <v>414.53</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>378.87</v>
+        <v>380.23</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>412.75</v>
+        <v>413.96</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>405.45</v>
+        <v>406.49</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>865.58</v>
+        <v>870.14</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.18</v>
+        <v>391.17</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.89</v>
+        <v>349.9</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.3</v>
+        <v>386.35</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.3099999999999</v>
+        <v>978.3</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.41</v>
+        <v>678.48</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.55</v>
+        <v>672.35</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.71</v>
+        <v>538.7</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>626.49</v>
+        <v>627.15</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>617.78</v>
+        <v>618.4299999999999</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>611.13</v>
+        <v>611.66</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>689.78</v>
+        <v>690.86</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>613.3099999999999</v>
+        <v>614.5599999999999</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>439.26</v>
+        <v>439.99</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>385.27</v>
+        <v>385.88</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>383.88</v>
+        <v>384.49</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>432.95</v>
+        <v>433.57</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>376.31</v>
+        <v>376.58</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>326.83</v>
+        <v>327.05</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>329.59</v>
+        <v>329.86</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>374.48</v>
+        <v>374.78</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>331.16</v>
+        <v>323.17</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>332.41</v>
+        <v>332.64</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>433.6</v>
+        <v>433.62</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6522,7 +6522,7 @@
         <v/>
       </c>
       <c r="J103" s="4" t="n">
-        <v>241.35</v>
+        <v>161.36</v>
       </c>
       <c r="K103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($J103="",0,$J103))</f>
@@ -6573,7 +6573,7 @@
         <v/>
       </c>
       <c r="J104" s="4" t="n">
-        <v>238.47</v>
+        <v>185.66</v>
       </c>
       <c r="K104" s="21">
         <f>IF(OR($B104="",$I104=""),"",$I104-IF($J104="",0,$J104))</f>
@@ -6777,7 +6777,7 @@
         <v/>
       </c>
       <c r="J108" s="4" t="n">
-        <v>243.65</v>
+        <v>187.34</v>
       </c>
       <c r="K108" s="21">
         <f>IF(OR($B108="",$I108=""),"",$I108-IF($J108="",0,$J108))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>586.91</v>
+        <v>437.61</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>585.62</v>
+        <v>382.63</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7021,14 +7021,18 @@
       <c r="F113" s="26" t="n">
         <v>75</v>
       </c>
-      <c r="G113" s="24" t="inlineStr"/>
-      <c r="H113" s="25" t="inlineStr"/>
+      <c r="G113" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H113" s="25" t="n">
+        <v>1137.85</v>
+      </c>
       <c r="I113" s="21">
         <f>IF(OR($B113="",$H113=""),"",IF($C113="LONG",($H113-$E113)*$F113,($E113-$H113)*$F113))</f>
         <v/>
       </c>
       <c r="J113" s="4" t="n">
-        <v>118.32</v>
+        <v>130.14</v>
       </c>
       <c r="K113" s="21">
         <f>IF(OR($B113="",$I113=""),"",$I113-IF($J113="",0,$J113))</f>
@@ -7079,7 +7083,7 @@
         <v/>
       </c>
       <c r="J114" s="4" t="n">
-        <v>84.17</v>
+        <v>126.99</v>
       </c>
       <c r="K114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($J114="",0,$J114))</f>
@@ -7130,7 +7134,7 @@
         <v/>
       </c>
       <c r="J115" s="4" t="n">
-        <v>82.8</v>
+        <v>133.49</v>
       </c>
       <c r="K115" s="21">
         <f>IF(OR($B115="",$I115=""),"",$I115-IF($J115="",0,$J115))</f>
@@ -7170,14 +7174,18 @@
       <c r="F116" s="26" t="n">
         <v>847</v>
       </c>
-      <c r="G116" s="24" t="inlineStr"/>
-      <c r="H116" s="25" t="inlineStr"/>
+      <c r="G116" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H116" s="25" t="n">
+        <v>213.8</v>
+      </c>
       <c r="I116" s="21">
         <f>IF(OR($B116="",$H116=""),"",IF($C116="LONG",($H116-$E116)*$F116,($E116-$H116)*$F116))</f>
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>281.03</v>
+        <v>530.04</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7217,14 +7225,18 @@
       <c r="F117" s="26" t="n">
         <v>207</v>
       </c>
-      <c r="G117" s="24" t="inlineStr"/>
-      <c r="H117" s="25" t="inlineStr"/>
+      <c r="G117" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H117" s="25" t="n">
+        <v>1460.09</v>
+      </c>
       <c r="I117" s="21">
         <f>IF(OR($B117="",$H117=""),"",IF($C117="LONG",($H117-$E117)*$F117,($E117-$H117)*$F117))</f>
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>403.11</v>
+        <v>796.39</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7264,14 +7276,18 @@
       <c r="F118" s="26" t="n">
         <v>1022</v>
       </c>
-      <c r="G118" s="24" t="inlineStr"/>
-      <c r="H118" s="25" t="inlineStr"/>
+      <c r="G118" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H118" s="25" t="n">
+        <v>87.33</v>
+      </c>
       <c r="I118" s="21">
         <f>IF(OR($B118="",$H118=""),"",IF($C118="LONG",($H118-$E118)*$F118,($E118-$H118)*$F118))</f>
         <v/>
       </c>
       <c r="J118" s="4" t="n">
-        <v>118.47</v>
+        <v>211.06</v>
       </c>
       <c r="K118" s="21">
         <f>IF(OR($B118="",$I118=""),"",$I118-IF($J118="",0,$J118))</f>
@@ -7322,7 +7338,7 @@
         <v/>
       </c>
       <c r="J119" s="4" t="n">
-        <v>85.81999999999999</v>
+        <v>145.85</v>
       </c>
       <c r="K119" s="21">
         <f>IF(OR($B119="",$I119=""),"",$I119-IF($J119="",0,$J119))</f>
@@ -7362,14 +7378,18 @@
       <c r="F120" s="26" t="n">
         <v>1026</v>
       </c>
-      <c r="G120" s="24" t="inlineStr"/>
-      <c r="H120" s="25" t="inlineStr"/>
+      <c r="G120" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H120" s="25" t="n">
+        <v>172.17</v>
+      </c>
       <c r="I120" s="21">
         <f>IF(OR($B120="",$H120=""),"",IF($C120="LONG",($H120-$E120)*$F120,($E120-$H120)*$F120))</f>
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>280.35</v>
+        <v>523.87</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7409,14 +7429,18 @@
       <c r="F121" s="26" t="n">
         <v>923</v>
       </c>
-      <c r="G121" s="24" t="inlineStr"/>
-      <c r="H121" s="25" t="inlineStr"/>
+      <c r="G121" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H121" s="25" t="n">
+        <v>201.1</v>
+      </c>
       <c r="I121" s="21">
         <f>IF(OR($B121="",$H121=""),"",IF($C121="LONG",($H121-$E121)*$F121,($E121-$H121)*$F121))</f>
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>282.31</v>
+        <v>529.11</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7467,7 +7491,7 @@
         <v/>
       </c>
       <c r="J122" s="4" t="n">
-        <v>117.84</v>
+        <v>243.77</v>
       </c>
       <c r="K122" s="21">
         <f>IF(OR($B122="",$I122=""),"",$I122-IF($J122="",0,$J122))</f>
@@ -7518,7 +7542,7 @@
         <v/>
       </c>
       <c r="J123" s="4" t="n">
-        <v>118.82</v>
+        <v>296.19</v>
       </c>
       <c r="K123" s="21">
         <f>IF(OR($B123="",$I123=""),"",$I123-IF($J123="",0,$J123))</f>
@@ -7534,19 +7558,43 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="23" t="n"/>
-      <c r="B124" s="23" t="n"/>
-      <c r="C124" s="23" t="n"/>
-      <c r="D124" s="24" t="n"/>
-      <c r="E124" s="25" t="n"/>
-      <c r="F124" s="26" t="n"/>
-      <c r="G124" s="24" t="n"/>
-      <c r="H124" s="25" t="n"/>
+      <c r="A124" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091046509</t>
+        </is>
+      </c>
+      <c r="B124" s="23" t="inlineStr">
+        <is>
+          <t>ANTELOPUS</t>
+        </is>
+      </c>
+      <c r="C124" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D124" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E124" s="25" t="n">
+        <v>1137.38</v>
+      </c>
+      <c r="F124" s="26" t="n">
+        <v>75</v>
+      </c>
+      <c r="G124" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H124" s="25" t="n">
+        <v>1134.24</v>
+      </c>
       <c r="I124" s="21">
         <f>IF(OR($B124="",$H124=""),"",IF($C124="LONG",($H124-$E124)*$F124,($E124-$H124)*$F124))</f>
         <v/>
       </c>
-      <c r="J124" s="4" t="n"/>
+      <c r="J124" s="4" t="n">
+        <v>77.45</v>
+      </c>
       <c r="K124" s="21">
         <f>IF(OR($B124="",$I124=""),"",$I124-IF($J124="",0,$J124))</f>
         <v/>
@@ -7561,19 +7609,43 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="23" t="n"/>
-      <c r="B125" s="23" t="n"/>
-      <c r="C125" s="23" t="n"/>
-      <c r="D125" s="24" t="n"/>
-      <c r="E125" s="25" t="n"/>
-      <c r="F125" s="26" t="n"/>
-      <c r="G125" s="24" t="n"/>
-      <c r="H125" s="25" t="n"/>
+      <c r="A125" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091019209</t>
+        </is>
+      </c>
+      <c r="B125" s="23" t="inlineStr">
+        <is>
+          <t>EIEL</t>
+        </is>
+      </c>
+      <c r="C125" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D125" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E125" s="25" t="n">
+        <v>213.59</v>
+      </c>
+      <c r="F125" s="26" t="n">
+        <v>847</v>
+      </c>
+      <c r="G125" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H125" s="25" t="n">
+        <v>213.18</v>
+      </c>
       <c r="I125" s="21">
         <f>IF(OR($B125="",$H125=""),"",IF($C125="LONG",($H125-$E125)*$F125,($E125-$H125)*$F125))</f>
         <v/>
       </c>
-      <c r="J125" s="4" t="n"/>
+      <c r="J125" s="4" t="n">
+        <v>111.37</v>
+      </c>
       <c r="K125" s="21">
         <f>IF(OR($B125="",$I125=""),"",$I125-IF($J125="",0,$J125))</f>
         <v/>
@@ -7588,19 +7660,43 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="23" t="n"/>
-      <c r="B126" s="23" t="n"/>
-      <c r="C126" s="23" t="n"/>
-      <c r="D126" s="24" t="n"/>
-      <c r="E126" s="25" t="n"/>
-      <c r="F126" s="26" t="n"/>
-      <c r="G126" s="24" t="n"/>
-      <c r="H126" s="25" t="n"/>
+      <c r="A126" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126091099109</t>
+        </is>
+      </c>
+      <c r="B126" s="23" t="inlineStr">
+        <is>
+          <t>INDNIPPON</t>
+        </is>
+      </c>
+      <c r="C126" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D126" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E126" s="25" t="n">
+        <v>1456.15</v>
+      </c>
+      <c r="F126" s="26" t="n">
+        <v>207</v>
+      </c>
+      <c r="G126" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H126" s="25" t="n">
+        <v>1552.9169</v>
+      </c>
       <c r="I126" s="21">
         <f>IF(OR($B126="",$H126=""),"",IF($C126="LONG",($H126-$E126)*$F126,($E126-$H126)*$F126))</f>
         <v/>
       </c>
-      <c r="J126" s="4" t="n"/>
+      <c r="J126" s="4" t="n">
+        <v>155.5</v>
+      </c>
       <c r="K126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($J126="",0,$J126))</f>
         <v/>
@@ -7615,19 +7711,39 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="23" t="n"/>
-      <c r="B127" s="23" t="n"/>
-      <c r="C127" s="23" t="n"/>
-      <c r="D127" s="24" t="n"/>
-      <c r="E127" s="25" t="n"/>
-      <c r="F127" s="26" t="n"/>
-      <c r="G127" s="24" t="n"/>
-      <c r="H127" s="25" t="n"/>
+      <c r="A127" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260910622509</t>
+        </is>
+      </c>
+      <c r="B127" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C127" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D127" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E127" s="25" t="n">
+        <v>253.0721</v>
+      </c>
+      <c r="F127" s="26" t="n">
+        <v>1146</v>
+      </c>
+      <c r="G127" s="24" t="inlineStr"/>
+      <c r="H127" s="25" t="inlineStr"/>
       <c r="I127" s="21">
         <f>IF(OR($B127="",$H127=""),"",IF($C127="LONG",($H127-$E127)*$F127,($E127-$H127)*$F127))</f>
         <v/>
       </c>
-      <c r="J127" s="4" t="n"/>
+      <c r="J127" s="4" t="n">
+        <v>418.12</v>
+      </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
         <v/>
@@ -7642,19 +7758,43 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="23" t="n"/>
-      <c r="B128" s="23" t="n"/>
-      <c r="C128" s="23" t="n"/>
-      <c r="D128" s="24" t="n"/>
-      <c r="E128" s="25" t="n"/>
-      <c r="F128" s="26" t="n"/>
-      <c r="G128" s="24" t="n"/>
-      <c r="H128" s="25" t="n"/>
+      <c r="A128" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260910389009</t>
+        </is>
+      </c>
+      <c r="B128" s="23" t="inlineStr">
+        <is>
+          <t>INDORAMA</t>
+        </is>
+      </c>
+      <c r="C128" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D128" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E128" s="25" t="n">
+        <v>87.26000000000001</v>
+      </c>
+      <c r="F128" s="26" t="n">
+        <v>1022</v>
+      </c>
+      <c r="G128" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H128" s="25" t="n">
+        <v>84.66</v>
+      </c>
       <c r="I128" s="21">
         <f>IF(OR($B128="",$H128=""),"",IF($C128="LONG",($H128-$E128)*$F128,($E128-$H128)*$F128))</f>
         <v/>
       </c>
-      <c r="J128" s="4" t="n"/>
+      <c r="J128" s="4" t="n">
+        <v>78.66</v>
+      </c>
       <c r="K128" s="21">
         <f>IF(OR($B128="",$I128=""),"",$I128-IF($J128="",0,$J128))</f>
         <v/>
@@ -7669,19 +7809,39 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="23" t="n"/>
-      <c r="B129" s="23" t="n"/>
-      <c r="C129" s="23" t="n"/>
-      <c r="D129" s="24" t="n"/>
-      <c r="E129" s="25" t="n"/>
-      <c r="F129" s="26" t="n"/>
-      <c r="G129" s="24" t="n"/>
-      <c r="H129" s="25" t="n"/>
+      <c r="A129" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091079309</t>
+        </is>
+      </c>
+      <c r="B129" s="23" t="inlineStr">
+        <is>
+          <t>KSL</t>
+        </is>
+      </c>
+      <c r="C129" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D129" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E129" s="25" t="n">
+        <v>968.7272</v>
+      </c>
+      <c r="F129" s="26" t="n">
+        <v>299</v>
+      </c>
+      <c r="G129" s="24" t="inlineStr"/>
+      <c r="H129" s="25" t="inlineStr"/>
       <c r="I129" s="21">
         <f>IF(OR($B129="",$H129=""),"",IF($C129="LONG",($H129-$E129)*$F129,($E129-$H129)*$F129))</f>
         <v/>
       </c>
-      <c r="J129" s="4" t="n"/>
+      <c r="J129" s="4" t="n">
+        <v>417.68</v>
+      </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
         <v/>
@@ -7696,19 +7856,43 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="23" t="n"/>
-      <c r="B130" s="23" t="n"/>
-      <c r="C130" s="23" t="n"/>
-      <c r="D130" s="24" t="n"/>
-      <c r="E130" s="25" t="n"/>
-      <c r="F130" s="26" t="n"/>
-      <c r="G130" s="24" t="n"/>
-      <c r="H130" s="25" t="n"/>
+      <c r="A130" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091046609</t>
+        </is>
+      </c>
+      <c r="B130" s="23" t="inlineStr">
+        <is>
+          <t>RESPONIND</t>
+        </is>
+      </c>
+      <c r="C130" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D130" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E130" s="25" t="n">
+        <v>172.11</v>
+      </c>
+      <c r="F130" s="26" t="n">
+        <v>1026</v>
+      </c>
+      <c r="G130" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H130" s="25" t="n">
+        <v>171.29</v>
+      </c>
       <c r="I130" s="21">
         <f>IF(OR($B130="",$H130=""),"",IF($C130="LONG",($H130-$E130)*$F130,($E130-$H130)*$F130))</f>
         <v/>
       </c>
-      <c r="J130" s="4" t="n"/>
+      <c r="J130" s="4" t="n">
+        <v>109.8</v>
+      </c>
       <c r="K130" s="21">
         <f>IF(OR($B130="",$I130=""),"",$I130-IF($J130="",0,$J130))</f>
         <v/>
@@ -7723,19 +7907,39 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="23" t="n"/>
-      <c r="B131" s="23" t="n"/>
-      <c r="C131" s="23" t="n"/>
-      <c r="D131" s="24" t="n"/>
-      <c r="E131" s="25" t="n"/>
-      <c r="F131" s="26" t="n"/>
-      <c r="G131" s="24" t="n"/>
-      <c r="H131" s="25" t="n"/>
+      <c r="A131" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260910622409</t>
+        </is>
+      </c>
+      <c r="B131" s="23" t="inlineStr">
+        <is>
+          <t>SAMHI</t>
+        </is>
+      </c>
+      <c r="C131" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D131" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E131" s="25" t="n">
+        <v>160.6529</v>
+      </c>
+      <c r="F131" s="26" t="n">
+        <v>1815</v>
+      </c>
+      <c r="G131" s="24" t="inlineStr"/>
+      <c r="H131" s="25" t="inlineStr"/>
       <c r="I131" s="21">
         <f>IF(OR($B131="",$H131=""),"",IF($C131="LONG",($H131-$E131)*$F131,($E131-$H131)*$F131))</f>
         <v/>
       </c>
-      <c r="J131" s="4" t="n"/>
+      <c r="J131" s="4" t="n">
+        <v>419.98</v>
+      </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
         <v/>
@@ -7750,19 +7954,43 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="23" t="n"/>
-      <c r="B132" s="23" t="n"/>
-      <c r="C132" s="23" t="n"/>
-      <c r="D132" s="24" t="n"/>
-      <c r="E132" s="25" t="n"/>
-      <c r="F132" s="26" t="n"/>
-      <c r="G132" s="24" t="n"/>
-      <c r="H132" s="25" t="n"/>
+      <c r="A132" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260910101209</t>
+        </is>
+      </c>
+      <c r="B132" s="23" t="inlineStr">
+        <is>
+          <t>SHAREINDIA</t>
+        </is>
+      </c>
+      <c r="C132" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D132" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E132" s="25" t="n">
+        <v>201.46</v>
+      </c>
+      <c r="F132" s="26" t="n">
+        <v>923</v>
+      </c>
+      <c r="G132" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H132" s="25" t="n">
+        <v>205</v>
+      </c>
       <c r="I132" s="21">
         <f>IF(OR($B132="",$H132=""),"",IF($C132="LONG",($H132-$E132)*$F132,($E132-$H132)*$F132))</f>
         <v/>
       </c>
-      <c r="J132" s="4" t="n"/>
+      <c r="J132" s="4" t="n">
+        <v>113.4</v>
+      </c>
       <c r="K132" s="21">
         <f>IF(OR($B132="",$I132=""),"",$I132-IF($J132="",0,$J132))</f>
         <v/>
@@ -7777,19 +8005,39 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="23" t="n"/>
-      <c r="B133" s="23" t="n"/>
-      <c r="C133" s="23" t="n"/>
-      <c r="D133" s="24" t="n"/>
-      <c r="E133" s="25" t="n"/>
-      <c r="F133" s="26" t="n"/>
-      <c r="G133" s="24" t="n"/>
-      <c r="H133" s="25" t="n"/>
+      <c r="A133" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091072709</t>
+        </is>
+      </c>
+      <c r="B133" s="23" t="inlineStr">
+        <is>
+          <t>VSSL</t>
+        </is>
+      </c>
+      <c r="C133" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D133" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E133" s="25" t="n">
+        <v>390.2742</v>
+      </c>
+      <c r="F133" s="26" t="n">
+        <v>739</v>
+      </c>
+      <c r="G133" s="24" t="inlineStr"/>
+      <c r="H133" s="25" t="inlineStr"/>
       <c r="I133" s="21">
         <f>IF(OR($B133="",$H133=""),"",IF($C133="LONG",($H133-$E133)*$F133,($E133-$H133)*$F133))</f>
         <v/>
       </c>
-      <c r="J133" s="4" t="n"/>
+      <c r="J133" s="4" t="n">
+        <v>416.21</v>
+      </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
         <v/>
@@ -7804,19 +8052,39 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="23" t="n"/>
-      <c r="B134" s="23" t="n"/>
-      <c r="C134" s="23" t="n"/>
-      <c r="D134" s="24" t="n"/>
-      <c r="E134" s="25" t="n"/>
-      <c r="F134" s="26" t="n"/>
-      <c r="G134" s="24" t="n"/>
-      <c r="H134" s="25" t="n"/>
+      <c r="A134" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260910622609</t>
+        </is>
+      </c>
+      <c r="B134" s="23" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="C134" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D134" s="24" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E134" s="25" t="n">
+        <v>8657.606</v>
+      </c>
+      <c r="F134" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="G134" s="24" t="inlineStr"/>
+      <c r="H134" s="25" t="inlineStr"/>
       <c r="I134" s="21">
         <f>IF(OR($B134="",$H134=""),"",IF($C134="LONG",($H134-$E134)*$F134,($E134-$H134)*$F134))</f>
         <v/>
       </c>
-      <c r="J134" s="4" t="n"/>
+      <c r="J134" s="4" t="n">
+        <v>412.99</v>
+      </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
         <v/>
@@ -31724,7 +31992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32969,7 +33237,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -33012,7 +33280,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -33055,7 +33323,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -33098,7 +33366,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -33141,7 +33409,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -33184,7 +33452,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -33227,7 +33495,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -33270,7 +33538,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -33313,7 +33581,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33356,7 +33624,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33399,7 +33667,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33442,7 +33710,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33485,7 +33753,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33528,7 +33796,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33571,7 +33839,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33614,7 +33882,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33657,7 +33925,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33700,7 +33968,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -33743,7 +34011,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -33786,7 +34054,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -33829,7 +34097,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -33872,7 +34140,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -33915,7 +34183,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -33958,7 +34226,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -34001,7 +34269,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -34044,7 +34312,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -34087,7 +34355,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -34130,7 +34398,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -34173,7 +34441,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -34216,7 +34484,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -34259,7 +34527,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -34302,7 +34570,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -34345,7 +34613,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -34388,7 +34656,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -34429,37 +34697,209 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B65" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A65)</f>
+        <v/>
+      </c>
+      <c r="C65" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A65,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D65" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A65,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E65" s="29">
+        <f>IFERROR($C65/$B65,"")</f>
+        <v/>
+      </c>
+      <c r="F65" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A65,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G65" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A65,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H65" s="21">
+        <f>IFERROR($G65/$B65,"")</f>
+        <v/>
+      </c>
+      <c r="I65" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A65),"")</f>
+        <v/>
+      </c>
+      <c r="J65" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A65),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B66" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A66)</f>
+        <v/>
+      </c>
+      <c r="C66" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A66,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D66" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A66,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E66" s="29">
+        <f>IFERROR($C66/$B66,"")</f>
+        <v/>
+      </c>
+      <c r="F66" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A66,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G66" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A66,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H66" s="21">
+        <f>IFERROR($G66/$B66,"")</f>
+        <v/>
+      </c>
+      <c r="I66" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A66),"")</f>
+        <v/>
+      </c>
+      <c r="J66" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A66),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B67" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A67)</f>
+        <v/>
+      </c>
+      <c r="C67" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A67,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D67" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A67,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E67" s="29">
+        <f>IFERROR($C67/$B67,"")</f>
+        <v/>
+      </c>
+      <c r="F67" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A67,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G67" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A67,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H67" s="21">
+        <f>IFERROR($G67/$B67,"")</f>
+        <v/>
+      </c>
+      <c r="I67" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A67),"")</f>
+        <v/>
+      </c>
+      <c r="J67" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A67),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B68" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A68)</f>
+        <v/>
+      </c>
+      <c r="C68" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A68,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D68" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A68,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E68" s="29">
+        <f>IFERROR($C68/$B68,"")</f>
+        <v/>
+      </c>
+      <c r="F68" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A68,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G68" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A68,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H68" s="21">
+        <f>IFERROR($G68/$B68,"")</f>
+        <v/>
+      </c>
+      <c r="I68" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A68),"")</f>
+        <v/>
+      </c>
+      <c r="J68" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A68),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B65" s="30">
-        <f>SUM(B4:B64)</f>
-        <v/>
-      </c>
-      <c r="C65" s="30">
-        <f>SUM(C4:C64)</f>
-        <v/>
-      </c>
-      <c r="D65" s="30">
-        <f>SUM(D4:D64)</f>
-        <v/>
-      </c>
-      <c r="E65" s="31">
-        <f>IFERROR(C65/B65,"")</f>
-        <v/>
-      </c>
-      <c r="F65" s="32">
-        <f>SUM(F4:F64)</f>
-        <v/>
-      </c>
-      <c r="G65" s="32">
-        <f>SUM(G4:G64)</f>
-        <v/>
-      </c>
-      <c r="H65" s="32">
-        <f>IFERROR(G65/B65,"")</f>
+      <c r="B69" s="30">
+        <f>SUM(B4:B68)</f>
+        <v/>
+      </c>
+      <c r="C69" s="30">
+        <f>SUM(C4:C68)</f>
+        <v/>
+      </c>
+      <c r="D69" s="30">
+        <f>SUM(D4:D68)</f>
+        <v/>
+      </c>
+      <c r="E69" s="31">
+        <f>IFERROR(C69/B69,"")</f>
+        <v/>
+      </c>
+      <c r="F69" s="32">
+        <f>SUM(F4:F68)</f>
+        <v/>
+      </c>
+      <c r="G69" s="32">
+        <f>SUM(G4:G68)</f>
+        <v/>
+      </c>
+      <c r="H69" s="32">
+        <f>IFERROR(G69/B69,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-11 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.84</v>
+        <v>571.8200000000001</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.87</v>
+        <v>688.91</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.6900000000001</v>
+        <v>570.67</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.11</v>
+        <v>663.08</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.6900000000001</v>
+        <v>590.67</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.65</v>
+        <v>398.64</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.2</v>
+        <v>414.18</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.53</v>
+        <v>414.51</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.23</v>
+        <v>380.28</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.96</v>
+        <v>413.94</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.49</v>
+        <v>406.47</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.14</v>
+        <v>870.3200000000001</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.17</v>
+        <v>391.16</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.79</v>
+        <v>349.78</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.9</v>
+        <v>349.89</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.35</v>
+        <v>386.38</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.3</v>
+        <v>978.27</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.7</v>
+        <v>957.67</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>992.3</v>
+        <v>992.26</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.74</v>
+        <v>599.6900000000001</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.85</v>
+        <v>600.8</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.48</v>
+        <v>678.54</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.35</v>
+        <v>672.47</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.7</v>
+        <v>538.67</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.15</v>
+        <v>627.83</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>618.4299999999999</v>
+        <v>619.1</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>611.66</v>
+        <v>612.2</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>690.86</v>
+        <v>691.97</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>614.5599999999999</v>
+        <v>615.86</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>439.99</v>
+        <v>440.62</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>385.88</v>
+        <v>386.52</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>384.49</v>
+        <v>385.13</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>433.57</v>
+        <v>434.2</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>376.58</v>
+        <v>376.86</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>327.05</v>
+        <v>327.29</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>329.86</v>
+        <v>330.13</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>374.78</v>
+        <v>375.06</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>323.17</v>
+        <v>323.33</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>332.64</v>
+        <v>324.62</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>433.62</v>
+        <v>433.66</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -7032,7 +7032,7 @@
         <v/>
       </c>
       <c r="J113" s="4" t="n">
-        <v>130.14</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="K113" s="21">
         <f>IF(OR($B113="",$I113=""),"",$I113-IF($J113="",0,$J113))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>530.04</v>
+        <v>394.17</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>796.39</v>
+        <v>494.15</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7287,7 +7287,7 @@
         <v/>
       </c>
       <c r="J118" s="4" t="n">
-        <v>211.06</v>
+        <v>145.41</v>
       </c>
       <c r="K118" s="21">
         <f>IF(OR($B118="",$I118=""),"",$I118-IF($J118="",0,$J118))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>523.87</v>
+        <v>391.34</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>529.11</v>
+        <v>343.5</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7593,7 +7593,7 @@
         <v/>
       </c>
       <c r="J124" s="4" t="n">
-        <v>77.45</v>
+        <v>139.07</v>
       </c>
       <c r="K124" s="21">
         <f>IF(OR($B124="",$I124=""),"",$I124-IF($J124="",0,$J124))</f>
@@ -7644,7 +7644,7 @@
         <v/>
       </c>
       <c r="J125" s="4" t="n">
-        <v>111.37</v>
+        <v>223.4</v>
       </c>
       <c r="K125" s="21">
         <f>IF(OR($B125="",$I125=""),"",$I125-IF($J125="",0,$J125))</f>
@@ -7695,7 +7695,7 @@
         <v/>
       </c>
       <c r="J126" s="4" t="n">
-        <v>155.5</v>
+        <v>442.09</v>
       </c>
       <c r="K126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($J126="",0,$J126))</f>
@@ -7735,14 +7735,18 @@
       <c r="F127" s="26" t="n">
         <v>1146</v>
       </c>
-      <c r="G127" s="24" t="inlineStr"/>
-      <c r="H127" s="25" t="inlineStr"/>
+      <c r="G127" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H127" s="25" t="n">
+        <v>263.23</v>
+      </c>
       <c r="I127" s="21">
         <f>IF(OR($B127="",$H127=""),"",IF($C127="LONG",($H127-$E127)*$F127,($E127-$H127)*$F127))</f>
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>418.12</v>
+        <v>814.21</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7793,7 +7797,7 @@
         <v/>
       </c>
       <c r="J128" s="4" t="n">
-        <v>78.66</v>
+        <v>143.17</v>
       </c>
       <c r="K128" s="21">
         <f>IF(OR($B128="",$I128=""),"",$I128-IF($J128="",0,$J128))</f>
@@ -7833,14 +7837,18 @@
       <c r="F129" s="26" t="n">
         <v>299</v>
       </c>
-      <c r="G129" s="24" t="inlineStr"/>
-      <c r="H129" s="25" t="inlineStr"/>
+      <c r="G129" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H129" s="25" t="n">
+        <v>970.53</v>
+      </c>
       <c r="I129" s="21">
         <f>IF(OR($B129="",$H129=""),"",IF($C129="LONG",($H129-$E129)*$F129,($E129-$H129)*$F129))</f>
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>417.68</v>
+        <v>801.76</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7891,7 +7899,7 @@
         <v/>
       </c>
       <c r="J130" s="4" t="n">
-        <v>109.8</v>
+        <v>218.38</v>
       </c>
       <c r="K130" s="21">
         <f>IF(OR($B130="",$I130=""),"",$I130-IF($J130="",0,$J130))</f>
@@ -7931,14 +7939,18 @@
       <c r="F131" s="26" t="n">
         <v>1815</v>
       </c>
-      <c r="G131" s="24" t="inlineStr"/>
-      <c r="H131" s="25" t="inlineStr"/>
+      <c r="G131" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H131" s="25" t="n">
+        <v>157.65</v>
+      </c>
       <c r="I131" s="21">
         <f>IF(OR($B131="",$H131=""),"",IF($C131="LONG",($H131-$E131)*$F131,($E131-$H131)*$F131))</f>
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>419.98</v>
+        <v>807.52</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -7989,7 +8001,7 @@
         <v/>
       </c>
       <c r="J132" s="4" t="n">
-        <v>113.4</v>
+        <v>276.97</v>
       </c>
       <c r="K132" s="21">
         <f>IF(OR($B132="",$I132=""),"",$I132-IF($J132="",0,$J132))</f>
@@ -8029,14 +8041,18 @@
       <c r="F133" s="26" t="n">
         <v>739</v>
       </c>
-      <c r="G133" s="24" t="inlineStr"/>
-      <c r="H133" s="25" t="inlineStr"/>
+      <c r="G133" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H133" s="25" t="n">
+        <v>395.2</v>
+      </c>
       <c r="I133" s="21">
         <f>IF(OR($B133="",$H133=""),"",IF($C133="LONG",($H133-$E133)*$F133,($E133-$H133)*$F133))</f>
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>416.21</v>
+        <v>801.97</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8076,14 +8092,18 @@
       <c r="F134" s="26" t="n">
         <v>33</v>
       </c>
-      <c r="G134" s="24" t="inlineStr"/>
-      <c r="H134" s="25" t="inlineStr"/>
+      <c r="G134" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H134" s="25" t="n">
+        <v>8730.18</v>
+      </c>
       <c r="I134" s="21">
         <f>IF(OR($B134="",$H134=""),"",IF($C134="LONG",($H134-$E134)*$F134,($E134-$H134)*$F134))</f>
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>412.99</v>
+        <v>794.09</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8099,19 +8119,39 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="23" t="n"/>
-      <c r="B135" s="23" t="n"/>
-      <c r="C135" s="23" t="n"/>
-      <c r="D135" s="24" t="n"/>
-      <c r="E135" s="25" t="n"/>
-      <c r="F135" s="26" t="n"/>
-      <c r="G135" s="24" t="n"/>
-      <c r="H135" s="25" t="n"/>
+      <c r="A135" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091161109</t>
+        </is>
+      </c>
+      <c r="B135" s="23" t="inlineStr">
+        <is>
+          <t>AWFIS</t>
+        </is>
+      </c>
+      <c r="C135" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D135" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E135" s="25" t="n">
+        <v>293.7202</v>
+      </c>
+      <c r="F135" s="26" t="n">
+        <v>618</v>
+      </c>
+      <c r="G135" s="24" t="inlineStr"/>
+      <c r="H135" s="25" t="inlineStr"/>
       <c r="I135" s="21">
         <f>IF(OR($B135="",$H135=""),"",IF($C135="LONG",($H135-$E135)*$F135,($E135-$H135)*$F135))</f>
         <v/>
       </c>
-      <c r="J135" s="4" t="n"/>
+      <c r="J135" s="4" t="n">
+        <v>289.29</v>
+      </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
         <v/>
@@ -8126,19 +8166,39 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="23" t="n"/>
-      <c r="B136" s="23" t="n"/>
-      <c r="C136" s="23" t="n"/>
-      <c r="D136" s="24" t="n"/>
-      <c r="E136" s="25" t="n"/>
-      <c r="F136" s="26" t="n"/>
-      <c r="G136" s="24" t="n"/>
-      <c r="H136" s="25" t="n"/>
+      <c r="A136" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260911696009</t>
+        </is>
+      </c>
+      <c r="B136" s="23" t="inlineStr">
+        <is>
+          <t>FILATEX</t>
+        </is>
+      </c>
+      <c r="C136" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D136" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E136" s="25" t="n">
+        <v>87.3199</v>
+      </c>
+      <c r="F136" s="26" t="n">
+        <v>1042</v>
+      </c>
+      <c r="G136" s="24" t="inlineStr"/>
+      <c r="H136" s="25" t="inlineStr"/>
       <c r="I136" s="21">
         <f>IF(OR($B136="",$H136=""),"",IF($C136="LONG",($H136-$E136)*$F136,($E136-$H136)*$F136))</f>
         <v/>
       </c>
-      <c r="J136" s="4" t="n"/>
+      <c r="J136" s="4" t="n">
+        <v>122.79</v>
+      </c>
       <c r="K136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($J136="",0,$J136))</f>
         <v/>
@@ -8153,19 +8213,43 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="23" t="n"/>
-      <c r="B137" s="23" t="n"/>
-      <c r="C137" s="23" t="n"/>
-      <c r="D137" s="24" t="n"/>
-      <c r="E137" s="25" t="n"/>
-      <c r="F137" s="26" t="n"/>
-      <c r="G137" s="24" t="n"/>
-      <c r="H137" s="25" t="n"/>
+      <c r="A137" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091115309</t>
+        </is>
+      </c>
+      <c r="B137" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C137" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D137" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E137" s="25" t="n">
+        <v>263.46</v>
+      </c>
+      <c r="F137" s="26" t="n">
+        <v>1146</v>
+      </c>
+      <c r="G137" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H137" s="25" t="n">
+        <v>262.88</v>
+      </c>
       <c r="I137" s="21">
         <f>IF(OR($B137="",$H137=""),"",IF($C137="LONG",($H137-$E137)*$F137,($E137-$H137)*$F137))</f>
         <v/>
       </c>
-      <c r="J137" s="4" t="n"/>
+      <c r="J137" s="4" t="n">
+        <v>154.28</v>
+      </c>
       <c r="K137" s="21">
         <f>IF(OR($B137="",$I137=""),"",$I137-IF($J137="",0,$J137))</f>
         <v/>
@@ -8180,19 +8264,39 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="23" t="n"/>
-      <c r="B138" s="23" t="n"/>
-      <c r="C138" s="23" t="n"/>
-      <c r="D138" s="24" t="n"/>
-      <c r="E138" s="25" t="n"/>
-      <c r="F138" s="26" t="n"/>
-      <c r="G138" s="24" t="n"/>
-      <c r="H138" s="25" t="n"/>
+      <c r="A138" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260911696409</t>
+        </is>
+      </c>
+      <c r="B138" s="23" t="inlineStr">
+        <is>
+          <t>KIRLOSIND</t>
+        </is>
+      </c>
+      <c r="C138" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D138" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E138" s="25" t="n">
+        <v>3826.583</v>
+      </c>
+      <c r="F138" s="26" t="n">
+        <v>47</v>
+      </c>
+      <c r="G138" s="24" t="inlineStr"/>
+      <c r="H138" s="25" t="inlineStr"/>
       <c r="I138" s="21">
         <f>IF(OR($B138="",$H138=""),"",IF($C138="LONG",($H138-$E138)*$F138,($E138-$H138)*$F138))</f>
         <v/>
       </c>
-      <c r="J138" s="4" t="n"/>
+      <c r="J138" s="4" t="n">
+        <v>287.3</v>
+      </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
         <v/>
@@ -8207,19 +8311,43 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="23" t="n"/>
-      <c r="B139" s="23" t="n"/>
-      <c r="C139" s="23" t="n"/>
-      <c r="D139" s="24" t="n"/>
-      <c r="E139" s="25" t="n"/>
-      <c r="F139" s="26" t="n"/>
-      <c r="G139" s="24" t="n"/>
-      <c r="H139" s="25" t="n"/>
+      <c r="A139" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260911440509</t>
+        </is>
+      </c>
+      <c r="B139" s="23" t="inlineStr">
+        <is>
+          <t>KSL</t>
+        </is>
+      </c>
+      <c r="C139" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D139" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E139" s="25" t="n">
+        <v>970.4299999999999</v>
+      </c>
+      <c r="F139" s="26" t="n">
+        <v>299</v>
+      </c>
+      <c r="G139" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H139" s="25" t="n">
+        <v>959.9299999999999</v>
+      </c>
       <c r="I139" s="21">
         <f>IF(OR($B139="",$H139=""),"",IF($C139="LONG",($H139-$E139)*$F139,($E139-$H139)*$F139))</f>
         <v/>
       </c>
-      <c r="J139" s="4" t="n"/>
+      <c r="J139" s="4" t="n">
+        <v>149.94</v>
+      </c>
       <c r="K139" s="21">
         <f>IF(OR($B139="",$I139=""),"",$I139-IF($J139="",0,$J139))</f>
         <v/>
@@ -8234,19 +8362,39 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="23" t="n"/>
-      <c r="B140" s="23" t="n"/>
-      <c r="C140" s="23" t="n"/>
-      <c r="D140" s="24" t="n"/>
-      <c r="E140" s="25" t="n"/>
-      <c r="F140" s="26" t="n"/>
-      <c r="G140" s="24" t="n"/>
-      <c r="H140" s="25" t="n"/>
+      <c r="A140" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260911696509</t>
+        </is>
+      </c>
+      <c r="B140" s="23" t="inlineStr">
+        <is>
+          <t>MOBIKWIK</t>
+        </is>
+      </c>
+      <c r="C140" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D140" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E140" s="25" t="n">
+        <v>209.9685</v>
+      </c>
+      <c r="F140" s="26" t="n">
+        <v>860</v>
+      </c>
+      <c r="G140" s="24" t="inlineStr"/>
+      <c r="H140" s="25" t="inlineStr"/>
       <c r="I140" s="21">
         <f>IF(OR($B140="",$H140=""),"",IF($C140="LONG",($H140-$E140)*$F140,($E140-$H140)*$F140))</f>
         <v/>
       </c>
-      <c r="J140" s="4" t="n"/>
+      <c r="J140" s="4" t="n">
+        <v>288.16</v>
+      </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
         <v/>
@@ -8261,19 +8409,39 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="23" t="n"/>
-      <c r="B141" s="23" t="n"/>
-      <c r="C141" s="23" t="n"/>
-      <c r="D141" s="24" t="n"/>
-      <c r="E141" s="25" t="n"/>
-      <c r="F141" s="26" t="n"/>
-      <c r="G141" s="24" t="n"/>
-      <c r="H141" s="25" t="n"/>
+      <c r="A141" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260911696609</t>
+        </is>
+      </c>
+      <c r="B141" s="23" t="inlineStr">
+        <is>
+          <t>QUADFUTURE</t>
+        </is>
+      </c>
+      <c r="C141" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D141" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E141" s="25" t="n">
+        <v>481.45</v>
+      </c>
+      <c r="F141" s="26" t="n">
+        <v>377</v>
+      </c>
+      <c r="G141" s="24" t="inlineStr"/>
+      <c r="H141" s="25" t="inlineStr"/>
       <c r="I141" s="21">
         <f>IF(OR($B141="",$H141=""),"",IF($C141="LONG",($H141-$E141)*$F141,($E141-$H141)*$F141))</f>
         <v/>
       </c>
-      <c r="J141" s="4" t="n"/>
+      <c r="J141" s="4" t="n">
+        <v>289.27</v>
+      </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
         <v/>
@@ -8288,19 +8456,39 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="23" t="n"/>
-      <c r="B142" s="23" t="n"/>
-      <c r="C142" s="23" t="n"/>
-      <c r="D142" s="24" t="n"/>
-      <c r="E142" s="25" t="n"/>
-      <c r="F142" s="26" t="n"/>
-      <c r="G142" s="24" t="n"/>
-      <c r="H142" s="25" t="n"/>
+      <c r="A142" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260911696809</t>
+        </is>
+      </c>
+      <c r="B142" s="23" t="inlineStr">
+        <is>
+          <t>RACLGEAR</t>
+        </is>
+      </c>
+      <c r="C142" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D142" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E142" s="25" t="n">
+        <v>1756.5941</v>
+      </c>
+      <c r="F142" s="26" t="n">
+        <v>103</v>
+      </c>
+      <c r="G142" s="24" t="inlineStr"/>
+      <c r="H142" s="25" t="inlineStr"/>
       <c r="I142" s="21">
         <f>IF(OR($B142="",$H142=""),"",IF($C142="LONG",($H142-$E142)*$F142,($E142-$H142)*$F142))</f>
         <v/>
       </c>
-      <c r="J142" s="4" t="n"/>
+      <c r="J142" s="4" t="n">
+        <v>288.59</v>
+      </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
         <v/>
@@ -8315,19 +8503,43 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="23" t="n"/>
-      <c r="B143" s="23" t="n"/>
-      <c r="C143" s="23" t="n"/>
-      <c r="D143" s="24" t="n"/>
-      <c r="E143" s="25" t="n"/>
-      <c r="F143" s="26" t="n"/>
-      <c r="G143" s="24" t="n"/>
-      <c r="H143" s="25" t="n"/>
+      <c r="A143" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260911438509</t>
+        </is>
+      </c>
+      <c r="B143" s="23" t="inlineStr">
+        <is>
+          <t>SAMHI</t>
+        </is>
+      </c>
+      <c r="C143" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D143" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E143" s="25" t="n">
+        <v>157.53</v>
+      </c>
+      <c r="F143" s="26" t="n">
+        <v>1815</v>
+      </c>
+      <c r="G143" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H143" s="25" t="n">
+        <v>157.18</v>
+      </c>
       <c r="I143" s="21">
         <f>IF(OR($B143="",$H143=""),"",IF($C143="LONG",($H143-$E143)*$F143,($E143-$H143)*$F143))</f>
         <v/>
       </c>
-      <c r="J143" s="4" t="n"/>
+      <c r="J143" s="4" t="n">
+        <v>148.6</v>
+      </c>
       <c r="K143" s="21">
         <f>IF(OR($B143="",$I143=""),"",$I143-IF($J143="",0,$J143))</f>
         <v/>
@@ -8342,19 +8554,39 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="23" t="n"/>
-      <c r="B144" s="23" t="n"/>
-      <c r="C144" s="23" t="n"/>
-      <c r="D144" s="24" t="n"/>
-      <c r="E144" s="25" t="n"/>
-      <c r="F144" s="26" t="n"/>
-      <c r="G144" s="24" t="n"/>
-      <c r="H144" s="25" t="n"/>
+      <c r="A144" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091161209</t>
+        </is>
+      </c>
+      <c r="B144" s="23" t="inlineStr">
+        <is>
+          <t>SIKA</t>
+        </is>
+      </c>
+      <c r="C144" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D144" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E144" s="25" t="n">
+        <v>1087.1632</v>
+      </c>
+      <c r="F144" s="26" t="n">
+        <v>83</v>
+      </c>
+      <c r="G144" s="24" t="inlineStr"/>
+      <c r="H144" s="25" t="inlineStr"/>
       <c r="I144" s="21">
         <f>IF(OR($B144="",$H144=""),"",IF($C144="LONG",($H144-$E144)*$F144,($E144-$H144)*$F144))</f>
         <v/>
       </c>
-      <c r="J144" s="4" t="n"/>
+      <c r="J144" s="4" t="n">
+        <v>121.89</v>
+      </c>
       <c r="K144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($J144="",0,$J144))</f>
         <v/>
@@ -8369,19 +8601,39 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="23" t="n"/>
-      <c r="B145" s="23" t="n"/>
-      <c r="C145" s="23" t="n"/>
-      <c r="D145" s="24" t="n"/>
-      <c r="E145" s="25" t="n"/>
-      <c r="F145" s="26" t="n"/>
-      <c r="G145" s="24" t="n"/>
-      <c r="H145" s="25" t="n"/>
+      <c r="A145" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260911696209</t>
+        </is>
+      </c>
+      <c r="B145" s="23" t="inlineStr">
+        <is>
+          <t>SMSPHARMA</t>
+        </is>
+      </c>
+      <c r="C145" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D145" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E145" s="25" t="n">
+        <v>462.4796</v>
+      </c>
+      <c r="F145" s="26" t="n">
+        <v>391</v>
+      </c>
+      <c r="G145" s="24" t="inlineStr"/>
+      <c r="H145" s="25" t="inlineStr"/>
       <c r="I145" s="21">
         <f>IF(OR($B145="",$H145=""),"",IF($C145="LONG",($H145-$E145)*$F145,($E145-$H145)*$F145))</f>
         <v/>
       </c>
-      <c r="J145" s="4" t="n"/>
+      <c r="J145" s="4" t="n">
+        <v>288.47</v>
+      </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
         <v/>
@@ -8396,19 +8648,43 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="23" t="n"/>
-      <c r="B146" s="23" t="n"/>
-      <c r="C146" s="23" t="n"/>
-      <c r="D146" s="24" t="n"/>
-      <c r="E146" s="25" t="n"/>
-      <c r="F146" s="26" t="n"/>
-      <c r="G146" s="24" t="n"/>
-      <c r="H146" s="25" t="n"/>
+      <c r="A146" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091141909</t>
+        </is>
+      </c>
+      <c r="B146" s="23" t="inlineStr">
+        <is>
+          <t>VSSL</t>
+        </is>
+      </c>
+      <c r="C146" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D146" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E146" s="25" t="n">
+        <v>394.09</v>
+      </c>
+      <c r="F146" s="26" t="n">
+        <v>739</v>
+      </c>
+      <c r="G146" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H146" s="25" t="n">
+        <v>401.45</v>
+      </c>
       <c r="I146" s="21">
         <f>IF(OR($B146="",$H146=""),"",IF($C146="LONG",($H146-$E146)*$F146,($E146-$H146)*$F146))</f>
         <v/>
       </c>
-      <c r="J146" s="4" t="n"/>
+      <c r="J146" s="4" t="n">
+        <v>150.9</v>
+      </c>
       <c r="K146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($J146="",0,$J146))</f>
         <v/>
@@ -8423,19 +8699,43 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="23" t="n"/>
-      <c r="B147" s="23" t="n"/>
-      <c r="C147" s="23" t="n"/>
-      <c r="D147" s="24" t="n"/>
-      <c r="E147" s="25" t="n"/>
-      <c r="F147" s="26" t="n"/>
-      <c r="G147" s="24" t="n"/>
-      <c r="H147" s="25" t="n"/>
+      <c r="A147" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091130609</t>
+        </is>
+      </c>
+      <c r="B147" s="23" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="C147" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D147" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E147" s="25" t="n">
+        <v>8724.209999999999</v>
+      </c>
+      <c r="F147" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="G147" s="24" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H147" s="25" t="n">
+        <v>8867.91</v>
+      </c>
       <c r="I147" s="21">
         <f>IF(OR($B147="",$H147=""),"",IF($C147="LONG",($H147-$E147)*$F147,($E147-$H147)*$F147))</f>
         <v/>
       </c>
-      <c r="J147" s="4" t="n"/>
+      <c r="J147" s="4" t="n">
+        <v>149.67</v>
+      </c>
       <c r="K147" s="21">
         <f>IF(OR($B147="",$I147=""),"",$I147-IF($J147="",0,$J147))</f>
         <v/>
@@ -31992,7 +32292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32205,7 +32505,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -32248,7 +32548,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -32291,7 +32591,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -32334,7 +32634,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>BFUTILITIE</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -32377,7 +32677,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -32420,7 +32720,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -32463,7 +32763,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -32506,7 +32806,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -32549,7 +32849,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -32592,7 +32892,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -32635,7 +32935,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -32678,7 +32978,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -32721,7 +33021,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -32764,7 +33064,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -32807,7 +33107,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -32850,7 +33150,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -32893,7 +33193,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -32936,7 +33236,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -32979,7 +33279,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -33022,7 +33322,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -33065,7 +33365,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -33108,7 +33408,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -33151,7 +33451,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -33194,7 +33494,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -33237,7 +33537,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -33280,7 +33580,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -33323,7 +33623,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -33366,7 +33666,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -33409,7 +33709,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -33452,7 +33752,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -33495,7 +33795,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -33538,7 +33838,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -33581,7 +33881,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -33624,7 +33924,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -33667,7 +33967,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -33710,7 +34010,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -33753,7 +34053,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -33796,7 +34096,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -33839,7 +34139,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -33882,7 +34182,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -33925,7 +34225,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -33968,7 +34268,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -34011,7 +34311,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -34054,7 +34354,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -34097,7 +34397,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -34140,7 +34440,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -34183,7 +34483,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -34226,7 +34526,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -34269,7 +34569,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -34312,7 +34612,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -34355,7 +34655,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -34398,7 +34698,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -34441,7 +34741,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -34484,7 +34784,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -34527,7 +34827,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -34570,7 +34870,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -34613,7 +34913,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -34656,7 +34956,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -34699,7 +34999,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -34742,7 +35042,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -34785,7 +35085,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -34828,7 +35128,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -34869,37 +35169,338 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+      <c r="A69" s="27" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="B69" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A69)</f>
+        <v/>
+      </c>
+      <c r="C69" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A69,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D69" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A69,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E69" s="29">
+        <f>IFERROR($C69/$B69,"")</f>
+        <v/>
+      </c>
+      <c r="F69" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A69,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G69" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A69,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H69" s="21">
+        <f>IFERROR($G69/$B69,"")</f>
+        <v/>
+      </c>
+      <c r="I69" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A69),"")</f>
+        <v/>
+      </c>
+      <c r="J69" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A69),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="27" t="inlineStr">
+        <is>
+          <t>VSSL</t>
+        </is>
+      </c>
+      <c r="B70" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A70)</f>
+        <v/>
+      </c>
+      <c r="C70" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A70,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D70" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A70,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E70" s="29">
+        <f>IFERROR($C70/$B70,"")</f>
+        <v/>
+      </c>
+      <c r="F70" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A70,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G70" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A70,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H70" s="21">
+        <f>IFERROR($G70/$B70,"")</f>
+        <v/>
+      </c>
+      <c r="I70" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A70),"")</f>
+        <v/>
+      </c>
+      <c r="J70" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A70),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B71" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A71)</f>
+        <v/>
+      </c>
+      <c r="C71" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A71,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D71" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A71,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E71" s="29">
+        <f>IFERROR($C71/$B71,"")</f>
+        <v/>
+      </c>
+      <c r="F71" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A71,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G71" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A71,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H71" s="21">
+        <f>IFERROR($G71/$B71,"")</f>
+        <v/>
+      </c>
+      <c r="I71" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A71),"")</f>
+        <v/>
+      </c>
+      <c r="J71" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A71),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B72" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A72)</f>
+        <v/>
+      </c>
+      <c r="C72" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A72,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D72" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A72,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E72" s="29">
+        <f>IFERROR($C72/$B72,"")</f>
+        <v/>
+      </c>
+      <c r="F72" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A72,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G72" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A72,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H72" s="21">
+        <f>IFERROR($G72/$B72,"")</f>
+        <v/>
+      </c>
+      <c r="I72" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A72),"")</f>
+        <v/>
+      </c>
+      <c r="J72" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A72),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B73" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A73)</f>
+        <v/>
+      </c>
+      <c r="C73" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A73,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D73" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A73,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E73" s="29">
+        <f>IFERROR($C73/$B73,"")</f>
+        <v/>
+      </c>
+      <c r="F73" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A73,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G73" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A73,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H73" s="21">
+        <f>IFERROR($G73/$B73,"")</f>
+        <v/>
+      </c>
+      <c r="I73" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A73),"")</f>
+        <v/>
+      </c>
+      <c r="J73" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A73),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B74" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A74)</f>
+        <v/>
+      </c>
+      <c r="C74" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A74,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D74" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A74,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E74" s="29">
+        <f>IFERROR($C74/$B74,"")</f>
+        <v/>
+      </c>
+      <c r="F74" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A74,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G74" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A74,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H74" s="21">
+        <f>IFERROR($G74/$B74,"")</f>
+        <v/>
+      </c>
+      <c r="I74" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A74),"")</f>
+        <v/>
+      </c>
+      <c r="J74" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A74),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B75" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A75)</f>
+        <v/>
+      </c>
+      <c r="C75" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A75,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D75" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A75,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E75" s="29">
+        <f>IFERROR($C75/$B75,"")</f>
+        <v/>
+      </c>
+      <c r="F75" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A75,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G75" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A75,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H75" s="21">
+        <f>IFERROR($G75/$B75,"")</f>
+        <v/>
+      </c>
+      <c r="I75" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A75),"")</f>
+        <v/>
+      </c>
+      <c r="J75" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A75),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B69" s="30">
-        <f>SUM(B4:B68)</f>
-        <v/>
-      </c>
-      <c r="C69" s="30">
-        <f>SUM(C4:C68)</f>
-        <v/>
-      </c>
-      <c r="D69" s="30">
-        <f>SUM(D4:D68)</f>
-        <v/>
-      </c>
-      <c r="E69" s="31">
-        <f>IFERROR(C69/B69,"")</f>
-        <v/>
-      </c>
-      <c r="F69" s="32">
-        <f>SUM(F4:F68)</f>
-        <v/>
-      </c>
-      <c r="G69" s="32">
-        <f>SUM(G4:G68)</f>
-        <v/>
-      </c>
-      <c r="H69" s="32">
-        <f>IFERROR(G69/B69,"")</f>
+      <c r="B76" s="30">
+        <f>SUM(B4:B75)</f>
+        <v/>
+      </c>
+      <c r="C76" s="30">
+        <f>SUM(C4:C75)</f>
+        <v/>
+      </c>
+      <c r="D76" s="30">
+        <f>SUM(D4:D75)</f>
+        <v/>
+      </c>
+      <c r="E76" s="31">
+        <f>IFERROR(C76/B76,"")</f>
+        <v/>
+      </c>
+      <c r="F76" s="32">
+        <f>SUM(F4:F75)</f>
+        <v/>
+      </c>
+      <c r="G76" s="32">
+        <f>SUM(G4:G75)</f>
+        <v/>
+      </c>
+      <c r="H76" s="32">
+        <f>IFERROR(G76/B76,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>